<commit_message>
Updated to Version 2 (2012-2022)
</commit_message>
<xml_diff>
--- a/step2_obtain_gdp_data/inputs/gdp_data/regional/KAZ/1. Gross regional product.xlsx
+++ b/step2_obtain_gdp_data/inputs/gdp_data/regional/KAZ/1. Gross regional product.xlsx
@@ -4,12 +4,12 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr showInkAnnotation="0" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1230" yWindow="165" windowWidth="17205" windowHeight="9075" activeTab="2"/>
+    <workbookView xWindow="345" yWindow="45" windowWidth="28065" windowHeight="10530" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name=" 1990-1997" sheetId="4" r:id="rId1"/>
     <sheet name="1998-2007" sheetId="5" r:id="rId2"/>
-    <sheet name="2008-2023" sheetId="3" r:id="rId3"/>
+    <sheet name="2008-2024" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="144525" fullPrecision="0"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="87">
   <si>
     <r>
       <t>1990</t>
@@ -289,59 +289,6 @@
     <t>1 half-year of 2022</t>
   </si>
   <si>
-    <r>
-      <t>2023</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <vertAlign val="superscript"/>
-        <sz val="8"/>
-        <rFont val="Roboto"/>
-        <charset val="204"/>
-      </rPr>
-      <t>2)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="8"/>
-        <rFont val="Roboto"/>
-        <charset val="204"/>
-      </rPr>
-      <t>1)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Roboto"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve"> quarterly calculations of GRP have been producing only from 2008</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="8"/>
-        <rFont val="Roboto"/>
-        <charset val="204"/>
-      </rPr>
-      <t>2)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Roboto"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve"> preliminary data </t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">Zhetisu </t>
   </si>
   <si>
@@ -358,7 +305,73 @@
   </si>
   <si>
     <r>
+      <t>Astana city</t>
+    </r>
+    <r>
       <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="8"/>
+        <rFont val="Roboto"/>
+        <charset val="204"/>
+      </rPr>
+      <t>2)</t>
+    </r>
+  </si>
+  <si>
+    <t>1 quarter of 2024</t>
+  </si>
+  <si>
+    <t>1  half-year of 2024</t>
+  </si>
+  <si>
+    <t>9 months of 2024</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <vertAlign val="superscript"/>
+        <sz val="8"/>
+        <rFont val="Roboto"/>
+        <charset val="204"/>
+      </rPr>
+      <t>1)</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <rFont val="Roboto"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve"> quarterly calculations of GRP have been producing only from 2008</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <vertAlign val="superscript"/>
+        <sz val="8"/>
+        <rFont val="Roboto"/>
+        <charset val="204"/>
+      </rPr>
+      <t>1)</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <rFont val="Roboto"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve"> 1990-1992 -mln. rubles</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
         <vertAlign val="superscript"/>
         <sz val="8"/>
         <rFont val="Roboto"/>
@@ -368,6 +381,7 @@
     </r>
     <r>
       <rPr>
+        <i/>
         <sz val="8"/>
         <rFont val="Roboto"/>
         <charset val="204"/>
@@ -378,25 +392,68 @@
   <si>
     <r>
       <rPr>
+        <i/>
         <vertAlign val="superscript"/>
         <sz val="8"/>
         <rFont val="Roboto"/>
         <charset val="204"/>
       </rPr>
-      <t>1)</t>
+      <t>2)</t>
     </r>
     <r>
       <rPr>
+        <i/>
         <sz val="8"/>
         <rFont val="Roboto"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve"> 1990-1992 -mln. rubles</t>
+      <t xml:space="preserve"> starting from the first half of 2018, GRP calculations were made taking into account new regions - Turkestan region and the city of Shymkent.</t>
     </r>
   </si>
   <si>
     <r>
-      <t>Astana city</t>
+      <rPr>
+        <i/>
+        <vertAlign val="superscript"/>
+        <sz val="8"/>
+        <rFont val="Roboto"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">3) </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <rFont val="Roboto"/>
+        <charset val="204"/>
+      </rPr>
+      <t>In connection with the formation of new administrative-territorial units, the Gross Regional Product for 2021 was recalculated.</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <vertAlign val="superscript"/>
+        <sz val="8"/>
+        <rFont val="Roboto"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <rFont val="Roboto"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2023 </t>
     </r>
     <r>
       <rPr>
@@ -405,7 +462,28 @@
         <rFont val="Roboto"/>
         <charset val="204"/>
       </rPr>
-      <t>2)</t>
+      <t>4</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <vertAlign val="superscript"/>
+        <sz val="8"/>
+        <rFont val="Roboto"/>
+        <charset val="204"/>
+      </rPr>
+      <t>4)</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <rFont val="Roboto"/>
+        <charset val="204"/>
+      </rPr>
+      <t>Data for 2023 have been republished due to revisions to sectoral indicators for transport and agriculture, as well as methodological clarifications for reports from the insurance sector and the general government sector. The indicators for taxes on products and subsidies on products  have been recalculated based on administrative data.</t>
     </r>
   </si>
 </sst>
@@ -465,14 +543,15 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <vertAlign val="superscript"/>
+      <sz val="10"/>
       <name val="Roboto"/>
       <charset val="204"/>
     </font>
     <font>
-      <b/>
+      <i/>
       <vertAlign val="superscript"/>
-      <sz val="10"/>
+      <sz val="8"/>
       <name val="Roboto"/>
       <charset val="204"/>
     </font>
@@ -491,7 +570,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -542,24 +621,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -588,9 +654,6 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -606,20 +669,8 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -643,15 +694,20 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -661,6 +717,15 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -968,926 +1033,926 @@
   <dimension ref="A1:S23"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22" style="19" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" style="19" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" style="19" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" style="19" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="19" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="19" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" style="19" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" style="19" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="21" width="11.42578125" style="19" customWidth="1"/>
-    <col min="22" max="25" width="11.7109375" style="19" customWidth="1"/>
-    <col min="26" max="26" width="12.140625" style="19" customWidth="1"/>
-    <col min="27" max="27" width="11.85546875" style="19" customWidth="1"/>
-    <col min="28" max="256" width="9.140625" style="19"/>
-    <col min="257" max="257" width="22" style="19" customWidth="1"/>
-    <col min="258" max="258" width="12.42578125" style="19" customWidth="1"/>
-    <col min="259" max="259" width="12.140625" style="19" customWidth="1"/>
-    <col min="260" max="260" width="12.28515625" style="19" customWidth="1"/>
-    <col min="261" max="261" width="10.5703125" style="19" customWidth="1"/>
-    <col min="262" max="262" width="11.5703125" style="19" customWidth="1"/>
-    <col min="263" max="263" width="10.85546875" style="19" customWidth="1"/>
-    <col min="264" max="264" width="11.140625" style="19" customWidth="1"/>
-    <col min="265" max="265" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="266" max="277" width="11.42578125" style="19" customWidth="1"/>
-    <col min="278" max="281" width="11.7109375" style="19" customWidth="1"/>
-    <col min="282" max="282" width="12.140625" style="19" customWidth="1"/>
-    <col min="283" max="283" width="11.85546875" style="19" customWidth="1"/>
-    <col min="284" max="512" width="9.140625" style="19"/>
-    <col min="513" max="513" width="22" style="19" customWidth="1"/>
-    <col min="514" max="514" width="12.42578125" style="19" customWidth="1"/>
-    <col min="515" max="515" width="12.140625" style="19" customWidth="1"/>
-    <col min="516" max="516" width="12.28515625" style="19" customWidth="1"/>
-    <col min="517" max="517" width="10.5703125" style="19" customWidth="1"/>
-    <col min="518" max="518" width="11.5703125" style="19" customWidth="1"/>
-    <col min="519" max="519" width="10.85546875" style="19" customWidth="1"/>
-    <col min="520" max="520" width="11.140625" style="19" customWidth="1"/>
-    <col min="521" max="521" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="522" max="533" width="11.42578125" style="19" customWidth="1"/>
-    <col min="534" max="537" width="11.7109375" style="19" customWidth="1"/>
-    <col min="538" max="538" width="12.140625" style="19" customWidth="1"/>
-    <col min="539" max="539" width="11.85546875" style="19" customWidth="1"/>
-    <col min="540" max="768" width="9.140625" style="19"/>
-    <col min="769" max="769" width="22" style="19" customWidth="1"/>
-    <col min="770" max="770" width="12.42578125" style="19" customWidth="1"/>
-    <col min="771" max="771" width="12.140625" style="19" customWidth="1"/>
-    <col min="772" max="772" width="12.28515625" style="19" customWidth="1"/>
-    <col min="773" max="773" width="10.5703125" style="19" customWidth="1"/>
-    <col min="774" max="774" width="11.5703125" style="19" customWidth="1"/>
-    <col min="775" max="775" width="10.85546875" style="19" customWidth="1"/>
-    <col min="776" max="776" width="11.140625" style="19" customWidth="1"/>
-    <col min="777" max="777" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="778" max="789" width="11.42578125" style="19" customWidth="1"/>
-    <col min="790" max="793" width="11.7109375" style="19" customWidth="1"/>
-    <col min="794" max="794" width="12.140625" style="19" customWidth="1"/>
-    <col min="795" max="795" width="11.85546875" style="19" customWidth="1"/>
-    <col min="796" max="1024" width="9.140625" style="19"/>
-    <col min="1025" max="1025" width="22" style="19" customWidth="1"/>
-    <col min="1026" max="1026" width="12.42578125" style="19" customWidth="1"/>
-    <col min="1027" max="1027" width="12.140625" style="19" customWidth="1"/>
-    <col min="1028" max="1028" width="12.28515625" style="19" customWidth="1"/>
-    <col min="1029" max="1029" width="10.5703125" style="19" customWidth="1"/>
-    <col min="1030" max="1030" width="11.5703125" style="19" customWidth="1"/>
-    <col min="1031" max="1031" width="10.85546875" style="19" customWidth="1"/>
-    <col min="1032" max="1032" width="11.140625" style="19" customWidth="1"/>
-    <col min="1033" max="1033" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="1034" max="1045" width="11.42578125" style="19" customWidth="1"/>
-    <col min="1046" max="1049" width="11.7109375" style="19" customWidth="1"/>
-    <col min="1050" max="1050" width="12.140625" style="19" customWidth="1"/>
-    <col min="1051" max="1051" width="11.85546875" style="19" customWidth="1"/>
-    <col min="1052" max="1280" width="9.140625" style="19"/>
-    <col min="1281" max="1281" width="22" style="19" customWidth="1"/>
-    <col min="1282" max="1282" width="12.42578125" style="19" customWidth="1"/>
-    <col min="1283" max="1283" width="12.140625" style="19" customWidth="1"/>
-    <col min="1284" max="1284" width="12.28515625" style="19" customWidth="1"/>
-    <col min="1285" max="1285" width="10.5703125" style="19" customWidth="1"/>
-    <col min="1286" max="1286" width="11.5703125" style="19" customWidth="1"/>
-    <col min="1287" max="1287" width="10.85546875" style="19" customWidth="1"/>
-    <col min="1288" max="1288" width="11.140625" style="19" customWidth="1"/>
-    <col min="1289" max="1289" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="1290" max="1301" width="11.42578125" style="19" customWidth="1"/>
-    <col min="1302" max="1305" width="11.7109375" style="19" customWidth="1"/>
-    <col min="1306" max="1306" width="12.140625" style="19" customWidth="1"/>
-    <col min="1307" max="1307" width="11.85546875" style="19" customWidth="1"/>
-    <col min="1308" max="1536" width="9.140625" style="19"/>
-    <col min="1537" max="1537" width="22" style="19" customWidth="1"/>
-    <col min="1538" max="1538" width="12.42578125" style="19" customWidth="1"/>
-    <col min="1539" max="1539" width="12.140625" style="19" customWidth="1"/>
-    <col min="1540" max="1540" width="12.28515625" style="19" customWidth="1"/>
-    <col min="1541" max="1541" width="10.5703125" style="19" customWidth="1"/>
-    <col min="1542" max="1542" width="11.5703125" style="19" customWidth="1"/>
-    <col min="1543" max="1543" width="10.85546875" style="19" customWidth="1"/>
-    <col min="1544" max="1544" width="11.140625" style="19" customWidth="1"/>
-    <col min="1545" max="1545" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="1546" max="1557" width="11.42578125" style="19" customWidth="1"/>
-    <col min="1558" max="1561" width="11.7109375" style="19" customWidth="1"/>
-    <col min="1562" max="1562" width="12.140625" style="19" customWidth="1"/>
-    <col min="1563" max="1563" width="11.85546875" style="19" customWidth="1"/>
-    <col min="1564" max="1792" width="9.140625" style="19"/>
-    <col min="1793" max="1793" width="22" style="19" customWidth="1"/>
-    <col min="1794" max="1794" width="12.42578125" style="19" customWidth="1"/>
-    <col min="1795" max="1795" width="12.140625" style="19" customWidth="1"/>
-    <col min="1796" max="1796" width="12.28515625" style="19" customWidth="1"/>
-    <col min="1797" max="1797" width="10.5703125" style="19" customWidth="1"/>
-    <col min="1798" max="1798" width="11.5703125" style="19" customWidth="1"/>
-    <col min="1799" max="1799" width="10.85546875" style="19" customWidth="1"/>
-    <col min="1800" max="1800" width="11.140625" style="19" customWidth="1"/>
-    <col min="1801" max="1801" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="1802" max="1813" width="11.42578125" style="19" customWidth="1"/>
-    <col min="1814" max="1817" width="11.7109375" style="19" customWidth="1"/>
-    <col min="1818" max="1818" width="12.140625" style="19" customWidth="1"/>
-    <col min="1819" max="1819" width="11.85546875" style="19" customWidth="1"/>
-    <col min="1820" max="2048" width="9.140625" style="19"/>
-    <col min="2049" max="2049" width="22" style="19" customWidth="1"/>
-    <col min="2050" max="2050" width="12.42578125" style="19" customWidth="1"/>
-    <col min="2051" max="2051" width="12.140625" style="19" customWidth="1"/>
-    <col min="2052" max="2052" width="12.28515625" style="19" customWidth="1"/>
-    <col min="2053" max="2053" width="10.5703125" style="19" customWidth="1"/>
-    <col min="2054" max="2054" width="11.5703125" style="19" customWidth="1"/>
-    <col min="2055" max="2055" width="10.85546875" style="19" customWidth="1"/>
-    <col min="2056" max="2056" width="11.140625" style="19" customWidth="1"/>
-    <col min="2057" max="2057" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="2058" max="2069" width="11.42578125" style="19" customWidth="1"/>
-    <col min="2070" max="2073" width="11.7109375" style="19" customWidth="1"/>
-    <col min="2074" max="2074" width="12.140625" style="19" customWidth="1"/>
-    <col min="2075" max="2075" width="11.85546875" style="19" customWidth="1"/>
-    <col min="2076" max="2304" width="9.140625" style="19"/>
-    <col min="2305" max="2305" width="22" style="19" customWidth="1"/>
-    <col min="2306" max="2306" width="12.42578125" style="19" customWidth="1"/>
-    <col min="2307" max="2307" width="12.140625" style="19" customWidth="1"/>
-    <col min="2308" max="2308" width="12.28515625" style="19" customWidth="1"/>
-    <col min="2309" max="2309" width="10.5703125" style="19" customWidth="1"/>
-    <col min="2310" max="2310" width="11.5703125" style="19" customWidth="1"/>
-    <col min="2311" max="2311" width="10.85546875" style="19" customWidth="1"/>
-    <col min="2312" max="2312" width="11.140625" style="19" customWidth="1"/>
-    <col min="2313" max="2313" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="2314" max="2325" width="11.42578125" style="19" customWidth="1"/>
-    <col min="2326" max="2329" width="11.7109375" style="19" customWidth="1"/>
-    <col min="2330" max="2330" width="12.140625" style="19" customWidth="1"/>
-    <col min="2331" max="2331" width="11.85546875" style="19" customWidth="1"/>
-    <col min="2332" max="2560" width="9.140625" style="19"/>
-    <col min="2561" max="2561" width="22" style="19" customWidth="1"/>
-    <col min="2562" max="2562" width="12.42578125" style="19" customWidth="1"/>
-    <col min="2563" max="2563" width="12.140625" style="19" customWidth="1"/>
-    <col min="2564" max="2564" width="12.28515625" style="19" customWidth="1"/>
-    <col min="2565" max="2565" width="10.5703125" style="19" customWidth="1"/>
-    <col min="2566" max="2566" width="11.5703125" style="19" customWidth="1"/>
-    <col min="2567" max="2567" width="10.85546875" style="19" customWidth="1"/>
-    <col min="2568" max="2568" width="11.140625" style="19" customWidth="1"/>
-    <col min="2569" max="2569" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="2570" max="2581" width="11.42578125" style="19" customWidth="1"/>
-    <col min="2582" max="2585" width="11.7109375" style="19" customWidth="1"/>
-    <col min="2586" max="2586" width="12.140625" style="19" customWidth="1"/>
-    <col min="2587" max="2587" width="11.85546875" style="19" customWidth="1"/>
-    <col min="2588" max="2816" width="9.140625" style="19"/>
-    <col min="2817" max="2817" width="22" style="19" customWidth="1"/>
-    <col min="2818" max="2818" width="12.42578125" style="19" customWidth="1"/>
-    <col min="2819" max="2819" width="12.140625" style="19" customWidth="1"/>
-    <col min="2820" max="2820" width="12.28515625" style="19" customWidth="1"/>
-    <col min="2821" max="2821" width="10.5703125" style="19" customWidth="1"/>
-    <col min="2822" max="2822" width="11.5703125" style="19" customWidth="1"/>
-    <col min="2823" max="2823" width="10.85546875" style="19" customWidth="1"/>
-    <col min="2824" max="2824" width="11.140625" style="19" customWidth="1"/>
-    <col min="2825" max="2825" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="2826" max="2837" width="11.42578125" style="19" customWidth="1"/>
-    <col min="2838" max="2841" width="11.7109375" style="19" customWidth="1"/>
-    <col min="2842" max="2842" width="12.140625" style="19" customWidth="1"/>
-    <col min="2843" max="2843" width="11.85546875" style="19" customWidth="1"/>
-    <col min="2844" max="3072" width="9.140625" style="19"/>
-    <col min="3073" max="3073" width="22" style="19" customWidth="1"/>
-    <col min="3074" max="3074" width="12.42578125" style="19" customWidth="1"/>
-    <col min="3075" max="3075" width="12.140625" style="19" customWidth="1"/>
-    <col min="3076" max="3076" width="12.28515625" style="19" customWidth="1"/>
-    <col min="3077" max="3077" width="10.5703125" style="19" customWidth="1"/>
-    <col min="3078" max="3078" width="11.5703125" style="19" customWidth="1"/>
-    <col min="3079" max="3079" width="10.85546875" style="19" customWidth="1"/>
-    <col min="3080" max="3080" width="11.140625" style="19" customWidth="1"/>
-    <col min="3081" max="3081" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="3082" max="3093" width="11.42578125" style="19" customWidth="1"/>
-    <col min="3094" max="3097" width="11.7109375" style="19" customWidth="1"/>
-    <col min="3098" max="3098" width="12.140625" style="19" customWidth="1"/>
-    <col min="3099" max="3099" width="11.85546875" style="19" customWidth="1"/>
-    <col min="3100" max="3328" width="9.140625" style="19"/>
-    <col min="3329" max="3329" width="22" style="19" customWidth="1"/>
-    <col min="3330" max="3330" width="12.42578125" style="19" customWidth="1"/>
-    <col min="3331" max="3331" width="12.140625" style="19" customWidth="1"/>
-    <col min="3332" max="3332" width="12.28515625" style="19" customWidth="1"/>
-    <col min="3333" max="3333" width="10.5703125" style="19" customWidth="1"/>
-    <col min="3334" max="3334" width="11.5703125" style="19" customWidth="1"/>
-    <col min="3335" max="3335" width="10.85546875" style="19" customWidth="1"/>
-    <col min="3336" max="3336" width="11.140625" style="19" customWidth="1"/>
-    <col min="3337" max="3337" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="3338" max="3349" width="11.42578125" style="19" customWidth="1"/>
-    <col min="3350" max="3353" width="11.7109375" style="19" customWidth="1"/>
-    <col min="3354" max="3354" width="12.140625" style="19" customWidth="1"/>
-    <col min="3355" max="3355" width="11.85546875" style="19" customWidth="1"/>
-    <col min="3356" max="3584" width="9.140625" style="19"/>
-    <col min="3585" max="3585" width="22" style="19" customWidth="1"/>
-    <col min="3586" max="3586" width="12.42578125" style="19" customWidth="1"/>
-    <col min="3587" max="3587" width="12.140625" style="19" customWidth="1"/>
-    <col min="3588" max="3588" width="12.28515625" style="19" customWidth="1"/>
-    <col min="3589" max="3589" width="10.5703125" style="19" customWidth="1"/>
-    <col min="3590" max="3590" width="11.5703125" style="19" customWidth="1"/>
-    <col min="3591" max="3591" width="10.85546875" style="19" customWidth="1"/>
-    <col min="3592" max="3592" width="11.140625" style="19" customWidth="1"/>
-    <col min="3593" max="3593" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="3594" max="3605" width="11.42578125" style="19" customWidth="1"/>
-    <col min="3606" max="3609" width="11.7109375" style="19" customWidth="1"/>
-    <col min="3610" max="3610" width="12.140625" style="19" customWidth="1"/>
-    <col min="3611" max="3611" width="11.85546875" style="19" customWidth="1"/>
-    <col min="3612" max="3840" width="9.140625" style="19"/>
-    <col min="3841" max="3841" width="22" style="19" customWidth="1"/>
-    <col min="3842" max="3842" width="12.42578125" style="19" customWidth="1"/>
-    <col min="3843" max="3843" width="12.140625" style="19" customWidth="1"/>
-    <col min="3844" max="3844" width="12.28515625" style="19" customWidth="1"/>
-    <col min="3845" max="3845" width="10.5703125" style="19" customWidth="1"/>
-    <col min="3846" max="3846" width="11.5703125" style="19" customWidth="1"/>
-    <col min="3847" max="3847" width="10.85546875" style="19" customWidth="1"/>
-    <col min="3848" max="3848" width="11.140625" style="19" customWidth="1"/>
-    <col min="3849" max="3849" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="3850" max="3861" width="11.42578125" style="19" customWidth="1"/>
-    <col min="3862" max="3865" width="11.7109375" style="19" customWidth="1"/>
-    <col min="3866" max="3866" width="12.140625" style="19" customWidth="1"/>
-    <col min="3867" max="3867" width="11.85546875" style="19" customWidth="1"/>
-    <col min="3868" max="4096" width="9.140625" style="19"/>
-    <col min="4097" max="4097" width="22" style="19" customWidth="1"/>
-    <col min="4098" max="4098" width="12.42578125" style="19" customWidth="1"/>
-    <col min="4099" max="4099" width="12.140625" style="19" customWidth="1"/>
-    <col min="4100" max="4100" width="12.28515625" style="19" customWidth="1"/>
-    <col min="4101" max="4101" width="10.5703125" style="19" customWidth="1"/>
-    <col min="4102" max="4102" width="11.5703125" style="19" customWidth="1"/>
-    <col min="4103" max="4103" width="10.85546875" style="19" customWidth="1"/>
-    <col min="4104" max="4104" width="11.140625" style="19" customWidth="1"/>
-    <col min="4105" max="4105" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="4106" max="4117" width="11.42578125" style="19" customWidth="1"/>
-    <col min="4118" max="4121" width="11.7109375" style="19" customWidth="1"/>
-    <col min="4122" max="4122" width="12.140625" style="19" customWidth="1"/>
-    <col min="4123" max="4123" width="11.85546875" style="19" customWidth="1"/>
-    <col min="4124" max="4352" width="9.140625" style="19"/>
-    <col min="4353" max="4353" width="22" style="19" customWidth="1"/>
-    <col min="4354" max="4354" width="12.42578125" style="19" customWidth="1"/>
-    <col min="4355" max="4355" width="12.140625" style="19" customWidth="1"/>
-    <col min="4356" max="4356" width="12.28515625" style="19" customWidth="1"/>
-    <col min="4357" max="4357" width="10.5703125" style="19" customWidth="1"/>
-    <col min="4358" max="4358" width="11.5703125" style="19" customWidth="1"/>
-    <col min="4359" max="4359" width="10.85546875" style="19" customWidth="1"/>
-    <col min="4360" max="4360" width="11.140625" style="19" customWidth="1"/>
-    <col min="4361" max="4361" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="4362" max="4373" width="11.42578125" style="19" customWidth="1"/>
-    <col min="4374" max="4377" width="11.7109375" style="19" customWidth="1"/>
-    <col min="4378" max="4378" width="12.140625" style="19" customWidth="1"/>
-    <col min="4379" max="4379" width="11.85546875" style="19" customWidth="1"/>
-    <col min="4380" max="4608" width="9.140625" style="19"/>
-    <col min="4609" max="4609" width="22" style="19" customWidth="1"/>
-    <col min="4610" max="4610" width="12.42578125" style="19" customWidth="1"/>
-    <col min="4611" max="4611" width="12.140625" style="19" customWidth="1"/>
-    <col min="4612" max="4612" width="12.28515625" style="19" customWidth="1"/>
-    <col min="4613" max="4613" width="10.5703125" style="19" customWidth="1"/>
-    <col min="4614" max="4614" width="11.5703125" style="19" customWidth="1"/>
-    <col min="4615" max="4615" width="10.85546875" style="19" customWidth="1"/>
-    <col min="4616" max="4616" width="11.140625" style="19" customWidth="1"/>
-    <col min="4617" max="4617" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="4618" max="4629" width="11.42578125" style="19" customWidth="1"/>
-    <col min="4630" max="4633" width="11.7109375" style="19" customWidth="1"/>
-    <col min="4634" max="4634" width="12.140625" style="19" customWidth="1"/>
-    <col min="4635" max="4635" width="11.85546875" style="19" customWidth="1"/>
-    <col min="4636" max="4864" width="9.140625" style="19"/>
-    <col min="4865" max="4865" width="22" style="19" customWidth="1"/>
-    <col min="4866" max="4866" width="12.42578125" style="19" customWidth="1"/>
-    <col min="4867" max="4867" width="12.140625" style="19" customWidth="1"/>
-    <col min="4868" max="4868" width="12.28515625" style="19" customWidth="1"/>
-    <col min="4869" max="4869" width="10.5703125" style="19" customWidth="1"/>
-    <col min="4870" max="4870" width="11.5703125" style="19" customWidth="1"/>
-    <col min="4871" max="4871" width="10.85546875" style="19" customWidth="1"/>
-    <col min="4872" max="4872" width="11.140625" style="19" customWidth="1"/>
-    <col min="4873" max="4873" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="4874" max="4885" width="11.42578125" style="19" customWidth="1"/>
-    <col min="4886" max="4889" width="11.7109375" style="19" customWidth="1"/>
-    <col min="4890" max="4890" width="12.140625" style="19" customWidth="1"/>
-    <col min="4891" max="4891" width="11.85546875" style="19" customWidth="1"/>
-    <col min="4892" max="5120" width="9.140625" style="19"/>
-    <col min="5121" max="5121" width="22" style="19" customWidth="1"/>
-    <col min="5122" max="5122" width="12.42578125" style="19" customWidth="1"/>
-    <col min="5123" max="5123" width="12.140625" style="19" customWidth="1"/>
-    <col min="5124" max="5124" width="12.28515625" style="19" customWidth="1"/>
-    <col min="5125" max="5125" width="10.5703125" style="19" customWidth="1"/>
-    <col min="5126" max="5126" width="11.5703125" style="19" customWidth="1"/>
-    <col min="5127" max="5127" width="10.85546875" style="19" customWidth="1"/>
-    <col min="5128" max="5128" width="11.140625" style="19" customWidth="1"/>
-    <col min="5129" max="5129" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="5130" max="5141" width="11.42578125" style="19" customWidth="1"/>
-    <col min="5142" max="5145" width="11.7109375" style="19" customWidth="1"/>
-    <col min="5146" max="5146" width="12.140625" style="19" customWidth="1"/>
-    <col min="5147" max="5147" width="11.85546875" style="19" customWidth="1"/>
-    <col min="5148" max="5376" width="9.140625" style="19"/>
-    <col min="5377" max="5377" width="22" style="19" customWidth="1"/>
-    <col min="5378" max="5378" width="12.42578125" style="19" customWidth="1"/>
-    <col min="5379" max="5379" width="12.140625" style="19" customWidth="1"/>
-    <col min="5380" max="5380" width="12.28515625" style="19" customWidth="1"/>
-    <col min="5381" max="5381" width="10.5703125" style="19" customWidth="1"/>
-    <col min="5382" max="5382" width="11.5703125" style="19" customWidth="1"/>
-    <col min="5383" max="5383" width="10.85546875" style="19" customWidth="1"/>
-    <col min="5384" max="5384" width="11.140625" style="19" customWidth="1"/>
-    <col min="5385" max="5385" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="5386" max="5397" width="11.42578125" style="19" customWidth="1"/>
-    <col min="5398" max="5401" width="11.7109375" style="19" customWidth="1"/>
-    <col min="5402" max="5402" width="12.140625" style="19" customWidth="1"/>
-    <col min="5403" max="5403" width="11.85546875" style="19" customWidth="1"/>
-    <col min="5404" max="5632" width="9.140625" style="19"/>
-    <col min="5633" max="5633" width="22" style="19" customWidth="1"/>
-    <col min="5634" max="5634" width="12.42578125" style="19" customWidth="1"/>
-    <col min="5635" max="5635" width="12.140625" style="19" customWidth="1"/>
-    <col min="5636" max="5636" width="12.28515625" style="19" customWidth="1"/>
-    <col min="5637" max="5637" width="10.5703125" style="19" customWidth="1"/>
-    <col min="5638" max="5638" width="11.5703125" style="19" customWidth="1"/>
-    <col min="5639" max="5639" width="10.85546875" style="19" customWidth="1"/>
-    <col min="5640" max="5640" width="11.140625" style="19" customWidth="1"/>
-    <col min="5641" max="5641" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="5642" max="5653" width="11.42578125" style="19" customWidth="1"/>
-    <col min="5654" max="5657" width="11.7109375" style="19" customWidth="1"/>
-    <col min="5658" max="5658" width="12.140625" style="19" customWidth="1"/>
-    <col min="5659" max="5659" width="11.85546875" style="19" customWidth="1"/>
-    <col min="5660" max="5888" width="9.140625" style="19"/>
-    <col min="5889" max="5889" width="22" style="19" customWidth="1"/>
-    <col min="5890" max="5890" width="12.42578125" style="19" customWidth="1"/>
-    <col min="5891" max="5891" width="12.140625" style="19" customWidth="1"/>
-    <col min="5892" max="5892" width="12.28515625" style="19" customWidth="1"/>
-    <col min="5893" max="5893" width="10.5703125" style="19" customWidth="1"/>
-    <col min="5894" max="5894" width="11.5703125" style="19" customWidth="1"/>
-    <col min="5895" max="5895" width="10.85546875" style="19" customWidth="1"/>
-    <col min="5896" max="5896" width="11.140625" style="19" customWidth="1"/>
-    <col min="5897" max="5897" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="5898" max="5909" width="11.42578125" style="19" customWidth="1"/>
-    <col min="5910" max="5913" width="11.7109375" style="19" customWidth="1"/>
-    <col min="5914" max="5914" width="12.140625" style="19" customWidth="1"/>
-    <col min="5915" max="5915" width="11.85546875" style="19" customWidth="1"/>
-    <col min="5916" max="6144" width="9.140625" style="19"/>
-    <col min="6145" max="6145" width="22" style="19" customWidth="1"/>
-    <col min="6146" max="6146" width="12.42578125" style="19" customWidth="1"/>
-    <col min="6147" max="6147" width="12.140625" style="19" customWidth="1"/>
-    <col min="6148" max="6148" width="12.28515625" style="19" customWidth="1"/>
-    <col min="6149" max="6149" width="10.5703125" style="19" customWidth="1"/>
-    <col min="6150" max="6150" width="11.5703125" style="19" customWidth="1"/>
-    <col min="6151" max="6151" width="10.85546875" style="19" customWidth="1"/>
-    <col min="6152" max="6152" width="11.140625" style="19" customWidth="1"/>
-    <col min="6153" max="6153" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="6154" max="6165" width="11.42578125" style="19" customWidth="1"/>
-    <col min="6166" max="6169" width="11.7109375" style="19" customWidth="1"/>
-    <col min="6170" max="6170" width="12.140625" style="19" customWidth="1"/>
-    <col min="6171" max="6171" width="11.85546875" style="19" customWidth="1"/>
-    <col min="6172" max="6400" width="9.140625" style="19"/>
-    <col min="6401" max="6401" width="22" style="19" customWidth="1"/>
-    <col min="6402" max="6402" width="12.42578125" style="19" customWidth="1"/>
-    <col min="6403" max="6403" width="12.140625" style="19" customWidth="1"/>
-    <col min="6404" max="6404" width="12.28515625" style="19" customWidth="1"/>
-    <col min="6405" max="6405" width="10.5703125" style="19" customWidth="1"/>
-    <col min="6406" max="6406" width="11.5703125" style="19" customWidth="1"/>
-    <col min="6407" max="6407" width="10.85546875" style="19" customWidth="1"/>
-    <col min="6408" max="6408" width="11.140625" style="19" customWidth="1"/>
-    <col min="6409" max="6409" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="6410" max="6421" width="11.42578125" style="19" customWidth="1"/>
-    <col min="6422" max="6425" width="11.7109375" style="19" customWidth="1"/>
-    <col min="6426" max="6426" width="12.140625" style="19" customWidth="1"/>
-    <col min="6427" max="6427" width="11.85546875" style="19" customWidth="1"/>
-    <col min="6428" max="6656" width="9.140625" style="19"/>
-    <col min="6657" max="6657" width="22" style="19" customWidth="1"/>
-    <col min="6658" max="6658" width="12.42578125" style="19" customWidth="1"/>
-    <col min="6659" max="6659" width="12.140625" style="19" customWidth="1"/>
-    <col min="6660" max="6660" width="12.28515625" style="19" customWidth="1"/>
-    <col min="6661" max="6661" width="10.5703125" style="19" customWidth="1"/>
-    <col min="6662" max="6662" width="11.5703125" style="19" customWidth="1"/>
-    <col min="6663" max="6663" width="10.85546875" style="19" customWidth="1"/>
-    <col min="6664" max="6664" width="11.140625" style="19" customWidth="1"/>
-    <col min="6665" max="6665" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="6666" max="6677" width="11.42578125" style="19" customWidth="1"/>
-    <col min="6678" max="6681" width="11.7109375" style="19" customWidth="1"/>
-    <col min="6682" max="6682" width="12.140625" style="19" customWidth="1"/>
-    <col min="6683" max="6683" width="11.85546875" style="19" customWidth="1"/>
-    <col min="6684" max="6912" width="9.140625" style="19"/>
-    <col min="6913" max="6913" width="22" style="19" customWidth="1"/>
-    <col min="6914" max="6914" width="12.42578125" style="19" customWidth="1"/>
-    <col min="6915" max="6915" width="12.140625" style="19" customWidth="1"/>
-    <col min="6916" max="6916" width="12.28515625" style="19" customWidth="1"/>
-    <col min="6917" max="6917" width="10.5703125" style="19" customWidth="1"/>
-    <col min="6918" max="6918" width="11.5703125" style="19" customWidth="1"/>
-    <col min="6919" max="6919" width="10.85546875" style="19" customWidth="1"/>
-    <col min="6920" max="6920" width="11.140625" style="19" customWidth="1"/>
-    <col min="6921" max="6921" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="6922" max="6933" width="11.42578125" style="19" customWidth="1"/>
-    <col min="6934" max="6937" width="11.7109375" style="19" customWidth="1"/>
-    <col min="6938" max="6938" width="12.140625" style="19" customWidth="1"/>
-    <col min="6939" max="6939" width="11.85546875" style="19" customWidth="1"/>
-    <col min="6940" max="7168" width="9.140625" style="19"/>
-    <col min="7169" max="7169" width="22" style="19" customWidth="1"/>
-    <col min="7170" max="7170" width="12.42578125" style="19" customWidth="1"/>
-    <col min="7171" max="7171" width="12.140625" style="19" customWidth="1"/>
-    <col min="7172" max="7172" width="12.28515625" style="19" customWidth="1"/>
-    <col min="7173" max="7173" width="10.5703125" style="19" customWidth="1"/>
-    <col min="7174" max="7174" width="11.5703125" style="19" customWidth="1"/>
-    <col min="7175" max="7175" width="10.85546875" style="19" customWidth="1"/>
-    <col min="7176" max="7176" width="11.140625" style="19" customWidth="1"/>
-    <col min="7177" max="7177" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="7178" max="7189" width="11.42578125" style="19" customWidth="1"/>
-    <col min="7190" max="7193" width="11.7109375" style="19" customWidth="1"/>
-    <col min="7194" max="7194" width="12.140625" style="19" customWidth="1"/>
-    <col min="7195" max="7195" width="11.85546875" style="19" customWidth="1"/>
-    <col min="7196" max="7424" width="9.140625" style="19"/>
-    <col min="7425" max="7425" width="22" style="19" customWidth="1"/>
-    <col min="7426" max="7426" width="12.42578125" style="19" customWidth="1"/>
-    <col min="7427" max="7427" width="12.140625" style="19" customWidth="1"/>
-    <col min="7428" max="7428" width="12.28515625" style="19" customWidth="1"/>
-    <col min="7429" max="7429" width="10.5703125" style="19" customWidth="1"/>
-    <col min="7430" max="7430" width="11.5703125" style="19" customWidth="1"/>
-    <col min="7431" max="7431" width="10.85546875" style="19" customWidth="1"/>
-    <col min="7432" max="7432" width="11.140625" style="19" customWidth="1"/>
-    <col min="7433" max="7433" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="7434" max="7445" width="11.42578125" style="19" customWidth="1"/>
-    <col min="7446" max="7449" width="11.7109375" style="19" customWidth="1"/>
-    <col min="7450" max="7450" width="12.140625" style="19" customWidth="1"/>
-    <col min="7451" max="7451" width="11.85546875" style="19" customWidth="1"/>
-    <col min="7452" max="7680" width="9.140625" style="19"/>
-    <col min="7681" max="7681" width="22" style="19" customWidth="1"/>
-    <col min="7682" max="7682" width="12.42578125" style="19" customWidth="1"/>
-    <col min="7683" max="7683" width="12.140625" style="19" customWidth="1"/>
-    <col min="7684" max="7684" width="12.28515625" style="19" customWidth="1"/>
-    <col min="7685" max="7685" width="10.5703125" style="19" customWidth="1"/>
-    <col min="7686" max="7686" width="11.5703125" style="19" customWidth="1"/>
-    <col min="7687" max="7687" width="10.85546875" style="19" customWidth="1"/>
-    <col min="7688" max="7688" width="11.140625" style="19" customWidth="1"/>
-    <col min="7689" max="7689" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="7690" max="7701" width="11.42578125" style="19" customWidth="1"/>
-    <col min="7702" max="7705" width="11.7109375" style="19" customWidth="1"/>
-    <col min="7706" max="7706" width="12.140625" style="19" customWidth="1"/>
-    <col min="7707" max="7707" width="11.85546875" style="19" customWidth="1"/>
-    <col min="7708" max="7936" width="9.140625" style="19"/>
-    <col min="7937" max="7937" width="22" style="19" customWidth="1"/>
-    <col min="7938" max="7938" width="12.42578125" style="19" customWidth="1"/>
-    <col min="7939" max="7939" width="12.140625" style="19" customWidth="1"/>
-    <col min="7940" max="7940" width="12.28515625" style="19" customWidth="1"/>
-    <col min="7941" max="7941" width="10.5703125" style="19" customWidth="1"/>
-    <col min="7942" max="7942" width="11.5703125" style="19" customWidth="1"/>
-    <col min="7943" max="7943" width="10.85546875" style="19" customWidth="1"/>
-    <col min="7944" max="7944" width="11.140625" style="19" customWidth="1"/>
-    <col min="7945" max="7945" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="7946" max="7957" width="11.42578125" style="19" customWidth="1"/>
-    <col min="7958" max="7961" width="11.7109375" style="19" customWidth="1"/>
-    <col min="7962" max="7962" width="12.140625" style="19" customWidth="1"/>
-    <col min="7963" max="7963" width="11.85546875" style="19" customWidth="1"/>
-    <col min="7964" max="8192" width="9.140625" style="19"/>
-    <col min="8193" max="8193" width="22" style="19" customWidth="1"/>
-    <col min="8194" max="8194" width="12.42578125" style="19" customWidth="1"/>
-    <col min="8195" max="8195" width="12.140625" style="19" customWidth="1"/>
-    <col min="8196" max="8196" width="12.28515625" style="19" customWidth="1"/>
-    <col min="8197" max="8197" width="10.5703125" style="19" customWidth="1"/>
-    <col min="8198" max="8198" width="11.5703125" style="19" customWidth="1"/>
-    <col min="8199" max="8199" width="10.85546875" style="19" customWidth="1"/>
-    <col min="8200" max="8200" width="11.140625" style="19" customWidth="1"/>
-    <col min="8201" max="8201" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="8202" max="8213" width="11.42578125" style="19" customWidth="1"/>
-    <col min="8214" max="8217" width="11.7109375" style="19" customWidth="1"/>
-    <col min="8218" max="8218" width="12.140625" style="19" customWidth="1"/>
-    <col min="8219" max="8219" width="11.85546875" style="19" customWidth="1"/>
-    <col min="8220" max="8448" width="9.140625" style="19"/>
-    <col min="8449" max="8449" width="22" style="19" customWidth="1"/>
-    <col min="8450" max="8450" width="12.42578125" style="19" customWidth="1"/>
-    <col min="8451" max="8451" width="12.140625" style="19" customWidth="1"/>
-    <col min="8452" max="8452" width="12.28515625" style="19" customWidth="1"/>
-    <col min="8453" max="8453" width="10.5703125" style="19" customWidth="1"/>
-    <col min="8454" max="8454" width="11.5703125" style="19" customWidth="1"/>
-    <col min="8455" max="8455" width="10.85546875" style="19" customWidth="1"/>
-    <col min="8456" max="8456" width="11.140625" style="19" customWidth="1"/>
-    <col min="8457" max="8457" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="8458" max="8469" width="11.42578125" style="19" customWidth="1"/>
-    <col min="8470" max="8473" width="11.7109375" style="19" customWidth="1"/>
-    <col min="8474" max="8474" width="12.140625" style="19" customWidth="1"/>
-    <col min="8475" max="8475" width="11.85546875" style="19" customWidth="1"/>
-    <col min="8476" max="8704" width="9.140625" style="19"/>
-    <col min="8705" max="8705" width="22" style="19" customWidth="1"/>
-    <col min="8706" max="8706" width="12.42578125" style="19" customWidth="1"/>
-    <col min="8707" max="8707" width="12.140625" style="19" customWidth="1"/>
-    <col min="8708" max="8708" width="12.28515625" style="19" customWidth="1"/>
-    <col min="8709" max="8709" width="10.5703125" style="19" customWidth="1"/>
-    <col min="8710" max="8710" width="11.5703125" style="19" customWidth="1"/>
-    <col min="8711" max="8711" width="10.85546875" style="19" customWidth="1"/>
-    <col min="8712" max="8712" width="11.140625" style="19" customWidth="1"/>
-    <col min="8713" max="8713" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="8714" max="8725" width="11.42578125" style="19" customWidth="1"/>
-    <col min="8726" max="8729" width="11.7109375" style="19" customWidth="1"/>
-    <col min="8730" max="8730" width="12.140625" style="19" customWidth="1"/>
-    <col min="8731" max="8731" width="11.85546875" style="19" customWidth="1"/>
-    <col min="8732" max="8960" width="9.140625" style="19"/>
-    <col min="8961" max="8961" width="22" style="19" customWidth="1"/>
-    <col min="8962" max="8962" width="12.42578125" style="19" customWidth="1"/>
-    <col min="8963" max="8963" width="12.140625" style="19" customWidth="1"/>
-    <col min="8964" max="8964" width="12.28515625" style="19" customWidth="1"/>
-    <col min="8965" max="8965" width="10.5703125" style="19" customWidth="1"/>
-    <col min="8966" max="8966" width="11.5703125" style="19" customWidth="1"/>
-    <col min="8967" max="8967" width="10.85546875" style="19" customWidth="1"/>
-    <col min="8968" max="8968" width="11.140625" style="19" customWidth="1"/>
-    <col min="8969" max="8969" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="8970" max="8981" width="11.42578125" style="19" customWidth="1"/>
-    <col min="8982" max="8985" width="11.7109375" style="19" customWidth="1"/>
-    <col min="8986" max="8986" width="12.140625" style="19" customWidth="1"/>
-    <col min="8987" max="8987" width="11.85546875" style="19" customWidth="1"/>
-    <col min="8988" max="9216" width="9.140625" style="19"/>
-    <col min="9217" max="9217" width="22" style="19" customWidth="1"/>
-    <col min="9218" max="9218" width="12.42578125" style="19" customWidth="1"/>
-    <col min="9219" max="9219" width="12.140625" style="19" customWidth="1"/>
-    <col min="9220" max="9220" width="12.28515625" style="19" customWidth="1"/>
-    <col min="9221" max="9221" width="10.5703125" style="19" customWidth="1"/>
-    <col min="9222" max="9222" width="11.5703125" style="19" customWidth="1"/>
-    <col min="9223" max="9223" width="10.85546875" style="19" customWidth="1"/>
-    <col min="9224" max="9224" width="11.140625" style="19" customWidth="1"/>
-    <col min="9225" max="9225" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="9226" max="9237" width="11.42578125" style="19" customWidth="1"/>
-    <col min="9238" max="9241" width="11.7109375" style="19" customWidth="1"/>
-    <col min="9242" max="9242" width="12.140625" style="19" customWidth="1"/>
-    <col min="9243" max="9243" width="11.85546875" style="19" customWidth="1"/>
-    <col min="9244" max="9472" width="9.140625" style="19"/>
-    <col min="9473" max="9473" width="22" style="19" customWidth="1"/>
-    <col min="9474" max="9474" width="12.42578125" style="19" customWidth="1"/>
-    <col min="9475" max="9475" width="12.140625" style="19" customWidth="1"/>
-    <col min="9476" max="9476" width="12.28515625" style="19" customWidth="1"/>
-    <col min="9477" max="9477" width="10.5703125" style="19" customWidth="1"/>
-    <col min="9478" max="9478" width="11.5703125" style="19" customWidth="1"/>
-    <col min="9479" max="9479" width="10.85546875" style="19" customWidth="1"/>
-    <col min="9480" max="9480" width="11.140625" style="19" customWidth="1"/>
-    <col min="9481" max="9481" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="9482" max="9493" width="11.42578125" style="19" customWidth="1"/>
-    <col min="9494" max="9497" width="11.7109375" style="19" customWidth="1"/>
-    <col min="9498" max="9498" width="12.140625" style="19" customWidth="1"/>
-    <col min="9499" max="9499" width="11.85546875" style="19" customWidth="1"/>
-    <col min="9500" max="9728" width="9.140625" style="19"/>
-    <col min="9729" max="9729" width="22" style="19" customWidth="1"/>
-    <col min="9730" max="9730" width="12.42578125" style="19" customWidth="1"/>
-    <col min="9731" max="9731" width="12.140625" style="19" customWidth="1"/>
-    <col min="9732" max="9732" width="12.28515625" style="19" customWidth="1"/>
-    <col min="9733" max="9733" width="10.5703125" style="19" customWidth="1"/>
-    <col min="9734" max="9734" width="11.5703125" style="19" customWidth="1"/>
-    <col min="9735" max="9735" width="10.85546875" style="19" customWidth="1"/>
-    <col min="9736" max="9736" width="11.140625" style="19" customWidth="1"/>
-    <col min="9737" max="9737" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="9738" max="9749" width="11.42578125" style="19" customWidth="1"/>
-    <col min="9750" max="9753" width="11.7109375" style="19" customWidth="1"/>
-    <col min="9754" max="9754" width="12.140625" style="19" customWidth="1"/>
-    <col min="9755" max="9755" width="11.85546875" style="19" customWidth="1"/>
-    <col min="9756" max="9984" width="9.140625" style="19"/>
-    <col min="9985" max="9985" width="22" style="19" customWidth="1"/>
-    <col min="9986" max="9986" width="12.42578125" style="19" customWidth="1"/>
-    <col min="9987" max="9987" width="12.140625" style="19" customWidth="1"/>
-    <col min="9988" max="9988" width="12.28515625" style="19" customWidth="1"/>
-    <col min="9989" max="9989" width="10.5703125" style="19" customWidth="1"/>
-    <col min="9990" max="9990" width="11.5703125" style="19" customWidth="1"/>
-    <col min="9991" max="9991" width="10.85546875" style="19" customWidth="1"/>
-    <col min="9992" max="9992" width="11.140625" style="19" customWidth="1"/>
-    <col min="9993" max="9993" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="9994" max="10005" width="11.42578125" style="19" customWidth="1"/>
-    <col min="10006" max="10009" width="11.7109375" style="19" customWidth="1"/>
-    <col min="10010" max="10010" width="12.140625" style="19" customWidth="1"/>
-    <col min="10011" max="10011" width="11.85546875" style="19" customWidth="1"/>
-    <col min="10012" max="10240" width="9.140625" style="19"/>
-    <col min="10241" max="10241" width="22" style="19" customWidth="1"/>
-    <col min="10242" max="10242" width="12.42578125" style="19" customWidth="1"/>
-    <col min="10243" max="10243" width="12.140625" style="19" customWidth="1"/>
-    <col min="10244" max="10244" width="12.28515625" style="19" customWidth="1"/>
-    <col min="10245" max="10245" width="10.5703125" style="19" customWidth="1"/>
-    <col min="10246" max="10246" width="11.5703125" style="19" customWidth="1"/>
-    <col min="10247" max="10247" width="10.85546875" style="19" customWidth="1"/>
-    <col min="10248" max="10248" width="11.140625" style="19" customWidth="1"/>
-    <col min="10249" max="10249" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="10250" max="10261" width="11.42578125" style="19" customWidth="1"/>
-    <col min="10262" max="10265" width="11.7109375" style="19" customWidth="1"/>
-    <col min="10266" max="10266" width="12.140625" style="19" customWidth="1"/>
-    <col min="10267" max="10267" width="11.85546875" style="19" customWidth="1"/>
-    <col min="10268" max="10496" width="9.140625" style="19"/>
-    <col min="10497" max="10497" width="22" style="19" customWidth="1"/>
-    <col min="10498" max="10498" width="12.42578125" style="19" customWidth="1"/>
-    <col min="10499" max="10499" width="12.140625" style="19" customWidth="1"/>
-    <col min="10500" max="10500" width="12.28515625" style="19" customWidth="1"/>
-    <col min="10501" max="10501" width="10.5703125" style="19" customWidth="1"/>
-    <col min="10502" max="10502" width="11.5703125" style="19" customWidth="1"/>
-    <col min="10503" max="10503" width="10.85546875" style="19" customWidth="1"/>
-    <col min="10504" max="10504" width="11.140625" style="19" customWidth="1"/>
-    <col min="10505" max="10505" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="10506" max="10517" width="11.42578125" style="19" customWidth="1"/>
-    <col min="10518" max="10521" width="11.7109375" style="19" customWidth="1"/>
-    <col min="10522" max="10522" width="12.140625" style="19" customWidth="1"/>
-    <col min="10523" max="10523" width="11.85546875" style="19" customWidth="1"/>
-    <col min="10524" max="10752" width="9.140625" style="19"/>
-    <col min="10753" max="10753" width="22" style="19" customWidth="1"/>
-    <col min="10754" max="10754" width="12.42578125" style="19" customWidth="1"/>
-    <col min="10755" max="10755" width="12.140625" style="19" customWidth="1"/>
-    <col min="10756" max="10756" width="12.28515625" style="19" customWidth="1"/>
-    <col min="10757" max="10757" width="10.5703125" style="19" customWidth="1"/>
-    <col min="10758" max="10758" width="11.5703125" style="19" customWidth="1"/>
-    <col min="10759" max="10759" width="10.85546875" style="19" customWidth="1"/>
-    <col min="10760" max="10760" width="11.140625" style="19" customWidth="1"/>
-    <col min="10761" max="10761" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="10762" max="10773" width="11.42578125" style="19" customWidth="1"/>
-    <col min="10774" max="10777" width="11.7109375" style="19" customWidth="1"/>
-    <col min="10778" max="10778" width="12.140625" style="19" customWidth="1"/>
-    <col min="10779" max="10779" width="11.85546875" style="19" customWidth="1"/>
-    <col min="10780" max="11008" width="9.140625" style="19"/>
-    <col min="11009" max="11009" width="22" style="19" customWidth="1"/>
-    <col min="11010" max="11010" width="12.42578125" style="19" customWidth="1"/>
-    <col min="11011" max="11011" width="12.140625" style="19" customWidth="1"/>
-    <col min="11012" max="11012" width="12.28515625" style="19" customWidth="1"/>
-    <col min="11013" max="11013" width="10.5703125" style="19" customWidth="1"/>
-    <col min="11014" max="11014" width="11.5703125" style="19" customWidth="1"/>
-    <col min="11015" max="11015" width="10.85546875" style="19" customWidth="1"/>
-    <col min="11016" max="11016" width="11.140625" style="19" customWidth="1"/>
-    <col min="11017" max="11017" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="11018" max="11029" width="11.42578125" style="19" customWidth="1"/>
-    <col min="11030" max="11033" width="11.7109375" style="19" customWidth="1"/>
-    <col min="11034" max="11034" width="12.140625" style="19" customWidth="1"/>
-    <col min="11035" max="11035" width="11.85546875" style="19" customWidth="1"/>
-    <col min="11036" max="11264" width="9.140625" style="19"/>
-    <col min="11265" max="11265" width="22" style="19" customWidth="1"/>
-    <col min="11266" max="11266" width="12.42578125" style="19" customWidth="1"/>
-    <col min="11267" max="11267" width="12.140625" style="19" customWidth="1"/>
-    <col min="11268" max="11268" width="12.28515625" style="19" customWidth="1"/>
-    <col min="11269" max="11269" width="10.5703125" style="19" customWidth="1"/>
-    <col min="11270" max="11270" width="11.5703125" style="19" customWidth="1"/>
-    <col min="11271" max="11271" width="10.85546875" style="19" customWidth="1"/>
-    <col min="11272" max="11272" width="11.140625" style="19" customWidth="1"/>
-    <col min="11273" max="11273" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="11274" max="11285" width="11.42578125" style="19" customWidth="1"/>
-    <col min="11286" max="11289" width="11.7109375" style="19" customWidth="1"/>
-    <col min="11290" max="11290" width="12.140625" style="19" customWidth="1"/>
-    <col min="11291" max="11291" width="11.85546875" style="19" customWidth="1"/>
-    <col min="11292" max="11520" width="9.140625" style="19"/>
-    <col min="11521" max="11521" width="22" style="19" customWidth="1"/>
-    <col min="11522" max="11522" width="12.42578125" style="19" customWidth="1"/>
-    <col min="11523" max="11523" width="12.140625" style="19" customWidth="1"/>
-    <col min="11524" max="11524" width="12.28515625" style="19" customWidth="1"/>
-    <col min="11525" max="11525" width="10.5703125" style="19" customWidth="1"/>
-    <col min="11526" max="11526" width="11.5703125" style="19" customWidth="1"/>
-    <col min="11527" max="11527" width="10.85546875" style="19" customWidth="1"/>
-    <col min="11528" max="11528" width="11.140625" style="19" customWidth="1"/>
-    <col min="11529" max="11529" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="11530" max="11541" width="11.42578125" style="19" customWidth="1"/>
-    <col min="11542" max="11545" width="11.7109375" style="19" customWidth="1"/>
-    <col min="11546" max="11546" width="12.140625" style="19" customWidth="1"/>
-    <col min="11547" max="11547" width="11.85546875" style="19" customWidth="1"/>
-    <col min="11548" max="11776" width="9.140625" style="19"/>
-    <col min="11777" max="11777" width="22" style="19" customWidth="1"/>
-    <col min="11778" max="11778" width="12.42578125" style="19" customWidth="1"/>
-    <col min="11779" max="11779" width="12.140625" style="19" customWidth="1"/>
-    <col min="11780" max="11780" width="12.28515625" style="19" customWidth="1"/>
-    <col min="11781" max="11781" width="10.5703125" style="19" customWidth="1"/>
-    <col min="11782" max="11782" width="11.5703125" style="19" customWidth="1"/>
-    <col min="11783" max="11783" width="10.85546875" style="19" customWidth="1"/>
-    <col min="11784" max="11784" width="11.140625" style="19" customWidth="1"/>
-    <col min="11785" max="11785" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="11786" max="11797" width="11.42578125" style="19" customWidth="1"/>
-    <col min="11798" max="11801" width="11.7109375" style="19" customWidth="1"/>
-    <col min="11802" max="11802" width="12.140625" style="19" customWidth="1"/>
-    <col min="11803" max="11803" width="11.85546875" style="19" customWidth="1"/>
-    <col min="11804" max="12032" width="9.140625" style="19"/>
-    <col min="12033" max="12033" width="22" style="19" customWidth="1"/>
-    <col min="12034" max="12034" width="12.42578125" style="19" customWidth="1"/>
-    <col min="12035" max="12035" width="12.140625" style="19" customWidth="1"/>
-    <col min="12036" max="12036" width="12.28515625" style="19" customWidth="1"/>
-    <col min="12037" max="12037" width="10.5703125" style="19" customWidth="1"/>
-    <col min="12038" max="12038" width="11.5703125" style="19" customWidth="1"/>
-    <col min="12039" max="12039" width="10.85546875" style="19" customWidth="1"/>
-    <col min="12040" max="12040" width="11.140625" style="19" customWidth="1"/>
-    <col min="12041" max="12041" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="12042" max="12053" width="11.42578125" style="19" customWidth="1"/>
-    <col min="12054" max="12057" width="11.7109375" style="19" customWidth="1"/>
-    <col min="12058" max="12058" width="12.140625" style="19" customWidth="1"/>
-    <col min="12059" max="12059" width="11.85546875" style="19" customWidth="1"/>
-    <col min="12060" max="12288" width="9.140625" style="19"/>
-    <col min="12289" max="12289" width="22" style="19" customWidth="1"/>
-    <col min="12290" max="12290" width="12.42578125" style="19" customWidth="1"/>
-    <col min="12291" max="12291" width="12.140625" style="19" customWidth="1"/>
-    <col min="12292" max="12292" width="12.28515625" style="19" customWidth="1"/>
-    <col min="12293" max="12293" width="10.5703125" style="19" customWidth="1"/>
-    <col min="12294" max="12294" width="11.5703125" style="19" customWidth="1"/>
-    <col min="12295" max="12295" width="10.85546875" style="19" customWidth="1"/>
-    <col min="12296" max="12296" width="11.140625" style="19" customWidth="1"/>
-    <col min="12297" max="12297" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="12298" max="12309" width="11.42578125" style="19" customWidth="1"/>
-    <col min="12310" max="12313" width="11.7109375" style="19" customWidth="1"/>
-    <col min="12314" max="12314" width="12.140625" style="19" customWidth="1"/>
-    <col min="12315" max="12315" width="11.85546875" style="19" customWidth="1"/>
-    <col min="12316" max="12544" width="9.140625" style="19"/>
-    <col min="12545" max="12545" width="22" style="19" customWidth="1"/>
-    <col min="12546" max="12546" width="12.42578125" style="19" customWidth="1"/>
-    <col min="12547" max="12547" width="12.140625" style="19" customWidth="1"/>
-    <col min="12548" max="12548" width="12.28515625" style="19" customWidth="1"/>
-    <col min="12549" max="12549" width="10.5703125" style="19" customWidth="1"/>
-    <col min="12550" max="12550" width="11.5703125" style="19" customWidth="1"/>
-    <col min="12551" max="12551" width="10.85546875" style="19" customWidth="1"/>
-    <col min="12552" max="12552" width="11.140625" style="19" customWidth="1"/>
-    <col min="12553" max="12553" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="12554" max="12565" width="11.42578125" style="19" customWidth="1"/>
-    <col min="12566" max="12569" width="11.7109375" style="19" customWidth="1"/>
-    <col min="12570" max="12570" width="12.140625" style="19" customWidth="1"/>
-    <col min="12571" max="12571" width="11.85546875" style="19" customWidth="1"/>
-    <col min="12572" max="12800" width="9.140625" style="19"/>
-    <col min="12801" max="12801" width="22" style="19" customWidth="1"/>
-    <col min="12802" max="12802" width="12.42578125" style="19" customWidth="1"/>
-    <col min="12803" max="12803" width="12.140625" style="19" customWidth="1"/>
-    <col min="12804" max="12804" width="12.28515625" style="19" customWidth="1"/>
-    <col min="12805" max="12805" width="10.5703125" style="19" customWidth="1"/>
-    <col min="12806" max="12806" width="11.5703125" style="19" customWidth="1"/>
-    <col min="12807" max="12807" width="10.85546875" style="19" customWidth="1"/>
-    <col min="12808" max="12808" width="11.140625" style="19" customWidth="1"/>
-    <col min="12809" max="12809" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="12810" max="12821" width="11.42578125" style="19" customWidth="1"/>
-    <col min="12822" max="12825" width="11.7109375" style="19" customWidth="1"/>
-    <col min="12826" max="12826" width="12.140625" style="19" customWidth="1"/>
-    <col min="12827" max="12827" width="11.85546875" style="19" customWidth="1"/>
-    <col min="12828" max="13056" width="9.140625" style="19"/>
-    <col min="13057" max="13057" width="22" style="19" customWidth="1"/>
-    <col min="13058" max="13058" width="12.42578125" style="19" customWidth="1"/>
-    <col min="13059" max="13059" width="12.140625" style="19" customWidth="1"/>
-    <col min="13060" max="13060" width="12.28515625" style="19" customWidth="1"/>
-    <col min="13061" max="13061" width="10.5703125" style="19" customWidth="1"/>
-    <col min="13062" max="13062" width="11.5703125" style="19" customWidth="1"/>
-    <col min="13063" max="13063" width="10.85546875" style="19" customWidth="1"/>
-    <col min="13064" max="13064" width="11.140625" style="19" customWidth="1"/>
-    <col min="13065" max="13065" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="13066" max="13077" width="11.42578125" style="19" customWidth="1"/>
-    <col min="13078" max="13081" width="11.7109375" style="19" customWidth="1"/>
-    <col min="13082" max="13082" width="12.140625" style="19" customWidth="1"/>
-    <col min="13083" max="13083" width="11.85546875" style="19" customWidth="1"/>
-    <col min="13084" max="13312" width="9.140625" style="19"/>
-    <col min="13313" max="13313" width="22" style="19" customWidth="1"/>
-    <col min="13314" max="13314" width="12.42578125" style="19" customWidth="1"/>
-    <col min="13315" max="13315" width="12.140625" style="19" customWidth="1"/>
-    <col min="13316" max="13316" width="12.28515625" style="19" customWidth="1"/>
-    <col min="13317" max="13317" width="10.5703125" style="19" customWidth="1"/>
-    <col min="13318" max="13318" width="11.5703125" style="19" customWidth="1"/>
-    <col min="13319" max="13319" width="10.85546875" style="19" customWidth="1"/>
-    <col min="13320" max="13320" width="11.140625" style="19" customWidth="1"/>
-    <col min="13321" max="13321" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="13322" max="13333" width="11.42578125" style="19" customWidth="1"/>
-    <col min="13334" max="13337" width="11.7109375" style="19" customWidth="1"/>
-    <col min="13338" max="13338" width="12.140625" style="19" customWidth="1"/>
-    <col min="13339" max="13339" width="11.85546875" style="19" customWidth="1"/>
-    <col min="13340" max="13568" width="9.140625" style="19"/>
-    <col min="13569" max="13569" width="22" style="19" customWidth="1"/>
-    <col min="13570" max="13570" width="12.42578125" style="19" customWidth="1"/>
-    <col min="13571" max="13571" width="12.140625" style="19" customWidth="1"/>
-    <col min="13572" max="13572" width="12.28515625" style="19" customWidth="1"/>
-    <col min="13573" max="13573" width="10.5703125" style="19" customWidth="1"/>
-    <col min="13574" max="13574" width="11.5703125" style="19" customWidth="1"/>
-    <col min="13575" max="13575" width="10.85546875" style="19" customWidth="1"/>
-    <col min="13576" max="13576" width="11.140625" style="19" customWidth="1"/>
-    <col min="13577" max="13577" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="13578" max="13589" width="11.42578125" style="19" customWidth="1"/>
-    <col min="13590" max="13593" width="11.7109375" style="19" customWidth="1"/>
-    <col min="13594" max="13594" width="12.140625" style="19" customWidth="1"/>
-    <col min="13595" max="13595" width="11.85546875" style="19" customWidth="1"/>
-    <col min="13596" max="13824" width="9.140625" style="19"/>
-    <col min="13825" max="13825" width="22" style="19" customWidth="1"/>
-    <col min="13826" max="13826" width="12.42578125" style="19" customWidth="1"/>
-    <col min="13827" max="13827" width="12.140625" style="19" customWidth="1"/>
-    <col min="13828" max="13828" width="12.28515625" style="19" customWidth="1"/>
-    <col min="13829" max="13829" width="10.5703125" style="19" customWidth="1"/>
-    <col min="13830" max="13830" width="11.5703125" style="19" customWidth="1"/>
-    <col min="13831" max="13831" width="10.85546875" style="19" customWidth="1"/>
-    <col min="13832" max="13832" width="11.140625" style="19" customWidth="1"/>
-    <col min="13833" max="13833" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="13834" max="13845" width="11.42578125" style="19" customWidth="1"/>
-    <col min="13846" max="13849" width="11.7109375" style="19" customWidth="1"/>
-    <col min="13850" max="13850" width="12.140625" style="19" customWidth="1"/>
-    <col min="13851" max="13851" width="11.85546875" style="19" customWidth="1"/>
-    <col min="13852" max="14080" width="9.140625" style="19"/>
-    <col min="14081" max="14081" width="22" style="19" customWidth="1"/>
-    <col min="14082" max="14082" width="12.42578125" style="19" customWidth="1"/>
-    <col min="14083" max="14083" width="12.140625" style="19" customWidth="1"/>
-    <col min="14084" max="14084" width="12.28515625" style="19" customWidth="1"/>
-    <col min="14085" max="14085" width="10.5703125" style="19" customWidth="1"/>
-    <col min="14086" max="14086" width="11.5703125" style="19" customWidth="1"/>
-    <col min="14087" max="14087" width="10.85546875" style="19" customWidth="1"/>
-    <col min="14088" max="14088" width="11.140625" style="19" customWidth="1"/>
-    <col min="14089" max="14089" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="14090" max="14101" width="11.42578125" style="19" customWidth="1"/>
-    <col min="14102" max="14105" width="11.7109375" style="19" customWidth="1"/>
-    <col min="14106" max="14106" width="12.140625" style="19" customWidth="1"/>
-    <col min="14107" max="14107" width="11.85546875" style="19" customWidth="1"/>
-    <col min="14108" max="14336" width="9.140625" style="19"/>
-    <col min="14337" max="14337" width="22" style="19" customWidth="1"/>
-    <col min="14338" max="14338" width="12.42578125" style="19" customWidth="1"/>
-    <col min="14339" max="14339" width="12.140625" style="19" customWidth="1"/>
-    <col min="14340" max="14340" width="12.28515625" style="19" customWidth="1"/>
-    <col min="14341" max="14341" width="10.5703125" style="19" customWidth="1"/>
-    <col min="14342" max="14342" width="11.5703125" style="19" customWidth="1"/>
-    <col min="14343" max="14343" width="10.85546875" style="19" customWidth="1"/>
-    <col min="14344" max="14344" width="11.140625" style="19" customWidth="1"/>
-    <col min="14345" max="14345" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="14346" max="14357" width="11.42578125" style="19" customWidth="1"/>
-    <col min="14358" max="14361" width="11.7109375" style="19" customWidth="1"/>
-    <col min="14362" max="14362" width="12.140625" style="19" customWidth="1"/>
-    <col min="14363" max="14363" width="11.85546875" style="19" customWidth="1"/>
-    <col min="14364" max="14592" width="9.140625" style="19"/>
-    <col min="14593" max="14593" width="22" style="19" customWidth="1"/>
-    <col min="14594" max="14594" width="12.42578125" style="19" customWidth="1"/>
-    <col min="14595" max="14595" width="12.140625" style="19" customWidth="1"/>
-    <col min="14596" max="14596" width="12.28515625" style="19" customWidth="1"/>
-    <col min="14597" max="14597" width="10.5703125" style="19" customWidth="1"/>
-    <col min="14598" max="14598" width="11.5703125" style="19" customWidth="1"/>
-    <col min="14599" max="14599" width="10.85546875" style="19" customWidth="1"/>
-    <col min="14600" max="14600" width="11.140625" style="19" customWidth="1"/>
-    <col min="14601" max="14601" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="14602" max="14613" width="11.42578125" style="19" customWidth="1"/>
-    <col min="14614" max="14617" width="11.7109375" style="19" customWidth="1"/>
-    <col min="14618" max="14618" width="12.140625" style="19" customWidth="1"/>
-    <col min="14619" max="14619" width="11.85546875" style="19" customWidth="1"/>
-    <col min="14620" max="14848" width="9.140625" style="19"/>
-    <col min="14849" max="14849" width="22" style="19" customWidth="1"/>
-    <col min="14850" max="14850" width="12.42578125" style="19" customWidth="1"/>
-    <col min="14851" max="14851" width="12.140625" style="19" customWidth="1"/>
-    <col min="14852" max="14852" width="12.28515625" style="19" customWidth="1"/>
-    <col min="14853" max="14853" width="10.5703125" style="19" customWidth="1"/>
-    <col min="14854" max="14854" width="11.5703125" style="19" customWidth="1"/>
-    <col min="14855" max="14855" width="10.85546875" style="19" customWidth="1"/>
-    <col min="14856" max="14856" width="11.140625" style="19" customWidth="1"/>
-    <col min="14857" max="14857" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="14858" max="14869" width="11.42578125" style="19" customWidth="1"/>
-    <col min="14870" max="14873" width="11.7109375" style="19" customWidth="1"/>
-    <col min="14874" max="14874" width="12.140625" style="19" customWidth="1"/>
-    <col min="14875" max="14875" width="11.85546875" style="19" customWidth="1"/>
-    <col min="14876" max="15104" width="9.140625" style="19"/>
-    <col min="15105" max="15105" width="22" style="19" customWidth="1"/>
-    <col min="15106" max="15106" width="12.42578125" style="19" customWidth="1"/>
-    <col min="15107" max="15107" width="12.140625" style="19" customWidth="1"/>
-    <col min="15108" max="15108" width="12.28515625" style="19" customWidth="1"/>
-    <col min="15109" max="15109" width="10.5703125" style="19" customWidth="1"/>
-    <col min="15110" max="15110" width="11.5703125" style="19" customWidth="1"/>
-    <col min="15111" max="15111" width="10.85546875" style="19" customWidth="1"/>
-    <col min="15112" max="15112" width="11.140625" style="19" customWidth="1"/>
-    <col min="15113" max="15113" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="15114" max="15125" width="11.42578125" style="19" customWidth="1"/>
-    <col min="15126" max="15129" width="11.7109375" style="19" customWidth="1"/>
-    <col min="15130" max="15130" width="12.140625" style="19" customWidth="1"/>
-    <col min="15131" max="15131" width="11.85546875" style="19" customWidth="1"/>
-    <col min="15132" max="15360" width="9.140625" style="19"/>
-    <col min="15361" max="15361" width="22" style="19" customWidth="1"/>
-    <col min="15362" max="15362" width="12.42578125" style="19" customWidth="1"/>
-    <col min="15363" max="15363" width="12.140625" style="19" customWidth="1"/>
-    <col min="15364" max="15364" width="12.28515625" style="19" customWidth="1"/>
-    <col min="15365" max="15365" width="10.5703125" style="19" customWidth="1"/>
-    <col min="15366" max="15366" width="11.5703125" style="19" customWidth="1"/>
-    <col min="15367" max="15367" width="10.85546875" style="19" customWidth="1"/>
-    <col min="15368" max="15368" width="11.140625" style="19" customWidth="1"/>
-    <col min="15369" max="15369" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="15370" max="15381" width="11.42578125" style="19" customWidth="1"/>
-    <col min="15382" max="15385" width="11.7109375" style="19" customWidth="1"/>
-    <col min="15386" max="15386" width="12.140625" style="19" customWidth="1"/>
-    <col min="15387" max="15387" width="11.85546875" style="19" customWidth="1"/>
-    <col min="15388" max="15616" width="9.140625" style="19"/>
-    <col min="15617" max="15617" width="22" style="19" customWidth="1"/>
-    <col min="15618" max="15618" width="12.42578125" style="19" customWidth="1"/>
-    <col min="15619" max="15619" width="12.140625" style="19" customWidth="1"/>
-    <col min="15620" max="15620" width="12.28515625" style="19" customWidth="1"/>
-    <col min="15621" max="15621" width="10.5703125" style="19" customWidth="1"/>
-    <col min="15622" max="15622" width="11.5703125" style="19" customWidth="1"/>
-    <col min="15623" max="15623" width="10.85546875" style="19" customWidth="1"/>
-    <col min="15624" max="15624" width="11.140625" style="19" customWidth="1"/>
-    <col min="15625" max="15625" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="15626" max="15637" width="11.42578125" style="19" customWidth="1"/>
-    <col min="15638" max="15641" width="11.7109375" style="19" customWidth="1"/>
-    <col min="15642" max="15642" width="12.140625" style="19" customWidth="1"/>
-    <col min="15643" max="15643" width="11.85546875" style="19" customWidth="1"/>
-    <col min="15644" max="15872" width="9.140625" style="19"/>
-    <col min="15873" max="15873" width="22" style="19" customWidth="1"/>
-    <col min="15874" max="15874" width="12.42578125" style="19" customWidth="1"/>
-    <col min="15875" max="15875" width="12.140625" style="19" customWidth="1"/>
-    <col min="15876" max="15876" width="12.28515625" style="19" customWidth="1"/>
-    <col min="15877" max="15877" width="10.5703125" style="19" customWidth="1"/>
-    <col min="15878" max="15878" width="11.5703125" style="19" customWidth="1"/>
-    <col min="15879" max="15879" width="10.85546875" style="19" customWidth="1"/>
-    <col min="15880" max="15880" width="11.140625" style="19" customWidth="1"/>
-    <col min="15881" max="15881" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="15882" max="15893" width="11.42578125" style="19" customWidth="1"/>
-    <col min="15894" max="15897" width="11.7109375" style="19" customWidth="1"/>
-    <col min="15898" max="15898" width="12.140625" style="19" customWidth="1"/>
-    <col min="15899" max="15899" width="11.85546875" style="19" customWidth="1"/>
-    <col min="15900" max="16128" width="9.140625" style="19"/>
-    <col min="16129" max="16129" width="22" style="19" customWidth="1"/>
-    <col min="16130" max="16130" width="12.42578125" style="19" customWidth="1"/>
-    <col min="16131" max="16131" width="12.140625" style="19" customWidth="1"/>
-    <col min="16132" max="16132" width="12.28515625" style="19" customWidth="1"/>
-    <col min="16133" max="16133" width="10.5703125" style="19" customWidth="1"/>
-    <col min="16134" max="16134" width="11.5703125" style="19" customWidth="1"/>
-    <col min="16135" max="16135" width="10.85546875" style="19" customWidth="1"/>
-    <col min="16136" max="16136" width="11.140625" style="19" customWidth="1"/>
-    <col min="16137" max="16137" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="16138" max="16149" width="11.42578125" style="19" customWidth="1"/>
-    <col min="16150" max="16153" width="11.7109375" style="19" customWidth="1"/>
-    <col min="16154" max="16154" width="12.140625" style="19" customWidth="1"/>
-    <col min="16155" max="16155" width="11.85546875" style="19" customWidth="1"/>
-    <col min="16156" max="16384" width="9.140625" style="19"/>
+    <col min="1" max="1" width="22" style="18" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" style="18" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" style="18" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" style="18" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="18" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" style="18" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" style="18" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" style="18" customWidth="1"/>
+    <col min="9" max="9" width="11.5703125" style="18" bestFit="1" customWidth="1"/>
+    <col min="10" max="21" width="11.42578125" style="18" customWidth="1"/>
+    <col min="22" max="25" width="11.7109375" style="18" customWidth="1"/>
+    <col min="26" max="26" width="12.140625" style="18" customWidth="1"/>
+    <col min="27" max="27" width="11.85546875" style="18" customWidth="1"/>
+    <col min="28" max="256" width="9.140625" style="18"/>
+    <col min="257" max="257" width="22" style="18" customWidth="1"/>
+    <col min="258" max="258" width="12.42578125" style="18" customWidth="1"/>
+    <col min="259" max="259" width="12.140625" style="18" customWidth="1"/>
+    <col min="260" max="260" width="12.28515625" style="18" customWidth="1"/>
+    <col min="261" max="261" width="10.5703125" style="18" customWidth="1"/>
+    <col min="262" max="262" width="11.5703125" style="18" customWidth="1"/>
+    <col min="263" max="263" width="10.85546875" style="18" customWidth="1"/>
+    <col min="264" max="264" width="11.140625" style="18" customWidth="1"/>
+    <col min="265" max="265" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="266" max="277" width="11.42578125" style="18" customWidth="1"/>
+    <col min="278" max="281" width="11.7109375" style="18" customWidth="1"/>
+    <col min="282" max="282" width="12.140625" style="18" customWidth="1"/>
+    <col min="283" max="283" width="11.85546875" style="18" customWidth="1"/>
+    <col min="284" max="512" width="9.140625" style="18"/>
+    <col min="513" max="513" width="22" style="18" customWidth="1"/>
+    <col min="514" max="514" width="12.42578125" style="18" customWidth="1"/>
+    <col min="515" max="515" width="12.140625" style="18" customWidth="1"/>
+    <col min="516" max="516" width="12.28515625" style="18" customWidth="1"/>
+    <col min="517" max="517" width="10.5703125" style="18" customWidth="1"/>
+    <col min="518" max="518" width="11.5703125" style="18" customWidth="1"/>
+    <col min="519" max="519" width="10.85546875" style="18" customWidth="1"/>
+    <col min="520" max="520" width="11.140625" style="18" customWidth="1"/>
+    <col min="521" max="521" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="522" max="533" width="11.42578125" style="18" customWidth="1"/>
+    <col min="534" max="537" width="11.7109375" style="18" customWidth="1"/>
+    <col min="538" max="538" width="12.140625" style="18" customWidth="1"/>
+    <col min="539" max="539" width="11.85546875" style="18" customWidth="1"/>
+    <col min="540" max="768" width="9.140625" style="18"/>
+    <col min="769" max="769" width="22" style="18" customWidth="1"/>
+    <col min="770" max="770" width="12.42578125" style="18" customWidth="1"/>
+    <col min="771" max="771" width="12.140625" style="18" customWidth="1"/>
+    <col min="772" max="772" width="12.28515625" style="18" customWidth="1"/>
+    <col min="773" max="773" width="10.5703125" style="18" customWidth="1"/>
+    <col min="774" max="774" width="11.5703125" style="18" customWidth="1"/>
+    <col min="775" max="775" width="10.85546875" style="18" customWidth="1"/>
+    <col min="776" max="776" width="11.140625" style="18" customWidth="1"/>
+    <col min="777" max="777" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="778" max="789" width="11.42578125" style="18" customWidth="1"/>
+    <col min="790" max="793" width="11.7109375" style="18" customWidth="1"/>
+    <col min="794" max="794" width="12.140625" style="18" customWidth="1"/>
+    <col min="795" max="795" width="11.85546875" style="18" customWidth="1"/>
+    <col min="796" max="1024" width="9.140625" style="18"/>
+    <col min="1025" max="1025" width="22" style="18" customWidth="1"/>
+    <col min="1026" max="1026" width="12.42578125" style="18" customWidth="1"/>
+    <col min="1027" max="1027" width="12.140625" style="18" customWidth="1"/>
+    <col min="1028" max="1028" width="12.28515625" style="18" customWidth="1"/>
+    <col min="1029" max="1029" width="10.5703125" style="18" customWidth="1"/>
+    <col min="1030" max="1030" width="11.5703125" style="18" customWidth="1"/>
+    <col min="1031" max="1031" width="10.85546875" style="18" customWidth="1"/>
+    <col min="1032" max="1032" width="11.140625" style="18" customWidth="1"/>
+    <col min="1033" max="1033" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="1034" max="1045" width="11.42578125" style="18" customWidth="1"/>
+    <col min="1046" max="1049" width="11.7109375" style="18" customWidth="1"/>
+    <col min="1050" max="1050" width="12.140625" style="18" customWidth="1"/>
+    <col min="1051" max="1051" width="11.85546875" style="18" customWidth="1"/>
+    <col min="1052" max="1280" width="9.140625" style="18"/>
+    <col min="1281" max="1281" width="22" style="18" customWidth="1"/>
+    <col min="1282" max="1282" width="12.42578125" style="18" customWidth="1"/>
+    <col min="1283" max="1283" width="12.140625" style="18" customWidth="1"/>
+    <col min="1284" max="1284" width="12.28515625" style="18" customWidth="1"/>
+    <col min="1285" max="1285" width="10.5703125" style="18" customWidth="1"/>
+    <col min="1286" max="1286" width="11.5703125" style="18" customWidth="1"/>
+    <col min="1287" max="1287" width="10.85546875" style="18" customWidth="1"/>
+    <col min="1288" max="1288" width="11.140625" style="18" customWidth="1"/>
+    <col min="1289" max="1289" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="1290" max="1301" width="11.42578125" style="18" customWidth="1"/>
+    <col min="1302" max="1305" width="11.7109375" style="18" customWidth="1"/>
+    <col min="1306" max="1306" width="12.140625" style="18" customWidth="1"/>
+    <col min="1307" max="1307" width="11.85546875" style="18" customWidth="1"/>
+    <col min="1308" max="1536" width="9.140625" style="18"/>
+    <col min="1537" max="1537" width="22" style="18" customWidth="1"/>
+    <col min="1538" max="1538" width="12.42578125" style="18" customWidth="1"/>
+    <col min="1539" max="1539" width="12.140625" style="18" customWidth="1"/>
+    <col min="1540" max="1540" width="12.28515625" style="18" customWidth="1"/>
+    <col min="1541" max="1541" width="10.5703125" style="18" customWidth="1"/>
+    <col min="1542" max="1542" width="11.5703125" style="18" customWidth="1"/>
+    <col min="1543" max="1543" width="10.85546875" style="18" customWidth="1"/>
+    <col min="1544" max="1544" width="11.140625" style="18" customWidth="1"/>
+    <col min="1545" max="1545" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="1546" max="1557" width="11.42578125" style="18" customWidth="1"/>
+    <col min="1558" max="1561" width="11.7109375" style="18" customWidth="1"/>
+    <col min="1562" max="1562" width="12.140625" style="18" customWidth="1"/>
+    <col min="1563" max="1563" width="11.85546875" style="18" customWidth="1"/>
+    <col min="1564" max="1792" width="9.140625" style="18"/>
+    <col min="1793" max="1793" width="22" style="18" customWidth="1"/>
+    <col min="1794" max="1794" width="12.42578125" style="18" customWidth="1"/>
+    <col min="1795" max="1795" width="12.140625" style="18" customWidth="1"/>
+    <col min="1796" max="1796" width="12.28515625" style="18" customWidth="1"/>
+    <col min="1797" max="1797" width="10.5703125" style="18" customWidth="1"/>
+    <col min="1798" max="1798" width="11.5703125" style="18" customWidth="1"/>
+    <col min="1799" max="1799" width="10.85546875" style="18" customWidth="1"/>
+    <col min="1800" max="1800" width="11.140625" style="18" customWidth="1"/>
+    <col min="1801" max="1801" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="1802" max="1813" width="11.42578125" style="18" customWidth="1"/>
+    <col min="1814" max="1817" width="11.7109375" style="18" customWidth="1"/>
+    <col min="1818" max="1818" width="12.140625" style="18" customWidth="1"/>
+    <col min="1819" max="1819" width="11.85546875" style="18" customWidth="1"/>
+    <col min="1820" max="2048" width="9.140625" style="18"/>
+    <col min="2049" max="2049" width="22" style="18" customWidth="1"/>
+    <col min="2050" max="2050" width="12.42578125" style="18" customWidth="1"/>
+    <col min="2051" max="2051" width="12.140625" style="18" customWidth="1"/>
+    <col min="2052" max="2052" width="12.28515625" style="18" customWidth="1"/>
+    <col min="2053" max="2053" width="10.5703125" style="18" customWidth="1"/>
+    <col min="2054" max="2054" width="11.5703125" style="18" customWidth="1"/>
+    <col min="2055" max="2055" width="10.85546875" style="18" customWidth="1"/>
+    <col min="2056" max="2056" width="11.140625" style="18" customWidth="1"/>
+    <col min="2057" max="2057" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="2058" max="2069" width="11.42578125" style="18" customWidth="1"/>
+    <col min="2070" max="2073" width="11.7109375" style="18" customWidth="1"/>
+    <col min="2074" max="2074" width="12.140625" style="18" customWidth="1"/>
+    <col min="2075" max="2075" width="11.85546875" style="18" customWidth="1"/>
+    <col min="2076" max="2304" width="9.140625" style="18"/>
+    <col min="2305" max="2305" width="22" style="18" customWidth="1"/>
+    <col min="2306" max="2306" width="12.42578125" style="18" customWidth="1"/>
+    <col min="2307" max="2307" width="12.140625" style="18" customWidth="1"/>
+    <col min="2308" max="2308" width="12.28515625" style="18" customWidth="1"/>
+    <col min="2309" max="2309" width="10.5703125" style="18" customWidth="1"/>
+    <col min="2310" max="2310" width="11.5703125" style="18" customWidth="1"/>
+    <col min="2311" max="2311" width="10.85546875" style="18" customWidth="1"/>
+    <col min="2312" max="2312" width="11.140625" style="18" customWidth="1"/>
+    <col min="2313" max="2313" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="2314" max="2325" width="11.42578125" style="18" customWidth="1"/>
+    <col min="2326" max="2329" width="11.7109375" style="18" customWidth="1"/>
+    <col min="2330" max="2330" width="12.140625" style="18" customWidth="1"/>
+    <col min="2331" max="2331" width="11.85546875" style="18" customWidth="1"/>
+    <col min="2332" max="2560" width="9.140625" style="18"/>
+    <col min="2561" max="2561" width="22" style="18" customWidth="1"/>
+    <col min="2562" max="2562" width="12.42578125" style="18" customWidth="1"/>
+    <col min="2563" max="2563" width="12.140625" style="18" customWidth="1"/>
+    <col min="2564" max="2564" width="12.28515625" style="18" customWidth="1"/>
+    <col min="2565" max="2565" width="10.5703125" style="18" customWidth="1"/>
+    <col min="2566" max="2566" width="11.5703125" style="18" customWidth="1"/>
+    <col min="2567" max="2567" width="10.85546875" style="18" customWidth="1"/>
+    <col min="2568" max="2568" width="11.140625" style="18" customWidth="1"/>
+    <col min="2569" max="2569" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="2570" max="2581" width="11.42578125" style="18" customWidth="1"/>
+    <col min="2582" max="2585" width="11.7109375" style="18" customWidth="1"/>
+    <col min="2586" max="2586" width="12.140625" style="18" customWidth="1"/>
+    <col min="2587" max="2587" width="11.85546875" style="18" customWidth="1"/>
+    <col min="2588" max="2816" width="9.140625" style="18"/>
+    <col min="2817" max="2817" width="22" style="18" customWidth="1"/>
+    <col min="2818" max="2818" width="12.42578125" style="18" customWidth="1"/>
+    <col min="2819" max="2819" width="12.140625" style="18" customWidth="1"/>
+    <col min="2820" max="2820" width="12.28515625" style="18" customWidth="1"/>
+    <col min="2821" max="2821" width="10.5703125" style="18" customWidth="1"/>
+    <col min="2822" max="2822" width="11.5703125" style="18" customWidth="1"/>
+    <col min="2823" max="2823" width="10.85546875" style="18" customWidth="1"/>
+    <col min="2824" max="2824" width="11.140625" style="18" customWidth="1"/>
+    <col min="2825" max="2825" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="2826" max="2837" width="11.42578125" style="18" customWidth="1"/>
+    <col min="2838" max="2841" width="11.7109375" style="18" customWidth="1"/>
+    <col min="2842" max="2842" width="12.140625" style="18" customWidth="1"/>
+    <col min="2843" max="2843" width="11.85546875" style="18" customWidth="1"/>
+    <col min="2844" max="3072" width="9.140625" style="18"/>
+    <col min="3073" max="3073" width="22" style="18" customWidth="1"/>
+    <col min="3074" max="3074" width="12.42578125" style="18" customWidth="1"/>
+    <col min="3075" max="3075" width="12.140625" style="18" customWidth="1"/>
+    <col min="3076" max="3076" width="12.28515625" style="18" customWidth="1"/>
+    <col min="3077" max="3077" width="10.5703125" style="18" customWidth="1"/>
+    <col min="3078" max="3078" width="11.5703125" style="18" customWidth="1"/>
+    <col min="3079" max="3079" width="10.85546875" style="18" customWidth="1"/>
+    <col min="3080" max="3080" width="11.140625" style="18" customWidth="1"/>
+    <col min="3081" max="3081" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="3082" max="3093" width="11.42578125" style="18" customWidth="1"/>
+    <col min="3094" max="3097" width="11.7109375" style="18" customWidth="1"/>
+    <col min="3098" max="3098" width="12.140625" style="18" customWidth="1"/>
+    <col min="3099" max="3099" width="11.85546875" style="18" customWidth="1"/>
+    <col min="3100" max="3328" width="9.140625" style="18"/>
+    <col min="3329" max="3329" width="22" style="18" customWidth="1"/>
+    <col min="3330" max="3330" width="12.42578125" style="18" customWidth="1"/>
+    <col min="3331" max="3331" width="12.140625" style="18" customWidth="1"/>
+    <col min="3332" max="3332" width="12.28515625" style="18" customWidth="1"/>
+    <col min="3333" max="3333" width="10.5703125" style="18" customWidth="1"/>
+    <col min="3334" max="3334" width="11.5703125" style="18" customWidth="1"/>
+    <col min="3335" max="3335" width="10.85546875" style="18" customWidth="1"/>
+    <col min="3336" max="3336" width="11.140625" style="18" customWidth="1"/>
+    <col min="3337" max="3337" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="3338" max="3349" width="11.42578125" style="18" customWidth="1"/>
+    <col min="3350" max="3353" width="11.7109375" style="18" customWidth="1"/>
+    <col min="3354" max="3354" width="12.140625" style="18" customWidth="1"/>
+    <col min="3355" max="3355" width="11.85546875" style="18" customWidth="1"/>
+    <col min="3356" max="3584" width="9.140625" style="18"/>
+    <col min="3585" max="3585" width="22" style="18" customWidth="1"/>
+    <col min="3586" max="3586" width="12.42578125" style="18" customWidth="1"/>
+    <col min="3587" max="3587" width="12.140625" style="18" customWidth="1"/>
+    <col min="3588" max="3588" width="12.28515625" style="18" customWidth="1"/>
+    <col min="3589" max="3589" width="10.5703125" style="18" customWidth="1"/>
+    <col min="3590" max="3590" width="11.5703125" style="18" customWidth="1"/>
+    <col min="3591" max="3591" width="10.85546875" style="18" customWidth="1"/>
+    <col min="3592" max="3592" width="11.140625" style="18" customWidth="1"/>
+    <col min="3593" max="3593" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="3594" max="3605" width="11.42578125" style="18" customWidth="1"/>
+    <col min="3606" max="3609" width="11.7109375" style="18" customWidth="1"/>
+    <col min="3610" max="3610" width="12.140625" style="18" customWidth="1"/>
+    <col min="3611" max="3611" width="11.85546875" style="18" customWidth="1"/>
+    <col min="3612" max="3840" width="9.140625" style="18"/>
+    <col min="3841" max="3841" width="22" style="18" customWidth="1"/>
+    <col min="3842" max="3842" width="12.42578125" style="18" customWidth="1"/>
+    <col min="3843" max="3843" width="12.140625" style="18" customWidth="1"/>
+    <col min="3844" max="3844" width="12.28515625" style="18" customWidth="1"/>
+    <col min="3845" max="3845" width="10.5703125" style="18" customWidth="1"/>
+    <col min="3846" max="3846" width="11.5703125" style="18" customWidth="1"/>
+    <col min="3847" max="3847" width="10.85546875" style="18" customWidth="1"/>
+    <col min="3848" max="3848" width="11.140625" style="18" customWidth="1"/>
+    <col min="3849" max="3849" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="3850" max="3861" width="11.42578125" style="18" customWidth="1"/>
+    <col min="3862" max="3865" width="11.7109375" style="18" customWidth="1"/>
+    <col min="3866" max="3866" width="12.140625" style="18" customWidth="1"/>
+    <col min="3867" max="3867" width="11.85546875" style="18" customWidth="1"/>
+    <col min="3868" max="4096" width="9.140625" style="18"/>
+    <col min="4097" max="4097" width="22" style="18" customWidth="1"/>
+    <col min="4098" max="4098" width="12.42578125" style="18" customWidth="1"/>
+    <col min="4099" max="4099" width="12.140625" style="18" customWidth="1"/>
+    <col min="4100" max="4100" width="12.28515625" style="18" customWidth="1"/>
+    <col min="4101" max="4101" width="10.5703125" style="18" customWidth="1"/>
+    <col min="4102" max="4102" width="11.5703125" style="18" customWidth="1"/>
+    <col min="4103" max="4103" width="10.85546875" style="18" customWidth="1"/>
+    <col min="4104" max="4104" width="11.140625" style="18" customWidth="1"/>
+    <col min="4105" max="4105" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="4106" max="4117" width="11.42578125" style="18" customWidth="1"/>
+    <col min="4118" max="4121" width="11.7109375" style="18" customWidth="1"/>
+    <col min="4122" max="4122" width="12.140625" style="18" customWidth="1"/>
+    <col min="4123" max="4123" width="11.85546875" style="18" customWidth="1"/>
+    <col min="4124" max="4352" width="9.140625" style="18"/>
+    <col min="4353" max="4353" width="22" style="18" customWidth="1"/>
+    <col min="4354" max="4354" width="12.42578125" style="18" customWidth="1"/>
+    <col min="4355" max="4355" width="12.140625" style="18" customWidth="1"/>
+    <col min="4356" max="4356" width="12.28515625" style="18" customWidth="1"/>
+    <col min="4357" max="4357" width="10.5703125" style="18" customWidth="1"/>
+    <col min="4358" max="4358" width="11.5703125" style="18" customWidth="1"/>
+    <col min="4359" max="4359" width="10.85546875" style="18" customWidth="1"/>
+    <col min="4360" max="4360" width="11.140625" style="18" customWidth="1"/>
+    <col min="4361" max="4361" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="4362" max="4373" width="11.42578125" style="18" customWidth="1"/>
+    <col min="4374" max="4377" width="11.7109375" style="18" customWidth="1"/>
+    <col min="4378" max="4378" width="12.140625" style="18" customWidth="1"/>
+    <col min="4379" max="4379" width="11.85546875" style="18" customWidth="1"/>
+    <col min="4380" max="4608" width="9.140625" style="18"/>
+    <col min="4609" max="4609" width="22" style="18" customWidth="1"/>
+    <col min="4610" max="4610" width="12.42578125" style="18" customWidth="1"/>
+    <col min="4611" max="4611" width="12.140625" style="18" customWidth="1"/>
+    <col min="4612" max="4612" width="12.28515625" style="18" customWidth="1"/>
+    <col min="4613" max="4613" width="10.5703125" style="18" customWidth="1"/>
+    <col min="4614" max="4614" width="11.5703125" style="18" customWidth="1"/>
+    <col min="4615" max="4615" width="10.85546875" style="18" customWidth="1"/>
+    <col min="4616" max="4616" width="11.140625" style="18" customWidth="1"/>
+    <col min="4617" max="4617" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="4618" max="4629" width="11.42578125" style="18" customWidth="1"/>
+    <col min="4630" max="4633" width="11.7109375" style="18" customWidth="1"/>
+    <col min="4634" max="4634" width="12.140625" style="18" customWidth="1"/>
+    <col min="4635" max="4635" width="11.85546875" style="18" customWidth="1"/>
+    <col min="4636" max="4864" width="9.140625" style="18"/>
+    <col min="4865" max="4865" width="22" style="18" customWidth="1"/>
+    <col min="4866" max="4866" width="12.42578125" style="18" customWidth="1"/>
+    <col min="4867" max="4867" width="12.140625" style="18" customWidth="1"/>
+    <col min="4868" max="4868" width="12.28515625" style="18" customWidth="1"/>
+    <col min="4869" max="4869" width="10.5703125" style="18" customWidth="1"/>
+    <col min="4870" max="4870" width="11.5703125" style="18" customWidth="1"/>
+    <col min="4871" max="4871" width="10.85546875" style="18" customWidth="1"/>
+    <col min="4872" max="4872" width="11.140625" style="18" customWidth="1"/>
+    <col min="4873" max="4873" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="4874" max="4885" width="11.42578125" style="18" customWidth="1"/>
+    <col min="4886" max="4889" width="11.7109375" style="18" customWidth="1"/>
+    <col min="4890" max="4890" width="12.140625" style="18" customWidth="1"/>
+    <col min="4891" max="4891" width="11.85546875" style="18" customWidth="1"/>
+    <col min="4892" max="5120" width="9.140625" style="18"/>
+    <col min="5121" max="5121" width="22" style="18" customWidth="1"/>
+    <col min="5122" max="5122" width="12.42578125" style="18" customWidth="1"/>
+    <col min="5123" max="5123" width="12.140625" style="18" customWidth="1"/>
+    <col min="5124" max="5124" width="12.28515625" style="18" customWidth="1"/>
+    <col min="5125" max="5125" width="10.5703125" style="18" customWidth="1"/>
+    <col min="5126" max="5126" width="11.5703125" style="18" customWidth="1"/>
+    <col min="5127" max="5127" width="10.85546875" style="18" customWidth="1"/>
+    <col min="5128" max="5128" width="11.140625" style="18" customWidth="1"/>
+    <col min="5129" max="5129" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="5130" max="5141" width="11.42578125" style="18" customWidth="1"/>
+    <col min="5142" max="5145" width="11.7109375" style="18" customWidth="1"/>
+    <col min="5146" max="5146" width="12.140625" style="18" customWidth="1"/>
+    <col min="5147" max="5147" width="11.85546875" style="18" customWidth="1"/>
+    <col min="5148" max="5376" width="9.140625" style="18"/>
+    <col min="5377" max="5377" width="22" style="18" customWidth="1"/>
+    <col min="5378" max="5378" width="12.42578125" style="18" customWidth="1"/>
+    <col min="5379" max="5379" width="12.140625" style="18" customWidth="1"/>
+    <col min="5380" max="5380" width="12.28515625" style="18" customWidth="1"/>
+    <col min="5381" max="5381" width="10.5703125" style="18" customWidth="1"/>
+    <col min="5382" max="5382" width="11.5703125" style="18" customWidth="1"/>
+    <col min="5383" max="5383" width="10.85546875" style="18" customWidth="1"/>
+    <col min="5384" max="5384" width="11.140625" style="18" customWidth="1"/>
+    <col min="5385" max="5385" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="5386" max="5397" width="11.42578125" style="18" customWidth="1"/>
+    <col min="5398" max="5401" width="11.7109375" style="18" customWidth="1"/>
+    <col min="5402" max="5402" width="12.140625" style="18" customWidth="1"/>
+    <col min="5403" max="5403" width="11.85546875" style="18" customWidth="1"/>
+    <col min="5404" max="5632" width="9.140625" style="18"/>
+    <col min="5633" max="5633" width="22" style="18" customWidth="1"/>
+    <col min="5634" max="5634" width="12.42578125" style="18" customWidth="1"/>
+    <col min="5635" max="5635" width="12.140625" style="18" customWidth="1"/>
+    <col min="5636" max="5636" width="12.28515625" style="18" customWidth="1"/>
+    <col min="5637" max="5637" width="10.5703125" style="18" customWidth="1"/>
+    <col min="5638" max="5638" width="11.5703125" style="18" customWidth="1"/>
+    <col min="5639" max="5639" width="10.85546875" style="18" customWidth="1"/>
+    <col min="5640" max="5640" width="11.140625" style="18" customWidth="1"/>
+    <col min="5641" max="5641" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="5642" max="5653" width="11.42578125" style="18" customWidth="1"/>
+    <col min="5654" max="5657" width="11.7109375" style="18" customWidth="1"/>
+    <col min="5658" max="5658" width="12.140625" style="18" customWidth="1"/>
+    <col min="5659" max="5659" width="11.85546875" style="18" customWidth="1"/>
+    <col min="5660" max="5888" width="9.140625" style="18"/>
+    <col min="5889" max="5889" width="22" style="18" customWidth="1"/>
+    <col min="5890" max="5890" width="12.42578125" style="18" customWidth="1"/>
+    <col min="5891" max="5891" width="12.140625" style="18" customWidth="1"/>
+    <col min="5892" max="5892" width="12.28515625" style="18" customWidth="1"/>
+    <col min="5893" max="5893" width="10.5703125" style="18" customWidth="1"/>
+    <col min="5894" max="5894" width="11.5703125" style="18" customWidth="1"/>
+    <col min="5895" max="5895" width="10.85546875" style="18" customWidth="1"/>
+    <col min="5896" max="5896" width="11.140625" style="18" customWidth="1"/>
+    <col min="5897" max="5897" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="5898" max="5909" width="11.42578125" style="18" customWidth="1"/>
+    <col min="5910" max="5913" width="11.7109375" style="18" customWidth="1"/>
+    <col min="5914" max="5914" width="12.140625" style="18" customWidth="1"/>
+    <col min="5915" max="5915" width="11.85546875" style="18" customWidth="1"/>
+    <col min="5916" max="6144" width="9.140625" style="18"/>
+    <col min="6145" max="6145" width="22" style="18" customWidth="1"/>
+    <col min="6146" max="6146" width="12.42578125" style="18" customWidth="1"/>
+    <col min="6147" max="6147" width="12.140625" style="18" customWidth="1"/>
+    <col min="6148" max="6148" width="12.28515625" style="18" customWidth="1"/>
+    <col min="6149" max="6149" width="10.5703125" style="18" customWidth="1"/>
+    <col min="6150" max="6150" width="11.5703125" style="18" customWidth="1"/>
+    <col min="6151" max="6151" width="10.85546875" style="18" customWidth="1"/>
+    <col min="6152" max="6152" width="11.140625" style="18" customWidth="1"/>
+    <col min="6153" max="6153" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="6154" max="6165" width="11.42578125" style="18" customWidth="1"/>
+    <col min="6166" max="6169" width="11.7109375" style="18" customWidth="1"/>
+    <col min="6170" max="6170" width="12.140625" style="18" customWidth="1"/>
+    <col min="6171" max="6171" width="11.85546875" style="18" customWidth="1"/>
+    <col min="6172" max="6400" width="9.140625" style="18"/>
+    <col min="6401" max="6401" width="22" style="18" customWidth="1"/>
+    <col min="6402" max="6402" width="12.42578125" style="18" customWidth="1"/>
+    <col min="6403" max="6403" width="12.140625" style="18" customWidth="1"/>
+    <col min="6404" max="6404" width="12.28515625" style="18" customWidth="1"/>
+    <col min="6405" max="6405" width="10.5703125" style="18" customWidth="1"/>
+    <col min="6406" max="6406" width="11.5703125" style="18" customWidth="1"/>
+    <col min="6407" max="6407" width="10.85546875" style="18" customWidth="1"/>
+    <col min="6408" max="6408" width="11.140625" style="18" customWidth="1"/>
+    <col min="6409" max="6409" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="6410" max="6421" width="11.42578125" style="18" customWidth="1"/>
+    <col min="6422" max="6425" width="11.7109375" style="18" customWidth="1"/>
+    <col min="6426" max="6426" width="12.140625" style="18" customWidth="1"/>
+    <col min="6427" max="6427" width="11.85546875" style="18" customWidth="1"/>
+    <col min="6428" max="6656" width="9.140625" style="18"/>
+    <col min="6657" max="6657" width="22" style="18" customWidth="1"/>
+    <col min="6658" max="6658" width="12.42578125" style="18" customWidth="1"/>
+    <col min="6659" max="6659" width="12.140625" style="18" customWidth="1"/>
+    <col min="6660" max="6660" width="12.28515625" style="18" customWidth="1"/>
+    <col min="6661" max="6661" width="10.5703125" style="18" customWidth="1"/>
+    <col min="6662" max="6662" width="11.5703125" style="18" customWidth="1"/>
+    <col min="6663" max="6663" width="10.85546875" style="18" customWidth="1"/>
+    <col min="6664" max="6664" width="11.140625" style="18" customWidth="1"/>
+    <col min="6665" max="6665" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="6666" max="6677" width="11.42578125" style="18" customWidth="1"/>
+    <col min="6678" max="6681" width="11.7109375" style="18" customWidth="1"/>
+    <col min="6682" max="6682" width="12.140625" style="18" customWidth="1"/>
+    <col min="6683" max="6683" width="11.85546875" style="18" customWidth="1"/>
+    <col min="6684" max="6912" width="9.140625" style="18"/>
+    <col min="6913" max="6913" width="22" style="18" customWidth="1"/>
+    <col min="6914" max="6914" width="12.42578125" style="18" customWidth="1"/>
+    <col min="6915" max="6915" width="12.140625" style="18" customWidth="1"/>
+    <col min="6916" max="6916" width="12.28515625" style="18" customWidth="1"/>
+    <col min="6917" max="6917" width="10.5703125" style="18" customWidth="1"/>
+    <col min="6918" max="6918" width="11.5703125" style="18" customWidth="1"/>
+    <col min="6919" max="6919" width="10.85546875" style="18" customWidth="1"/>
+    <col min="6920" max="6920" width="11.140625" style="18" customWidth="1"/>
+    <col min="6921" max="6921" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="6922" max="6933" width="11.42578125" style="18" customWidth="1"/>
+    <col min="6934" max="6937" width="11.7109375" style="18" customWidth="1"/>
+    <col min="6938" max="6938" width="12.140625" style="18" customWidth="1"/>
+    <col min="6939" max="6939" width="11.85546875" style="18" customWidth="1"/>
+    <col min="6940" max="7168" width="9.140625" style="18"/>
+    <col min="7169" max="7169" width="22" style="18" customWidth="1"/>
+    <col min="7170" max="7170" width="12.42578125" style="18" customWidth="1"/>
+    <col min="7171" max="7171" width="12.140625" style="18" customWidth="1"/>
+    <col min="7172" max="7172" width="12.28515625" style="18" customWidth="1"/>
+    <col min="7173" max="7173" width="10.5703125" style="18" customWidth="1"/>
+    <col min="7174" max="7174" width="11.5703125" style="18" customWidth="1"/>
+    <col min="7175" max="7175" width="10.85546875" style="18" customWidth="1"/>
+    <col min="7176" max="7176" width="11.140625" style="18" customWidth="1"/>
+    <col min="7177" max="7177" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="7178" max="7189" width="11.42578125" style="18" customWidth="1"/>
+    <col min="7190" max="7193" width="11.7109375" style="18" customWidth="1"/>
+    <col min="7194" max="7194" width="12.140625" style="18" customWidth="1"/>
+    <col min="7195" max="7195" width="11.85546875" style="18" customWidth="1"/>
+    <col min="7196" max="7424" width="9.140625" style="18"/>
+    <col min="7425" max="7425" width="22" style="18" customWidth="1"/>
+    <col min="7426" max="7426" width="12.42578125" style="18" customWidth="1"/>
+    <col min="7427" max="7427" width="12.140625" style="18" customWidth="1"/>
+    <col min="7428" max="7428" width="12.28515625" style="18" customWidth="1"/>
+    <col min="7429" max="7429" width="10.5703125" style="18" customWidth="1"/>
+    <col min="7430" max="7430" width="11.5703125" style="18" customWidth="1"/>
+    <col min="7431" max="7431" width="10.85546875" style="18" customWidth="1"/>
+    <col min="7432" max="7432" width="11.140625" style="18" customWidth="1"/>
+    <col min="7433" max="7433" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="7434" max="7445" width="11.42578125" style="18" customWidth="1"/>
+    <col min="7446" max="7449" width="11.7109375" style="18" customWidth="1"/>
+    <col min="7450" max="7450" width="12.140625" style="18" customWidth="1"/>
+    <col min="7451" max="7451" width="11.85546875" style="18" customWidth="1"/>
+    <col min="7452" max="7680" width="9.140625" style="18"/>
+    <col min="7681" max="7681" width="22" style="18" customWidth="1"/>
+    <col min="7682" max="7682" width="12.42578125" style="18" customWidth="1"/>
+    <col min="7683" max="7683" width="12.140625" style="18" customWidth="1"/>
+    <col min="7684" max="7684" width="12.28515625" style="18" customWidth="1"/>
+    <col min="7685" max="7685" width="10.5703125" style="18" customWidth="1"/>
+    <col min="7686" max="7686" width="11.5703125" style="18" customWidth="1"/>
+    <col min="7687" max="7687" width="10.85546875" style="18" customWidth="1"/>
+    <col min="7688" max="7688" width="11.140625" style="18" customWidth="1"/>
+    <col min="7689" max="7689" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="7690" max="7701" width="11.42578125" style="18" customWidth="1"/>
+    <col min="7702" max="7705" width="11.7109375" style="18" customWidth="1"/>
+    <col min="7706" max="7706" width="12.140625" style="18" customWidth="1"/>
+    <col min="7707" max="7707" width="11.85546875" style="18" customWidth="1"/>
+    <col min="7708" max="7936" width="9.140625" style="18"/>
+    <col min="7937" max="7937" width="22" style="18" customWidth="1"/>
+    <col min="7938" max="7938" width="12.42578125" style="18" customWidth="1"/>
+    <col min="7939" max="7939" width="12.140625" style="18" customWidth="1"/>
+    <col min="7940" max="7940" width="12.28515625" style="18" customWidth="1"/>
+    <col min="7941" max="7941" width="10.5703125" style="18" customWidth="1"/>
+    <col min="7942" max="7942" width="11.5703125" style="18" customWidth="1"/>
+    <col min="7943" max="7943" width="10.85546875" style="18" customWidth="1"/>
+    <col min="7944" max="7944" width="11.140625" style="18" customWidth="1"/>
+    <col min="7945" max="7945" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="7946" max="7957" width="11.42578125" style="18" customWidth="1"/>
+    <col min="7958" max="7961" width="11.7109375" style="18" customWidth="1"/>
+    <col min="7962" max="7962" width="12.140625" style="18" customWidth="1"/>
+    <col min="7963" max="7963" width="11.85546875" style="18" customWidth="1"/>
+    <col min="7964" max="8192" width="9.140625" style="18"/>
+    <col min="8193" max="8193" width="22" style="18" customWidth="1"/>
+    <col min="8194" max="8194" width="12.42578125" style="18" customWidth="1"/>
+    <col min="8195" max="8195" width="12.140625" style="18" customWidth="1"/>
+    <col min="8196" max="8196" width="12.28515625" style="18" customWidth="1"/>
+    <col min="8197" max="8197" width="10.5703125" style="18" customWidth="1"/>
+    <col min="8198" max="8198" width="11.5703125" style="18" customWidth="1"/>
+    <col min="8199" max="8199" width="10.85546875" style="18" customWidth="1"/>
+    <col min="8200" max="8200" width="11.140625" style="18" customWidth="1"/>
+    <col min="8201" max="8201" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="8202" max="8213" width="11.42578125" style="18" customWidth="1"/>
+    <col min="8214" max="8217" width="11.7109375" style="18" customWidth="1"/>
+    <col min="8218" max="8218" width="12.140625" style="18" customWidth="1"/>
+    <col min="8219" max="8219" width="11.85546875" style="18" customWidth="1"/>
+    <col min="8220" max="8448" width="9.140625" style="18"/>
+    <col min="8449" max="8449" width="22" style="18" customWidth="1"/>
+    <col min="8450" max="8450" width="12.42578125" style="18" customWidth="1"/>
+    <col min="8451" max="8451" width="12.140625" style="18" customWidth="1"/>
+    <col min="8452" max="8452" width="12.28515625" style="18" customWidth="1"/>
+    <col min="8453" max="8453" width="10.5703125" style="18" customWidth="1"/>
+    <col min="8454" max="8454" width="11.5703125" style="18" customWidth="1"/>
+    <col min="8455" max="8455" width="10.85546875" style="18" customWidth="1"/>
+    <col min="8456" max="8456" width="11.140625" style="18" customWidth="1"/>
+    <col min="8457" max="8457" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="8458" max="8469" width="11.42578125" style="18" customWidth="1"/>
+    <col min="8470" max="8473" width="11.7109375" style="18" customWidth="1"/>
+    <col min="8474" max="8474" width="12.140625" style="18" customWidth="1"/>
+    <col min="8475" max="8475" width="11.85546875" style="18" customWidth="1"/>
+    <col min="8476" max="8704" width="9.140625" style="18"/>
+    <col min="8705" max="8705" width="22" style="18" customWidth="1"/>
+    <col min="8706" max="8706" width="12.42578125" style="18" customWidth="1"/>
+    <col min="8707" max="8707" width="12.140625" style="18" customWidth="1"/>
+    <col min="8708" max="8708" width="12.28515625" style="18" customWidth="1"/>
+    <col min="8709" max="8709" width="10.5703125" style="18" customWidth="1"/>
+    <col min="8710" max="8710" width="11.5703125" style="18" customWidth="1"/>
+    <col min="8711" max="8711" width="10.85546875" style="18" customWidth="1"/>
+    <col min="8712" max="8712" width="11.140625" style="18" customWidth="1"/>
+    <col min="8713" max="8713" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="8714" max="8725" width="11.42578125" style="18" customWidth="1"/>
+    <col min="8726" max="8729" width="11.7109375" style="18" customWidth="1"/>
+    <col min="8730" max="8730" width="12.140625" style="18" customWidth="1"/>
+    <col min="8731" max="8731" width="11.85546875" style="18" customWidth="1"/>
+    <col min="8732" max="8960" width="9.140625" style="18"/>
+    <col min="8961" max="8961" width="22" style="18" customWidth="1"/>
+    <col min="8962" max="8962" width="12.42578125" style="18" customWidth="1"/>
+    <col min="8963" max="8963" width="12.140625" style="18" customWidth="1"/>
+    <col min="8964" max="8964" width="12.28515625" style="18" customWidth="1"/>
+    <col min="8965" max="8965" width="10.5703125" style="18" customWidth="1"/>
+    <col min="8966" max="8966" width="11.5703125" style="18" customWidth="1"/>
+    <col min="8967" max="8967" width="10.85546875" style="18" customWidth="1"/>
+    <col min="8968" max="8968" width="11.140625" style="18" customWidth="1"/>
+    <col min="8969" max="8969" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="8970" max="8981" width="11.42578125" style="18" customWidth="1"/>
+    <col min="8982" max="8985" width="11.7109375" style="18" customWidth="1"/>
+    <col min="8986" max="8986" width="12.140625" style="18" customWidth="1"/>
+    <col min="8987" max="8987" width="11.85546875" style="18" customWidth="1"/>
+    <col min="8988" max="9216" width="9.140625" style="18"/>
+    <col min="9217" max="9217" width="22" style="18" customWidth="1"/>
+    <col min="9218" max="9218" width="12.42578125" style="18" customWidth="1"/>
+    <col min="9219" max="9219" width="12.140625" style="18" customWidth="1"/>
+    <col min="9220" max="9220" width="12.28515625" style="18" customWidth="1"/>
+    <col min="9221" max="9221" width="10.5703125" style="18" customWidth="1"/>
+    <col min="9222" max="9222" width="11.5703125" style="18" customWidth="1"/>
+    <col min="9223" max="9223" width="10.85546875" style="18" customWidth="1"/>
+    <col min="9224" max="9224" width="11.140625" style="18" customWidth="1"/>
+    <col min="9225" max="9225" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="9226" max="9237" width="11.42578125" style="18" customWidth="1"/>
+    <col min="9238" max="9241" width="11.7109375" style="18" customWidth="1"/>
+    <col min="9242" max="9242" width="12.140625" style="18" customWidth="1"/>
+    <col min="9243" max="9243" width="11.85546875" style="18" customWidth="1"/>
+    <col min="9244" max="9472" width="9.140625" style="18"/>
+    <col min="9473" max="9473" width="22" style="18" customWidth="1"/>
+    <col min="9474" max="9474" width="12.42578125" style="18" customWidth="1"/>
+    <col min="9475" max="9475" width="12.140625" style="18" customWidth="1"/>
+    <col min="9476" max="9476" width="12.28515625" style="18" customWidth="1"/>
+    <col min="9477" max="9477" width="10.5703125" style="18" customWidth="1"/>
+    <col min="9478" max="9478" width="11.5703125" style="18" customWidth="1"/>
+    <col min="9479" max="9479" width="10.85546875" style="18" customWidth="1"/>
+    <col min="9480" max="9480" width="11.140625" style="18" customWidth="1"/>
+    <col min="9481" max="9481" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="9482" max="9493" width="11.42578125" style="18" customWidth="1"/>
+    <col min="9494" max="9497" width="11.7109375" style="18" customWidth="1"/>
+    <col min="9498" max="9498" width="12.140625" style="18" customWidth="1"/>
+    <col min="9499" max="9499" width="11.85546875" style="18" customWidth="1"/>
+    <col min="9500" max="9728" width="9.140625" style="18"/>
+    <col min="9729" max="9729" width="22" style="18" customWidth="1"/>
+    <col min="9730" max="9730" width="12.42578125" style="18" customWidth="1"/>
+    <col min="9731" max="9731" width="12.140625" style="18" customWidth="1"/>
+    <col min="9732" max="9732" width="12.28515625" style="18" customWidth="1"/>
+    <col min="9733" max="9733" width="10.5703125" style="18" customWidth="1"/>
+    <col min="9734" max="9734" width="11.5703125" style="18" customWidth="1"/>
+    <col min="9735" max="9735" width="10.85546875" style="18" customWidth="1"/>
+    <col min="9736" max="9736" width="11.140625" style="18" customWidth="1"/>
+    <col min="9737" max="9737" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="9738" max="9749" width="11.42578125" style="18" customWidth="1"/>
+    <col min="9750" max="9753" width="11.7109375" style="18" customWidth="1"/>
+    <col min="9754" max="9754" width="12.140625" style="18" customWidth="1"/>
+    <col min="9755" max="9755" width="11.85546875" style="18" customWidth="1"/>
+    <col min="9756" max="9984" width="9.140625" style="18"/>
+    <col min="9985" max="9985" width="22" style="18" customWidth="1"/>
+    <col min="9986" max="9986" width="12.42578125" style="18" customWidth="1"/>
+    <col min="9987" max="9987" width="12.140625" style="18" customWidth="1"/>
+    <col min="9988" max="9988" width="12.28515625" style="18" customWidth="1"/>
+    <col min="9989" max="9989" width="10.5703125" style="18" customWidth="1"/>
+    <col min="9990" max="9990" width="11.5703125" style="18" customWidth="1"/>
+    <col min="9991" max="9991" width="10.85546875" style="18" customWidth="1"/>
+    <col min="9992" max="9992" width="11.140625" style="18" customWidth="1"/>
+    <col min="9993" max="9993" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="9994" max="10005" width="11.42578125" style="18" customWidth="1"/>
+    <col min="10006" max="10009" width="11.7109375" style="18" customWidth="1"/>
+    <col min="10010" max="10010" width="12.140625" style="18" customWidth="1"/>
+    <col min="10011" max="10011" width="11.85546875" style="18" customWidth="1"/>
+    <col min="10012" max="10240" width="9.140625" style="18"/>
+    <col min="10241" max="10241" width="22" style="18" customWidth="1"/>
+    <col min="10242" max="10242" width="12.42578125" style="18" customWidth="1"/>
+    <col min="10243" max="10243" width="12.140625" style="18" customWidth="1"/>
+    <col min="10244" max="10244" width="12.28515625" style="18" customWidth="1"/>
+    <col min="10245" max="10245" width="10.5703125" style="18" customWidth="1"/>
+    <col min="10246" max="10246" width="11.5703125" style="18" customWidth="1"/>
+    <col min="10247" max="10247" width="10.85546875" style="18" customWidth="1"/>
+    <col min="10248" max="10248" width="11.140625" style="18" customWidth="1"/>
+    <col min="10249" max="10249" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="10250" max="10261" width="11.42578125" style="18" customWidth="1"/>
+    <col min="10262" max="10265" width="11.7109375" style="18" customWidth="1"/>
+    <col min="10266" max="10266" width="12.140625" style="18" customWidth="1"/>
+    <col min="10267" max="10267" width="11.85546875" style="18" customWidth="1"/>
+    <col min="10268" max="10496" width="9.140625" style="18"/>
+    <col min="10497" max="10497" width="22" style="18" customWidth="1"/>
+    <col min="10498" max="10498" width="12.42578125" style="18" customWidth="1"/>
+    <col min="10499" max="10499" width="12.140625" style="18" customWidth="1"/>
+    <col min="10500" max="10500" width="12.28515625" style="18" customWidth="1"/>
+    <col min="10501" max="10501" width="10.5703125" style="18" customWidth="1"/>
+    <col min="10502" max="10502" width="11.5703125" style="18" customWidth="1"/>
+    <col min="10503" max="10503" width="10.85546875" style="18" customWidth="1"/>
+    <col min="10504" max="10504" width="11.140625" style="18" customWidth="1"/>
+    <col min="10505" max="10505" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="10506" max="10517" width="11.42578125" style="18" customWidth="1"/>
+    <col min="10518" max="10521" width="11.7109375" style="18" customWidth="1"/>
+    <col min="10522" max="10522" width="12.140625" style="18" customWidth="1"/>
+    <col min="10523" max="10523" width="11.85546875" style="18" customWidth="1"/>
+    <col min="10524" max="10752" width="9.140625" style="18"/>
+    <col min="10753" max="10753" width="22" style="18" customWidth="1"/>
+    <col min="10754" max="10754" width="12.42578125" style="18" customWidth="1"/>
+    <col min="10755" max="10755" width="12.140625" style="18" customWidth="1"/>
+    <col min="10756" max="10756" width="12.28515625" style="18" customWidth="1"/>
+    <col min="10757" max="10757" width="10.5703125" style="18" customWidth="1"/>
+    <col min="10758" max="10758" width="11.5703125" style="18" customWidth="1"/>
+    <col min="10759" max="10759" width="10.85546875" style="18" customWidth="1"/>
+    <col min="10760" max="10760" width="11.140625" style="18" customWidth="1"/>
+    <col min="10761" max="10761" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="10762" max="10773" width="11.42578125" style="18" customWidth="1"/>
+    <col min="10774" max="10777" width="11.7109375" style="18" customWidth="1"/>
+    <col min="10778" max="10778" width="12.140625" style="18" customWidth="1"/>
+    <col min="10779" max="10779" width="11.85546875" style="18" customWidth="1"/>
+    <col min="10780" max="11008" width="9.140625" style="18"/>
+    <col min="11009" max="11009" width="22" style="18" customWidth="1"/>
+    <col min="11010" max="11010" width="12.42578125" style="18" customWidth="1"/>
+    <col min="11011" max="11011" width="12.140625" style="18" customWidth="1"/>
+    <col min="11012" max="11012" width="12.28515625" style="18" customWidth="1"/>
+    <col min="11013" max="11013" width="10.5703125" style="18" customWidth="1"/>
+    <col min="11014" max="11014" width="11.5703125" style="18" customWidth="1"/>
+    <col min="11015" max="11015" width="10.85546875" style="18" customWidth="1"/>
+    <col min="11016" max="11016" width="11.140625" style="18" customWidth="1"/>
+    <col min="11017" max="11017" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="11018" max="11029" width="11.42578125" style="18" customWidth="1"/>
+    <col min="11030" max="11033" width="11.7109375" style="18" customWidth="1"/>
+    <col min="11034" max="11034" width="12.140625" style="18" customWidth="1"/>
+    <col min="11035" max="11035" width="11.85546875" style="18" customWidth="1"/>
+    <col min="11036" max="11264" width="9.140625" style="18"/>
+    <col min="11265" max="11265" width="22" style="18" customWidth="1"/>
+    <col min="11266" max="11266" width="12.42578125" style="18" customWidth="1"/>
+    <col min="11267" max="11267" width="12.140625" style="18" customWidth="1"/>
+    <col min="11268" max="11268" width="12.28515625" style="18" customWidth="1"/>
+    <col min="11269" max="11269" width="10.5703125" style="18" customWidth="1"/>
+    <col min="11270" max="11270" width="11.5703125" style="18" customWidth="1"/>
+    <col min="11271" max="11271" width="10.85546875" style="18" customWidth="1"/>
+    <col min="11272" max="11272" width="11.140625" style="18" customWidth="1"/>
+    <col min="11273" max="11273" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="11274" max="11285" width="11.42578125" style="18" customWidth="1"/>
+    <col min="11286" max="11289" width="11.7109375" style="18" customWidth="1"/>
+    <col min="11290" max="11290" width="12.140625" style="18" customWidth="1"/>
+    <col min="11291" max="11291" width="11.85546875" style="18" customWidth="1"/>
+    <col min="11292" max="11520" width="9.140625" style="18"/>
+    <col min="11521" max="11521" width="22" style="18" customWidth="1"/>
+    <col min="11522" max="11522" width="12.42578125" style="18" customWidth="1"/>
+    <col min="11523" max="11523" width="12.140625" style="18" customWidth="1"/>
+    <col min="11524" max="11524" width="12.28515625" style="18" customWidth="1"/>
+    <col min="11525" max="11525" width="10.5703125" style="18" customWidth="1"/>
+    <col min="11526" max="11526" width="11.5703125" style="18" customWidth="1"/>
+    <col min="11527" max="11527" width="10.85546875" style="18" customWidth="1"/>
+    <col min="11528" max="11528" width="11.140625" style="18" customWidth="1"/>
+    <col min="11529" max="11529" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="11530" max="11541" width="11.42578125" style="18" customWidth="1"/>
+    <col min="11542" max="11545" width="11.7109375" style="18" customWidth="1"/>
+    <col min="11546" max="11546" width="12.140625" style="18" customWidth="1"/>
+    <col min="11547" max="11547" width="11.85546875" style="18" customWidth="1"/>
+    <col min="11548" max="11776" width="9.140625" style="18"/>
+    <col min="11777" max="11777" width="22" style="18" customWidth="1"/>
+    <col min="11778" max="11778" width="12.42578125" style="18" customWidth="1"/>
+    <col min="11779" max="11779" width="12.140625" style="18" customWidth="1"/>
+    <col min="11780" max="11780" width="12.28515625" style="18" customWidth="1"/>
+    <col min="11781" max="11781" width="10.5703125" style="18" customWidth="1"/>
+    <col min="11782" max="11782" width="11.5703125" style="18" customWidth="1"/>
+    <col min="11783" max="11783" width="10.85546875" style="18" customWidth="1"/>
+    <col min="11784" max="11784" width="11.140625" style="18" customWidth="1"/>
+    <col min="11785" max="11785" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="11786" max="11797" width="11.42578125" style="18" customWidth="1"/>
+    <col min="11798" max="11801" width="11.7109375" style="18" customWidth="1"/>
+    <col min="11802" max="11802" width="12.140625" style="18" customWidth="1"/>
+    <col min="11803" max="11803" width="11.85546875" style="18" customWidth="1"/>
+    <col min="11804" max="12032" width="9.140625" style="18"/>
+    <col min="12033" max="12033" width="22" style="18" customWidth="1"/>
+    <col min="12034" max="12034" width="12.42578125" style="18" customWidth="1"/>
+    <col min="12035" max="12035" width="12.140625" style="18" customWidth="1"/>
+    <col min="12036" max="12036" width="12.28515625" style="18" customWidth="1"/>
+    <col min="12037" max="12037" width="10.5703125" style="18" customWidth="1"/>
+    <col min="12038" max="12038" width="11.5703125" style="18" customWidth="1"/>
+    <col min="12039" max="12039" width="10.85546875" style="18" customWidth="1"/>
+    <col min="12040" max="12040" width="11.140625" style="18" customWidth="1"/>
+    <col min="12041" max="12041" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="12042" max="12053" width="11.42578125" style="18" customWidth="1"/>
+    <col min="12054" max="12057" width="11.7109375" style="18" customWidth="1"/>
+    <col min="12058" max="12058" width="12.140625" style="18" customWidth="1"/>
+    <col min="12059" max="12059" width="11.85546875" style="18" customWidth="1"/>
+    <col min="12060" max="12288" width="9.140625" style="18"/>
+    <col min="12289" max="12289" width="22" style="18" customWidth="1"/>
+    <col min="12290" max="12290" width="12.42578125" style="18" customWidth="1"/>
+    <col min="12291" max="12291" width="12.140625" style="18" customWidth="1"/>
+    <col min="12292" max="12292" width="12.28515625" style="18" customWidth="1"/>
+    <col min="12293" max="12293" width="10.5703125" style="18" customWidth="1"/>
+    <col min="12294" max="12294" width="11.5703125" style="18" customWidth="1"/>
+    <col min="12295" max="12295" width="10.85546875" style="18" customWidth="1"/>
+    <col min="12296" max="12296" width="11.140625" style="18" customWidth="1"/>
+    <col min="12297" max="12297" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="12298" max="12309" width="11.42578125" style="18" customWidth="1"/>
+    <col min="12310" max="12313" width="11.7109375" style="18" customWidth="1"/>
+    <col min="12314" max="12314" width="12.140625" style="18" customWidth="1"/>
+    <col min="12315" max="12315" width="11.85546875" style="18" customWidth="1"/>
+    <col min="12316" max="12544" width="9.140625" style="18"/>
+    <col min="12545" max="12545" width="22" style="18" customWidth="1"/>
+    <col min="12546" max="12546" width="12.42578125" style="18" customWidth="1"/>
+    <col min="12547" max="12547" width="12.140625" style="18" customWidth="1"/>
+    <col min="12548" max="12548" width="12.28515625" style="18" customWidth="1"/>
+    <col min="12549" max="12549" width="10.5703125" style="18" customWidth="1"/>
+    <col min="12550" max="12550" width="11.5703125" style="18" customWidth="1"/>
+    <col min="12551" max="12551" width="10.85546875" style="18" customWidth="1"/>
+    <col min="12552" max="12552" width="11.140625" style="18" customWidth="1"/>
+    <col min="12553" max="12553" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="12554" max="12565" width="11.42578125" style="18" customWidth="1"/>
+    <col min="12566" max="12569" width="11.7109375" style="18" customWidth="1"/>
+    <col min="12570" max="12570" width="12.140625" style="18" customWidth="1"/>
+    <col min="12571" max="12571" width="11.85546875" style="18" customWidth="1"/>
+    <col min="12572" max="12800" width="9.140625" style="18"/>
+    <col min="12801" max="12801" width="22" style="18" customWidth="1"/>
+    <col min="12802" max="12802" width="12.42578125" style="18" customWidth="1"/>
+    <col min="12803" max="12803" width="12.140625" style="18" customWidth="1"/>
+    <col min="12804" max="12804" width="12.28515625" style="18" customWidth="1"/>
+    <col min="12805" max="12805" width="10.5703125" style="18" customWidth="1"/>
+    <col min="12806" max="12806" width="11.5703125" style="18" customWidth="1"/>
+    <col min="12807" max="12807" width="10.85546875" style="18" customWidth="1"/>
+    <col min="12808" max="12808" width="11.140625" style="18" customWidth="1"/>
+    <col min="12809" max="12809" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="12810" max="12821" width="11.42578125" style="18" customWidth="1"/>
+    <col min="12822" max="12825" width="11.7109375" style="18" customWidth="1"/>
+    <col min="12826" max="12826" width="12.140625" style="18" customWidth="1"/>
+    <col min="12827" max="12827" width="11.85546875" style="18" customWidth="1"/>
+    <col min="12828" max="13056" width="9.140625" style="18"/>
+    <col min="13057" max="13057" width="22" style="18" customWidth="1"/>
+    <col min="13058" max="13058" width="12.42578125" style="18" customWidth="1"/>
+    <col min="13059" max="13059" width="12.140625" style="18" customWidth="1"/>
+    <col min="13060" max="13060" width="12.28515625" style="18" customWidth="1"/>
+    <col min="13061" max="13061" width="10.5703125" style="18" customWidth="1"/>
+    <col min="13062" max="13062" width="11.5703125" style="18" customWidth="1"/>
+    <col min="13063" max="13063" width="10.85546875" style="18" customWidth="1"/>
+    <col min="13064" max="13064" width="11.140625" style="18" customWidth="1"/>
+    <col min="13065" max="13065" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="13066" max="13077" width="11.42578125" style="18" customWidth="1"/>
+    <col min="13078" max="13081" width="11.7109375" style="18" customWidth="1"/>
+    <col min="13082" max="13082" width="12.140625" style="18" customWidth="1"/>
+    <col min="13083" max="13083" width="11.85546875" style="18" customWidth="1"/>
+    <col min="13084" max="13312" width="9.140625" style="18"/>
+    <col min="13313" max="13313" width="22" style="18" customWidth="1"/>
+    <col min="13314" max="13314" width="12.42578125" style="18" customWidth="1"/>
+    <col min="13315" max="13315" width="12.140625" style="18" customWidth="1"/>
+    <col min="13316" max="13316" width="12.28515625" style="18" customWidth="1"/>
+    <col min="13317" max="13317" width="10.5703125" style="18" customWidth="1"/>
+    <col min="13318" max="13318" width="11.5703125" style="18" customWidth="1"/>
+    <col min="13319" max="13319" width="10.85546875" style="18" customWidth="1"/>
+    <col min="13320" max="13320" width="11.140625" style="18" customWidth="1"/>
+    <col min="13321" max="13321" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="13322" max="13333" width="11.42578125" style="18" customWidth="1"/>
+    <col min="13334" max="13337" width="11.7109375" style="18" customWidth="1"/>
+    <col min="13338" max="13338" width="12.140625" style="18" customWidth="1"/>
+    <col min="13339" max="13339" width="11.85546875" style="18" customWidth="1"/>
+    <col min="13340" max="13568" width="9.140625" style="18"/>
+    <col min="13569" max="13569" width="22" style="18" customWidth="1"/>
+    <col min="13570" max="13570" width="12.42578125" style="18" customWidth="1"/>
+    <col min="13571" max="13571" width="12.140625" style="18" customWidth="1"/>
+    <col min="13572" max="13572" width="12.28515625" style="18" customWidth="1"/>
+    <col min="13573" max="13573" width="10.5703125" style="18" customWidth="1"/>
+    <col min="13574" max="13574" width="11.5703125" style="18" customWidth="1"/>
+    <col min="13575" max="13575" width="10.85546875" style="18" customWidth="1"/>
+    <col min="13576" max="13576" width="11.140625" style="18" customWidth="1"/>
+    <col min="13577" max="13577" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="13578" max="13589" width="11.42578125" style="18" customWidth="1"/>
+    <col min="13590" max="13593" width="11.7109375" style="18" customWidth="1"/>
+    <col min="13594" max="13594" width="12.140625" style="18" customWidth="1"/>
+    <col min="13595" max="13595" width="11.85546875" style="18" customWidth="1"/>
+    <col min="13596" max="13824" width="9.140625" style="18"/>
+    <col min="13825" max="13825" width="22" style="18" customWidth="1"/>
+    <col min="13826" max="13826" width="12.42578125" style="18" customWidth="1"/>
+    <col min="13827" max="13827" width="12.140625" style="18" customWidth="1"/>
+    <col min="13828" max="13828" width="12.28515625" style="18" customWidth="1"/>
+    <col min="13829" max="13829" width="10.5703125" style="18" customWidth="1"/>
+    <col min="13830" max="13830" width="11.5703125" style="18" customWidth="1"/>
+    <col min="13831" max="13831" width="10.85546875" style="18" customWidth="1"/>
+    <col min="13832" max="13832" width="11.140625" style="18" customWidth="1"/>
+    <col min="13833" max="13833" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="13834" max="13845" width="11.42578125" style="18" customWidth="1"/>
+    <col min="13846" max="13849" width="11.7109375" style="18" customWidth="1"/>
+    <col min="13850" max="13850" width="12.140625" style="18" customWidth="1"/>
+    <col min="13851" max="13851" width="11.85546875" style="18" customWidth="1"/>
+    <col min="13852" max="14080" width="9.140625" style="18"/>
+    <col min="14081" max="14081" width="22" style="18" customWidth="1"/>
+    <col min="14082" max="14082" width="12.42578125" style="18" customWidth="1"/>
+    <col min="14083" max="14083" width="12.140625" style="18" customWidth="1"/>
+    <col min="14084" max="14084" width="12.28515625" style="18" customWidth="1"/>
+    <col min="14085" max="14085" width="10.5703125" style="18" customWidth="1"/>
+    <col min="14086" max="14086" width="11.5703125" style="18" customWidth="1"/>
+    <col min="14087" max="14087" width="10.85546875" style="18" customWidth="1"/>
+    <col min="14088" max="14088" width="11.140625" style="18" customWidth="1"/>
+    <col min="14089" max="14089" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="14090" max="14101" width="11.42578125" style="18" customWidth="1"/>
+    <col min="14102" max="14105" width="11.7109375" style="18" customWidth="1"/>
+    <col min="14106" max="14106" width="12.140625" style="18" customWidth="1"/>
+    <col min="14107" max="14107" width="11.85546875" style="18" customWidth="1"/>
+    <col min="14108" max="14336" width="9.140625" style="18"/>
+    <col min="14337" max="14337" width="22" style="18" customWidth="1"/>
+    <col min="14338" max="14338" width="12.42578125" style="18" customWidth="1"/>
+    <col min="14339" max="14339" width="12.140625" style="18" customWidth="1"/>
+    <col min="14340" max="14340" width="12.28515625" style="18" customWidth="1"/>
+    <col min="14341" max="14341" width="10.5703125" style="18" customWidth="1"/>
+    <col min="14342" max="14342" width="11.5703125" style="18" customWidth="1"/>
+    <col min="14343" max="14343" width="10.85546875" style="18" customWidth="1"/>
+    <col min="14344" max="14344" width="11.140625" style="18" customWidth="1"/>
+    <col min="14345" max="14345" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="14346" max="14357" width="11.42578125" style="18" customWidth="1"/>
+    <col min="14358" max="14361" width="11.7109375" style="18" customWidth="1"/>
+    <col min="14362" max="14362" width="12.140625" style="18" customWidth="1"/>
+    <col min="14363" max="14363" width="11.85546875" style="18" customWidth="1"/>
+    <col min="14364" max="14592" width="9.140625" style="18"/>
+    <col min="14593" max="14593" width="22" style="18" customWidth="1"/>
+    <col min="14594" max="14594" width="12.42578125" style="18" customWidth="1"/>
+    <col min="14595" max="14595" width="12.140625" style="18" customWidth="1"/>
+    <col min="14596" max="14596" width="12.28515625" style="18" customWidth="1"/>
+    <col min="14597" max="14597" width="10.5703125" style="18" customWidth="1"/>
+    <col min="14598" max="14598" width="11.5703125" style="18" customWidth="1"/>
+    <col min="14599" max="14599" width="10.85546875" style="18" customWidth="1"/>
+    <col min="14600" max="14600" width="11.140625" style="18" customWidth="1"/>
+    <col min="14601" max="14601" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="14602" max="14613" width="11.42578125" style="18" customWidth="1"/>
+    <col min="14614" max="14617" width="11.7109375" style="18" customWidth="1"/>
+    <col min="14618" max="14618" width="12.140625" style="18" customWidth="1"/>
+    <col min="14619" max="14619" width="11.85546875" style="18" customWidth="1"/>
+    <col min="14620" max="14848" width="9.140625" style="18"/>
+    <col min="14849" max="14849" width="22" style="18" customWidth="1"/>
+    <col min="14850" max="14850" width="12.42578125" style="18" customWidth="1"/>
+    <col min="14851" max="14851" width="12.140625" style="18" customWidth="1"/>
+    <col min="14852" max="14852" width="12.28515625" style="18" customWidth="1"/>
+    <col min="14853" max="14853" width="10.5703125" style="18" customWidth="1"/>
+    <col min="14854" max="14854" width="11.5703125" style="18" customWidth="1"/>
+    <col min="14855" max="14855" width="10.85546875" style="18" customWidth="1"/>
+    <col min="14856" max="14856" width="11.140625" style="18" customWidth="1"/>
+    <col min="14857" max="14857" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="14858" max="14869" width="11.42578125" style="18" customWidth="1"/>
+    <col min="14870" max="14873" width="11.7109375" style="18" customWidth="1"/>
+    <col min="14874" max="14874" width="12.140625" style="18" customWidth="1"/>
+    <col min="14875" max="14875" width="11.85546875" style="18" customWidth="1"/>
+    <col min="14876" max="15104" width="9.140625" style="18"/>
+    <col min="15105" max="15105" width="22" style="18" customWidth="1"/>
+    <col min="15106" max="15106" width="12.42578125" style="18" customWidth="1"/>
+    <col min="15107" max="15107" width="12.140625" style="18" customWidth="1"/>
+    <col min="15108" max="15108" width="12.28515625" style="18" customWidth="1"/>
+    <col min="15109" max="15109" width="10.5703125" style="18" customWidth="1"/>
+    <col min="15110" max="15110" width="11.5703125" style="18" customWidth="1"/>
+    <col min="15111" max="15111" width="10.85546875" style="18" customWidth="1"/>
+    <col min="15112" max="15112" width="11.140625" style="18" customWidth="1"/>
+    <col min="15113" max="15113" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="15114" max="15125" width="11.42578125" style="18" customWidth="1"/>
+    <col min="15126" max="15129" width="11.7109375" style="18" customWidth="1"/>
+    <col min="15130" max="15130" width="12.140625" style="18" customWidth="1"/>
+    <col min="15131" max="15131" width="11.85546875" style="18" customWidth="1"/>
+    <col min="15132" max="15360" width="9.140625" style="18"/>
+    <col min="15361" max="15361" width="22" style="18" customWidth="1"/>
+    <col min="15362" max="15362" width="12.42578125" style="18" customWidth="1"/>
+    <col min="15363" max="15363" width="12.140625" style="18" customWidth="1"/>
+    <col min="15364" max="15364" width="12.28515625" style="18" customWidth="1"/>
+    <col min="15365" max="15365" width="10.5703125" style="18" customWidth="1"/>
+    <col min="15366" max="15366" width="11.5703125" style="18" customWidth="1"/>
+    <col min="15367" max="15367" width="10.85546875" style="18" customWidth="1"/>
+    <col min="15368" max="15368" width="11.140625" style="18" customWidth="1"/>
+    <col min="15369" max="15369" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="15370" max="15381" width="11.42578125" style="18" customWidth="1"/>
+    <col min="15382" max="15385" width="11.7109375" style="18" customWidth="1"/>
+    <col min="15386" max="15386" width="12.140625" style="18" customWidth="1"/>
+    <col min="15387" max="15387" width="11.85546875" style="18" customWidth="1"/>
+    <col min="15388" max="15616" width="9.140625" style="18"/>
+    <col min="15617" max="15617" width="22" style="18" customWidth="1"/>
+    <col min="15618" max="15618" width="12.42578125" style="18" customWidth="1"/>
+    <col min="15619" max="15619" width="12.140625" style="18" customWidth="1"/>
+    <col min="15620" max="15620" width="12.28515625" style="18" customWidth="1"/>
+    <col min="15621" max="15621" width="10.5703125" style="18" customWidth="1"/>
+    <col min="15622" max="15622" width="11.5703125" style="18" customWidth="1"/>
+    <col min="15623" max="15623" width="10.85546875" style="18" customWidth="1"/>
+    <col min="15624" max="15624" width="11.140625" style="18" customWidth="1"/>
+    <col min="15625" max="15625" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="15626" max="15637" width="11.42578125" style="18" customWidth="1"/>
+    <col min="15638" max="15641" width="11.7109375" style="18" customWidth="1"/>
+    <col min="15642" max="15642" width="12.140625" style="18" customWidth="1"/>
+    <col min="15643" max="15643" width="11.85546875" style="18" customWidth="1"/>
+    <col min="15644" max="15872" width="9.140625" style="18"/>
+    <col min="15873" max="15873" width="22" style="18" customWidth="1"/>
+    <col min="15874" max="15874" width="12.42578125" style="18" customWidth="1"/>
+    <col min="15875" max="15875" width="12.140625" style="18" customWidth="1"/>
+    <col min="15876" max="15876" width="12.28515625" style="18" customWidth="1"/>
+    <col min="15877" max="15877" width="10.5703125" style="18" customWidth="1"/>
+    <col min="15878" max="15878" width="11.5703125" style="18" customWidth="1"/>
+    <col min="15879" max="15879" width="10.85546875" style="18" customWidth="1"/>
+    <col min="15880" max="15880" width="11.140625" style="18" customWidth="1"/>
+    <col min="15881" max="15881" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="15882" max="15893" width="11.42578125" style="18" customWidth="1"/>
+    <col min="15894" max="15897" width="11.7109375" style="18" customWidth="1"/>
+    <col min="15898" max="15898" width="12.140625" style="18" customWidth="1"/>
+    <col min="15899" max="15899" width="11.85546875" style="18" customWidth="1"/>
+    <col min="15900" max="16128" width="9.140625" style="18"/>
+    <col min="16129" max="16129" width="22" style="18" customWidth="1"/>
+    <col min="16130" max="16130" width="12.42578125" style="18" customWidth="1"/>
+    <col min="16131" max="16131" width="12.140625" style="18" customWidth="1"/>
+    <col min="16132" max="16132" width="12.28515625" style="18" customWidth="1"/>
+    <col min="16133" max="16133" width="10.5703125" style="18" customWidth="1"/>
+    <col min="16134" max="16134" width="11.5703125" style="18" customWidth="1"/>
+    <col min="16135" max="16135" width="10.85546875" style="18" customWidth="1"/>
+    <col min="16136" max="16136" width="11.140625" style="18" customWidth="1"/>
+    <col min="16137" max="16137" width="10.7109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="16138" max="16149" width="11.42578125" style="18" customWidth="1"/>
+    <col min="16150" max="16153" width="11.7109375" style="18" customWidth="1"/>
+    <col min="16154" max="16154" width="12.140625" style="18" customWidth="1"/>
+    <col min="16155" max="16155" width="11.85546875" style="18" customWidth="1"/>
+    <col min="16156" max="16384" width="9.140625" style="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="15" x14ac:dyDescent="0.25">
-      <c r="A1" s="39" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A1" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
-      <c r="S1" s="18"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
+      <c r="S1" s="17"/>
     </row>
     <row r="2" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9"/>
@@ -1898,41 +1963,41 @@
       <c r="F2" s="9"/>
       <c r="G2" s="9"/>
       <c r="H2" s="9"/>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
     </row>
     <row r="3" spans="1:19" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="32"/>
-      <c r="B3" s="33" t="s">
+      <c r="A3" s="27"/>
+      <c r="B3" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="33" t="s">
+      <c r="D3" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="33">
+      <c r="E3" s="28">
         <v>1993</v>
       </c>
-      <c r="F3" s="33">
+      <c r="F3" s="28">
         <v>1994</v>
       </c>
-      <c r="G3" s="33">
+      <c r="G3" s="28">
         <v>1995</v>
       </c>
-      <c r="H3" s="33">
+      <c r="H3" s="28">
         <v>1996</v>
       </c>
-      <c r="I3" s="33">
+      <c r="I3" s="28">
         <v>1997</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="26" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="11">
@@ -1969,7 +2034,7 @@
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="22" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="12">
@@ -1998,7 +2063,7 @@
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="12">
@@ -2027,7 +2092,7 @@
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="22" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="12">
@@ -2056,7 +2121,7 @@
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A8" s="23" t="s">
+      <c r="A8" s="22" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="12">
@@ -2085,7 +2150,7 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="22" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="12">
@@ -2114,7 +2179,7 @@
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="22" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="12">
@@ -2143,7 +2208,7 @@
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="22" t="s">
         <v>11</v>
       </c>
       <c r="B11" s="12">
@@ -2172,7 +2237,7 @@
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="22" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="12">
@@ -2201,7 +2266,7 @@
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="22" t="s">
         <v>13</v>
       </c>
       <c r="B13" s="12">
@@ -2230,7 +2295,7 @@
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="22" t="s">
         <v>14</v>
       </c>
       <c r="B14" s="12">
@@ -2259,7 +2324,7 @@
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="22" t="s">
         <v>15</v>
       </c>
       <c r="B15" s="12">
@@ -2288,7 +2353,7 @@
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="22" t="s">
         <v>16</v>
       </c>
       <c r="B16" s="12">
@@ -2317,7 +2382,7 @@
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B17" s="12">
@@ -2346,7 +2411,7 @@
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A18" s="23" t="s">
+      <c r="A18" s="22" t="s">
         <v>18</v>
       </c>
       <c r="B18" s="12">
@@ -2375,8 +2440,8 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A19" s="23" t="s">
-        <v>81</v>
+      <c r="A19" s="22" t="s">
+        <v>76</v>
       </c>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
@@ -2390,7 +2455,7 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="23" t="s">
+      <c r="A20" s="22" t="s">
         <v>20</v>
       </c>
       <c r="B20" s="12">
@@ -2419,45 +2484,43 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A21" s="21"/>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A22" s="40" t="s">
-        <v>80</v>
-      </c>
-      <c r="B22" s="41"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="41"/>
-      <c r="E22" s="41"/>
-      <c r="F22" s="41"/>
-      <c r="G22" s="41"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="30"/>
+      <c r="A22" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="37"/>
+      <c r="I22" s="37"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A23" s="42" t="s">
-        <v>79</v>
-      </c>
-      <c r="B23" s="42"/>
-      <c r="C23" s="42"/>
-      <c r="D23" s="42"/>
-      <c r="E23" s="42"/>
-      <c r="F23" s="42"/>
-      <c r="G23" s="42"/>
+    <row r="23" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A23:G23"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3366,8 +3429,8 @@
     <col min="16154" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15" x14ac:dyDescent="0.25">
-      <c r="A1" s="39" t="s">
+    <row r="1" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A1" s="36" t="s">
         <v>21</v>
       </c>
       <c r="B1" s="3"/>
@@ -3394,640 +3457,640 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="12" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="35"/>
-      <c r="B3" s="37">
+      <c r="A3" s="30"/>
+      <c r="B3" s="32">
         <v>1998</v>
       </c>
-      <c r="C3" s="37">
+      <c r="C3" s="32">
         <v>1999</v>
       </c>
-      <c r="D3" s="37">
+      <c r="D3" s="32">
         <v>2000</v>
       </c>
-      <c r="E3" s="37">
+      <c r="E3" s="32">
         <v>2001</v>
       </c>
-      <c r="F3" s="37">
+      <c r="F3" s="32">
         <v>2002</v>
       </c>
-      <c r="G3" s="37">
+      <c r="G3" s="32">
         <v>2003</v>
       </c>
-      <c r="H3" s="37">
+      <c r="H3" s="32">
         <v>2004</v>
       </c>
-      <c r="I3" s="37">
+      <c r="I3" s="32">
         <v>2005</v>
       </c>
-      <c r="J3" s="37">
+      <c r="J3" s="32">
         <v>2006</v>
       </c>
-      <c r="K3" s="37">
+      <c r="K3" s="32">
         <v>2007</v>
       </c>
     </row>
     <row r="4" spans="1:17" s="5" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="36">
+      <c r="B4" s="31">
         <f t="shared" ref="B4:K4" si="0">SUM(B5:B20)</f>
         <v>1733263.5</v>
       </c>
-      <c r="C4" s="36">
+      <c r="C4" s="31">
         <f t="shared" si="0"/>
         <v>2016456.3</v>
       </c>
-      <c r="D4" s="36">
+      <c r="D4" s="31">
         <f t="shared" si="0"/>
         <v>2599901.6</v>
       </c>
-      <c r="E4" s="36">
+      <c r="E4" s="31">
         <f t="shared" si="0"/>
         <v>3250593.3</v>
       </c>
-      <c r="F4" s="36">
+      <c r="F4" s="31">
         <f t="shared" si="0"/>
         <v>3776277.3</v>
       </c>
-      <c r="G4" s="36">
+      <c r="G4" s="31">
         <f t="shared" si="0"/>
         <v>4611975.3</v>
       </c>
-      <c r="H4" s="36">
+      <c r="H4" s="31">
         <f t="shared" si="0"/>
         <v>5870134.2999999998</v>
       </c>
-      <c r="I4" s="36">
+      <c r="I4" s="31">
         <f t="shared" si="0"/>
         <v>7590593.5</v>
       </c>
-      <c r="J4" s="36">
+      <c r="J4" s="31">
         <f t="shared" si="0"/>
         <v>10213731.199999999</v>
       </c>
-      <c r="K4" s="36">
+      <c r="K4" s="31">
         <f t="shared" si="0"/>
         <v>12849794</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="24">
+      <c r="B5" s="23">
         <v>48922.2</v>
       </c>
-      <c r="C5" s="24">
+      <c r="C5" s="23">
         <v>78275.899999999994</v>
       </c>
-      <c r="D5" s="24">
+      <c r="D5" s="23">
         <v>82957.2</v>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="23">
         <v>107692.7</v>
       </c>
-      <c r="F5" s="24">
+      <c r="F5" s="23">
         <v>116616.4</v>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="23">
         <v>141570</v>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="23">
         <v>166162.5</v>
       </c>
-      <c r="I5" s="24">
+      <c r="I5" s="23">
         <v>196761.3</v>
       </c>
-      <c r="J5" s="24">
+      <c r="J5" s="23">
         <v>254186.2</v>
       </c>
-      <c r="K5" s="24">
+      <c r="K5" s="23">
         <v>406298.4</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="24">
+      <c r="B6" s="23">
         <v>89311.4</v>
       </c>
-      <c r="C6" s="24">
+      <c r="C6" s="23">
         <v>92937.8</v>
       </c>
-      <c r="D6" s="24">
+      <c r="D6" s="23">
         <v>118092.7</v>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="23">
         <v>147045.1</v>
       </c>
-      <c r="F6" s="24">
+      <c r="F6" s="23">
         <v>179594.7</v>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="23">
         <v>236692.9</v>
       </c>
-      <c r="H6" s="24">
+      <c r="H6" s="23">
         <v>295817.5</v>
       </c>
-      <c r="I6" s="24">
+      <c r="I6" s="23">
         <v>412959.4</v>
       </c>
-      <c r="J6" s="24">
+      <c r="J6" s="23">
         <v>517031.8</v>
       </c>
-      <c r="K6" s="24">
+      <c r="K6" s="23">
         <v>678938.6</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="24">
+      <c r="B7" s="23">
         <v>92478.3</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="23">
         <v>99257.4</v>
       </c>
-      <c r="D7" s="24">
+      <c r="D7" s="23">
         <v>124564.2</v>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="23">
         <v>158693.29999999999</v>
       </c>
-      <c r="F7" s="24">
+      <c r="F7" s="23">
         <v>185603.9</v>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="23">
         <v>230573.8</v>
       </c>
-      <c r="H7" s="24">
+      <c r="H7" s="23">
         <v>258440</v>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="23">
         <v>322696.90000000002</v>
       </c>
-      <c r="J7" s="24">
+      <c r="J7" s="23">
         <v>408617.2</v>
       </c>
-      <c r="K7" s="24">
+      <c r="K7" s="23">
         <v>550708.30000000005</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="24">
+      <c r="B8" s="23">
         <v>105444.9</v>
       </c>
-      <c r="C8" s="24">
+      <c r="C8" s="23">
         <v>138607.79999999999</v>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="23">
         <v>245478.2</v>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="23">
         <v>293405</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="23">
         <v>389545.6</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="23">
         <v>484127.9</v>
       </c>
-      <c r="H8" s="24">
+      <c r="H8" s="23">
         <v>639579.80000000005</v>
       </c>
-      <c r="I8" s="24">
+      <c r="I8" s="23">
         <v>808222</v>
       </c>
-      <c r="J8" s="24">
+      <c r="J8" s="23">
         <v>1094151.2</v>
       </c>
-      <c r="K8" s="24">
+      <c r="K8" s="23">
         <v>1234007.6000000001</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="24">
+      <c r="B9" s="23">
         <v>57774</v>
       </c>
-      <c r="C9" s="24">
+      <c r="C9" s="23">
         <v>76284.800000000003</v>
       </c>
-      <c r="D9" s="24">
+      <c r="D9" s="23">
         <v>118374.5</v>
       </c>
-      <c r="E9" s="24">
+      <c r="E9" s="23">
         <v>149938.29999999999</v>
       </c>
-      <c r="F9" s="24">
+      <c r="F9" s="23">
         <v>178368.4</v>
       </c>
-      <c r="G9" s="24">
+      <c r="G9" s="23">
         <v>200889.4</v>
       </c>
-      <c r="H9" s="24">
+      <c r="H9" s="23">
         <v>356921.5</v>
       </c>
-      <c r="I9" s="24">
+      <c r="I9" s="23">
         <v>401105.5</v>
       </c>
-      <c r="J9" s="24">
+      <c r="J9" s="23">
         <v>512319.9</v>
       </c>
-      <c r="K9" s="24">
+      <c r="K9" s="23">
         <v>617693.4</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="24">
+      <c r="B10" s="23">
         <v>48879.3</v>
       </c>
-      <c r="C10" s="24">
+      <c r="C10" s="23">
         <v>49676.9</v>
       </c>
-      <c r="D10" s="24">
+      <c r="D10" s="23">
         <v>57783.199999999997</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="23">
         <v>69859</v>
       </c>
-      <c r="F10" s="24">
+      <c r="F10" s="23">
         <v>82972.5</v>
       </c>
-      <c r="G10" s="24">
+      <c r="G10" s="23">
         <v>119500.4</v>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="23">
         <v>137238</v>
       </c>
-      <c r="I10" s="24">
+      <c r="I10" s="23">
         <v>168554.8</v>
       </c>
-      <c r="J10" s="24">
+      <c r="J10" s="23">
         <v>192205.3</v>
       </c>
-      <c r="K10" s="24">
+      <c r="K10" s="23">
         <v>266467.7</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="24">
+      <c r="B11" s="23">
         <v>200649.8</v>
       </c>
-      <c r="C11" s="24">
+      <c r="C11" s="23">
         <v>235372</v>
       </c>
-      <c r="D11" s="24">
+      <c r="D11" s="23">
         <v>299947.3</v>
       </c>
-      <c r="E11" s="24">
+      <c r="E11" s="23">
         <v>337702.5</v>
       </c>
-      <c r="F11" s="24">
+      <c r="F11" s="23">
         <v>370493.6</v>
       </c>
-      <c r="G11" s="24">
+      <c r="G11" s="23">
         <v>444418.8</v>
       </c>
-      <c r="H11" s="24">
+      <c r="H11" s="23">
         <v>508970.6</v>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="23">
         <v>679805.9</v>
       </c>
-      <c r="J11" s="24">
+      <c r="J11" s="23">
         <v>922634.5</v>
       </c>
-      <c r="K11" s="24">
+      <c r="K11" s="23">
         <v>1144309.3999999999</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="24">
+      <c r="B12" s="23">
         <v>121920.8</v>
       </c>
-      <c r="C12" s="24">
+      <c r="C12" s="23">
         <v>136400.79999999999</v>
       </c>
-      <c r="D12" s="24">
+      <c r="D12" s="23">
         <v>158853.29999999999</v>
       </c>
-      <c r="E12" s="24">
+      <c r="E12" s="23">
         <v>171666.3</v>
       </c>
-      <c r="F12" s="24">
+      <c r="F12" s="23">
         <v>185172</v>
       </c>
-      <c r="G12" s="24">
+      <c r="G12" s="23">
         <v>235111.5</v>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="23">
         <v>272279.09999999998</v>
       </c>
-      <c r="I12" s="24">
+      <c r="I12" s="23">
         <v>322711.3</v>
       </c>
-      <c r="J12" s="24">
+      <c r="J12" s="23">
         <v>387343.8</v>
       </c>
-      <c r="K12" s="24">
+      <c r="K12" s="23">
         <v>560378.30000000005</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="24">
+      <c r="B13" s="23">
         <v>38188</v>
       </c>
-      <c r="C13" s="24">
+      <c r="C13" s="23">
         <v>38470.5</v>
       </c>
-      <c r="D13" s="24">
+      <c r="D13" s="23">
         <v>57683</v>
       </c>
-      <c r="E13" s="24">
+      <c r="E13" s="23">
         <v>73363.100000000006</v>
       </c>
-      <c r="F13" s="24">
+      <c r="F13" s="23">
         <v>102531.8</v>
       </c>
-      <c r="G13" s="24">
+      <c r="G13" s="23">
         <v>135995.70000000001</v>
       </c>
-      <c r="H13" s="24">
+      <c r="H13" s="23">
         <v>179833.8</v>
       </c>
-      <c r="I13" s="24">
+      <c r="I13" s="23">
         <v>242378.5</v>
       </c>
-      <c r="J13" s="24">
+      <c r="J13" s="23">
         <v>363797.3</v>
       </c>
-      <c r="K13" s="24">
+      <c r="K13" s="23">
         <v>499619.9</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A14" s="25" t="s">
+      <c r="A14" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="24">
+      <c r="B14" s="23">
         <v>63966.9</v>
       </c>
-      <c r="C14" s="24">
+      <c r="C14" s="23">
         <v>82789.5</v>
       </c>
-      <c r="D14" s="24">
+      <c r="D14" s="23">
         <v>129386.8</v>
       </c>
-      <c r="E14" s="24">
+      <c r="E14" s="23">
         <v>147290.1</v>
       </c>
-      <c r="F14" s="24">
+      <c r="F14" s="23">
         <v>199802.9</v>
       </c>
-      <c r="G14" s="24">
+      <c r="G14" s="23">
         <v>217956.6</v>
       </c>
-      <c r="H14" s="24">
+      <c r="H14" s="23">
         <v>295804.79999999999</v>
       </c>
-      <c r="I14" s="24">
+      <c r="I14" s="23">
         <v>432225.2</v>
       </c>
-      <c r="J14" s="24">
+      <c r="J14" s="23">
         <v>593994</v>
       </c>
-      <c r="K14" s="24">
+      <c r="K14" s="23">
         <v>756591.8</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="24">
+      <c r="B15" s="23">
         <v>102086</v>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="23">
         <v>123415.1</v>
       </c>
-      <c r="D15" s="24">
+      <c r="D15" s="23">
         <v>179108.4</v>
       </c>
-      <c r="E15" s="24">
+      <c r="E15" s="23">
         <v>235573.6</v>
       </c>
-      <c r="F15" s="24">
+      <c r="F15" s="23">
         <v>245503.8</v>
       </c>
-      <c r="G15" s="24">
+      <c r="G15" s="23">
         <v>310743.2</v>
       </c>
-      <c r="H15" s="24">
+      <c r="H15" s="23">
         <v>309902.5</v>
       </c>
-      <c r="I15" s="24">
+      <c r="I15" s="23">
         <v>358008.7</v>
       </c>
-      <c r="J15" s="24">
+      <c r="J15" s="23">
         <v>423488.4</v>
       </c>
-      <c r="K15" s="24">
+      <c r="K15" s="23">
         <v>611763.80000000005</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="24">
+      <c r="B16" s="23">
         <v>133676.9</v>
       </c>
-      <c r="C16" s="24">
+      <c r="C16" s="23">
         <v>124814.3</v>
       </c>
-      <c r="D16" s="24">
+      <c r="D16" s="23">
         <v>167554</v>
       </c>
-      <c r="E16" s="24">
+      <c r="E16" s="23">
         <v>203707.2</v>
       </c>
-      <c r="F16" s="24">
+      <c r="F16" s="23">
         <v>216186.1</v>
       </c>
-      <c r="G16" s="24">
+      <c r="G16" s="23">
         <v>268696</v>
       </c>
-      <c r="H16" s="24">
+      <c r="H16" s="23">
         <v>334270.40000000002</v>
       </c>
-      <c r="I16" s="24">
+      <c r="I16" s="23">
         <v>384018.6</v>
       </c>
-      <c r="J16" s="24">
+      <c r="J16" s="23">
         <v>462208.2</v>
       </c>
-      <c r="K16" s="24">
+      <c r="K16" s="23">
         <v>591977.80000000005</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="24">
+      <c r="B17" s="23">
         <v>67998.7</v>
       </c>
-      <c r="C17" s="24">
+      <c r="C17" s="23">
         <v>74090.7</v>
       </c>
-      <c r="D17" s="24">
+      <c r="D17" s="23">
         <v>71109.100000000006</v>
       </c>
-      <c r="E17" s="24">
+      <c r="E17" s="23">
         <v>98773.8</v>
       </c>
-      <c r="F17" s="24">
+      <c r="F17" s="23">
         <v>111409.2</v>
       </c>
-      <c r="G17" s="24">
+      <c r="G17" s="23">
         <v>140487.1</v>
       </c>
-      <c r="H17" s="24">
+      <c r="H17" s="23">
         <v>151916</v>
       </c>
-      <c r="I17" s="24">
+      <c r="I17" s="23">
         <v>184672.3</v>
       </c>
-      <c r="J17" s="24">
+      <c r="J17" s="23">
         <v>236876.6</v>
       </c>
-      <c r="K17" s="24">
+      <c r="K17" s="23">
         <v>320390.7</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A18" s="23" t="s">
+      <c r="A18" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="24">
+      <c r="B18" s="23">
         <v>190543.1</v>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="23">
         <v>211964.7</v>
       </c>
-      <c r="D18" s="24">
+      <c r="D18" s="23">
         <v>238923.7</v>
       </c>
-      <c r="E18" s="24">
+      <c r="E18" s="23">
         <v>280590.2</v>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="23">
         <v>293339.90000000002</v>
       </c>
-      <c r="G18" s="24">
+      <c r="G18" s="23">
         <v>334290.09999999998</v>
       </c>
-      <c r="H18" s="24">
+      <c r="H18" s="23">
         <v>392014.8</v>
       </c>
-      <c r="I18" s="24">
+      <c r="I18" s="23">
         <v>467510</v>
       </c>
-      <c r="J18" s="24">
+      <c r="J18" s="23">
         <v>615123.19999999995</v>
       </c>
-      <c r="K18" s="24">
+      <c r="K18" s="23">
         <v>800527.5</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="24">
+      <c r="B19" s="23">
         <v>60533.1</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="23">
         <v>92836.1</v>
       </c>
-      <c r="D19" s="24">
+      <c r="D19" s="23">
         <v>134931.9</v>
       </c>
-      <c r="E19" s="24">
+      <c r="E19" s="23">
         <v>204425.9</v>
       </c>
-      <c r="F19" s="24">
+      <c r="F19" s="23">
         <v>230720.5</v>
       </c>
-      <c r="G19" s="24">
+      <c r="G19" s="23">
         <v>302164.2</v>
       </c>
-      <c r="H19" s="24">
+      <c r="H19" s="23">
         <v>468769.9</v>
       </c>
-      <c r="I19" s="24">
+      <c r="I19" s="23">
         <v>711612</v>
       </c>
-      <c r="J19" s="24">
+      <c r="J19" s="23">
         <v>957070.7</v>
       </c>
-      <c r="K19" s="24">
+      <c r="K19" s="23">
         <v>1134213.5</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A20" s="23" t="s">
+      <c r="A20" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="24">
+      <c r="B20" s="23">
         <v>310890.09999999998</v>
       </c>
-      <c r="C20" s="24">
+      <c r="C20" s="23">
         <v>361262</v>
       </c>
-      <c r="D20" s="24">
+      <c r="D20" s="23">
         <v>415154.1</v>
       </c>
-      <c r="E20" s="24">
+      <c r="E20" s="23">
         <v>570867.19999999995</v>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="23">
         <v>688416</v>
       </c>
-      <c r="G20" s="24">
+      <c r="G20" s="23">
         <v>808757.7</v>
       </c>
-      <c r="H20" s="24">
+      <c r="H20" s="23">
         <v>1102213.1000000001</v>
       </c>
-      <c r="I20" s="24">
+      <c r="I20" s="23">
         <v>1497351.1</v>
       </c>
-      <c r="J20" s="24">
+      <c r="J20" s="23">
         <v>2272682.9</v>
       </c>
-      <c r="K20" s="24">
+      <c r="K20" s="23">
         <v>2675907.2999999998</v>
       </c>
     </row>
@@ -4043,31 +4106,31 @@
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="43"/>
-      <c r="B22" s="44"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="44"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
+      <c r="A22" s="39"/>
+      <c r="B22" s="40"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A23" s="45"/>
-      <c r="B23" s="45"/>
-      <c r="C23" s="45"/>
-      <c r="D23" s="45"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="45"/>
-      <c r="J23" s="45"/>
-      <c r="K23" s="45"/>
-      <c r="L23" s="45"/>
-      <c r="M23" s="45"/>
-      <c r="N23" s="45"/>
+      <c r="A23" s="41"/>
+      <c r="B23" s="41"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="41"/>
+      <c r="H23" s="41"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="41"/>
+      <c r="K23" s="41"/>
+      <c r="L23" s="41"/>
+      <c r="M23" s="41"/>
+      <c r="N23" s="41"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
@@ -4093,15 +4156,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BN28"/>
+  <dimension ref="A1:BP30"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.85546875" style="9" customWidth="1"/>
     <col min="2" max="16384" width="11" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:66" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:68" ht="15" x14ac:dyDescent="0.2">
+      <c r="A1" s="17" t="s">
         <v>22</v>
       </c>
       <c r="B1" s="7"/>
@@ -4127,474 +4190,494 @@
       <c r="BE1" s="8"/>
       <c r="BI1" s="8"/>
     </row>
-    <row r="2" spans="1:66" ht="12" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.2">
       <c r="AM2" s="10"/>
       <c r="AT2" s="10"/>
       <c r="BI2" s="10"/>
-      <c r="BM2" s="10" t="s">
+      <c r="BN2" s="10"/>
+      <c r="BP2" s="10" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:66" s="29" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="26"/>
-      <c r="B3" s="26" t="s">
+    <row r="3" spans="1:68" s="25" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="43"/>
+      <c r="B3" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="26">
+      <c r="E3" s="43">
         <v>2008</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="G3" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="26" t="s">
+      <c r="H3" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="26">
+      <c r="I3" s="43">
         <v>2009</v>
       </c>
-      <c r="J3" s="26" t="s">
+      <c r="J3" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="K3" s="26" t="s">
+      <c r="K3" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="L3" s="26" t="s">
+      <c r="L3" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="M3" s="26">
+      <c r="M3" s="43">
         <v>2010</v>
       </c>
-      <c r="N3" s="26" t="s">
+      <c r="N3" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="O3" s="26" t="s">
+      <c r="O3" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="P3" s="26" t="s">
+      <c r="P3" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="Q3" s="26">
+      <c r="Q3" s="43">
         <v>2011</v>
       </c>
-      <c r="R3" s="26" t="s">
+      <c r="R3" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="S3" s="26" t="s">
+      <c r="S3" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="T3" s="26" t="s">
+      <c r="T3" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="U3" s="26">
+      <c r="U3" s="43">
         <v>2012</v>
       </c>
-      <c r="V3" s="26" t="s">
+      <c r="V3" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="W3" s="27" t="s">
+      <c r="W3" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="X3" s="26" t="s">
+      <c r="X3" s="43" t="s">
         <v>40</v>
       </c>
-      <c r="Y3" s="26">
+      <c r="Y3" s="43">
         <v>2013</v>
       </c>
-      <c r="Z3" s="26" t="s">
+      <c r="Z3" s="43" t="s">
         <v>41</v>
       </c>
-      <c r="AA3" s="26" t="s">
+      <c r="AA3" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="AB3" s="26" t="s">
+      <c r="AB3" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="AC3" s="26">
+      <c r="AC3" s="43">
         <v>2014</v>
       </c>
-      <c r="AD3" s="26" t="s">
+      <c r="AD3" s="43" t="s">
         <v>44</v>
       </c>
-      <c r="AE3" s="26" t="s">
+      <c r="AE3" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="AF3" s="26" t="s">
+      <c r="AF3" s="43" t="s">
         <v>46</v>
       </c>
-      <c r="AG3" s="26">
+      <c r="AG3" s="43">
         <v>2015</v>
       </c>
-      <c r="AH3" s="26" t="s">
+      <c r="AH3" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="AI3" s="26" t="s">
+      <c r="AI3" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="AJ3" s="28" t="s">
+      <c r="AJ3" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="AK3" s="28">
+      <c r="AK3" s="43">
         <v>2016</v>
       </c>
-      <c r="AL3" s="28" t="s">
+      <c r="AL3" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="AM3" s="26" t="s">
+      <c r="AM3" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="AN3" s="26" t="s">
+      <c r="AN3" s="43" t="s">
         <v>52</v>
       </c>
-      <c r="AO3" s="26">
+      <c r="AO3" s="43">
         <v>2017</v>
       </c>
-      <c r="AP3" s="26" t="s">
+      <c r="AP3" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="AQ3" s="26" t="s">
+      <c r="AQ3" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="AR3" s="26" t="s">
+      <c r="AR3" s="43" t="s">
         <v>55</v>
       </c>
-      <c r="AS3" s="26">
+      <c r="AS3" s="43">
         <v>2018</v>
       </c>
-      <c r="AT3" s="26" t="s">
+      <c r="AT3" s="43" t="s">
         <v>56</v>
       </c>
-      <c r="AU3" s="26" t="s">
+      <c r="AU3" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="AV3" s="26" t="s">
+      <c r="AV3" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="AW3" s="26">
+      <c r="AW3" s="43">
         <v>2019</v>
       </c>
-      <c r="AX3" s="26" t="s">
+      <c r="AX3" s="43" t="s">
         <v>59</v>
       </c>
-      <c r="AY3" s="26" t="s">
+      <c r="AY3" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="AZ3" s="26" t="s">
+      <c r="AZ3" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="BA3" s="26">
+      <c r="BA3" s="43">
         <v>2020</v>
       </c>
-      <c r="BB3" s="26" t="s">
+      <c r="BB3" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="BC3" s="26" t="s">
+      <c r="BC3" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="BD3" s="26" t="s">
+      <c r="BD3" s="43" t="s">
         <v>64</v>
       </c>
-      <c r="BE3" s="26">
+      <c r="BE3" s="43">
         <v>2021</v>
       </c>
-      <c r="BF3" s="26" t="s">
+      <c r="BF3" s="43" t="s">
         <v>65</v>
       </c>
-      <c r="BG3" s="26" t="s">
+      <c r="BG3" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="BH3" s="26" t="s">
+      <c r="BH3" s="43" t="s">
         <v>66</v>
       </c>
-      <c r="BI3" s="26">
+      <c r="BI3" s="43">
         <v>2022</v>
       </c>
-      <c r="BJ3" s="26" t="s">
+      <c r="BJ3" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="BK3" s="26" t="s">
+      <c r="BK3" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="BL3" s="28" t="s">
+      <c r="BL3" s="43" t="s">
         <v>69</v>
       </c>
-      <c r="BM3" s="26" t="s">
-        <v>71</v>
+      <c r="BM3" s="43" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN3" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="BO3" s="43" t="s">
+        <v>78</v>
+      </c>
+      <c r="BP3" s="43" t="s">
+        <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:66" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="31" t="s">
+    <row r="4" spans="1:68" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="12">
         <f>SUM(B5:B25)</f>
         <v>3207244.4</v>
       </c>
-      <c r="C4" s="11">
-        <f t="shared" ref="C4:BM4" si="0">SUM(C5:C25)</f>
+      <c r="C4" s="12">
+        <f t="shared" ref="C4:BN4" si="0">SUM(C5:C25)</f>
         <v>7195598.5999999996</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="12">
         <f t="shared" si="0"/>
         <v>11803580.9</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="12">
         <f t="shared" si="0"/>
         <v>16052919.199999999</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="12">
         <f t="shared" si="0"/>
         <v>3055263.8</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="12">
         <f t="shared" si="0"/>
         <v>6709780.9000000004</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="12">
         <f t="shared" si="0"/>
         <v>11220899.5</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="12">
         <f t="shared" si="0"/>
         <v>17007647</v>
       </c>
-      <c r="J4" s="11">
+      <c r="J4" s="12">
         <f t="shared" si="0"/>
         <v>4020878.4</v>
       </c>
-      <c r="K4" s="11">
+      <c r="K4" s="12">
         <f t="shared" si="0"/>
         <v>8712143.9000000004</v>
       </c>
-      <c r="L4" s="11">
+      <c r="L4" s="12">
         <f t="shared" si="0"/>
         <v>14135228.1</v>
       </c>
-      <c r="M4" s="11">
+      <c r="M4" s="12">
         <f t="shared" si="0"/>
         <v>21815517</v>
       </c>
-      <c r="N4" s="11">
+      <c r="N4" s="12">
         <f t="shared" si="0"/>
         <v>5240223.5</v>
       </c>
-      <c r="O4" s="11">
+      <c r="O4" s="12">
         <f>SUM(O5:O25)</f>
         <v>11240030.9</v>
       </c>
-      <c r="P4" s="11">
+      <c r="P4" s="12">
         <f t="shared" si="0"/>
         <v>18664939.5</v>
       </c>
-      <c r="Q4" s="11">
+      <c r="Q4" s="12">
         <f>Q6+Q7+Q8+Q9+Q10+Q11+Q13+Q14+Q15+Q16+Q17+Q18+Q19+Q22+Q23+Q24</f>
         <v>28243052.699999999</v>
       </c>
-      <c r="R4" s="11">
+      <c r="R4" s="12">
         <f t="shared" si="0"/>
         <v>6097729.9000000004</v>
       </c>
-      <c r="S4" s="11">
+      <c r="S4" s="12">
         <f t="shared" si="0"/>
         <v>12849001.6</v>
       </c>
-      <c r="T4" s="11">
+      <c r="T4" s="12">
         <f t="shared" si="0"/>
         <v>20848732.600000001</v>
       </c>
-      <c r="U4" s="11">
+      <c r="U4" s="12">
         <f>U6+U7+U8+U9+U10+U11+U13+U14+U15+U16+U17+U18+U19+U22+U23+U24</f>
         <v>31015186.600000001</v>
       </c>
-      <c r="V4" s="11">
+      <c r="V4" s="12">
         <f t="shared" si="0"/>
         <v>6966935</v>
       </c>
-      <c r="W4" s="11">
+      <c r="W4" s="12">
         <f t="shared" si="0"/>
         <v>14499992.199999999</v>
       </c>
-      <c r="X4" s="11">
+      <c r="X4" s="12">
         <f t="shared" si="0"/>
         <v>23767993.399999999</v>
       </c>
-      <c r="Y4" s="11">
+      <c r="Y4" s="12">
         <f>Y6+Y7+Y8+Y9+Y10+Y11+Y13+Y14+Y15+Y16+Y17+Y18+Y19+Y22+Y23+Y24</f>
         <v>35999025.100000001</v>
       </c>
-      <c r="Z4" s="11">
+      <c r="Z4" s="12">
         <f t="shared" si="0"/>
         <v>7933827.5</v>
       </c>
-      <c r="AA4" s="11">
+      <c r="AA4" s="12">
         <f t="shared" si="0"/>
         <v>16482952.199999999</v>
       </c>
-      <c r="AB4" s="11">
+      <c r="AB4" s="12">
         <f t="shared" si="0"/>
         <v>27040987.300000001</v>
       </c>
-      <c r="AC4" s="11">
+      <c r="AC4" s="12">
         <f>AC6+AC7+AC8+AC9+AC10+AC11+AC13+AC14+AC15+AC16+AC17+AC18+AC19+AC22+AC23+AC24</f>
         <v>39675832.899999999</v>
       </c>
-      <c r="AD4" s="11">
+      <c r="AD4" s="12">
         <f t="shared" si="0"/>
         <v>8267517.7000000002</v>
       </c>
-      <c r="AE4" s="11">
+      <c r="AE4" s="12">
         <f t="shared" si="0"/>
         <v>16804418.100000001</v>
       </c>
-      <c r="AF4" s="11">
+      <c r="AF4" s="12">
         <f t="shared" si="0"/>
         <v>27436536.699999999</v>
       </c>
-      <c r="AG4" s="11">
+      <c r="AG4" s="12">
         <f>AG6+AG7+AG8+AG9+AG10+AG11+AG13+AG14+AG15+AG16+AG17+AG18+AG19+AG22+AG23+AG24</f>
         <v>40884133.600000001</v>
       </c>
-      <c r="AH4" s="11">
+      <c r="AH4" s="12">
         <f t="shared" si="0"/>
         <v>9309090.9000000004</v>
       </c>
-      <c r="AI4" s="11">
+      <c r="AI4" s="12">
         <f t="shared" si="0"/>
         <v>19357056.899999999</v>
       </c>
-      <c r="AJ4" s="11">
+      <c r="AJ4" s="12">
         <f t="shared" si="0"/>
         <v>31355126.100000001</v>
       </c>
-      <c r="AK4" s="11">
+      <c r="AK4" s="12">
         <f>AK6+AK7+AK8+AK9+AK10+AK11+AK13+AK14+AK15+AK16+AK17+AK18+AK19+AK22+AK23+AK24</f>
         <v>46971150</v>
       </c>
-      <c r="AL4" s="11">
+      <c r="AL4" s="12">
         <f t="shared" si="0"/>
         <v>10431358</v>
       </c>
-      <c r="AM4" s="11">
+      <c r="AM4" s="12">
         <f t="shared" si="0"/>
         <v>21546269.699999999</v>
       </c>
-      <c r="AN4" s="11">
+      <c r="AN4" s="12">
         <f>SUM(AN5:AN25)</f>
         <v>35142065.200000003</v>
       </c>
-      <c r="AO4" s="11">
+      <c r="AO4" s="12">
         <f>AO6+AO7+AO8+AO9+AO10+AO11+AO13+AO14+AO15+AO16+AO17+AO18+AO19+AO22+AO23+AO24</f>
         <v>54378857.799999997</v>
       </c>
-      <c r="AP4" s="11">
+      <c r="AP4" s="12">
         <f t="shared" si="0"/>
         <v>11786166.699999999</v>
       </c>
-      <c r="AQ4" s="11">
+      <c r="AQ4" s="12">
         <f t="shared" si="0"/>
         <v>24857119.199999999</v>
       </c>
-      <c r="AR4" s="11">
+      <c r="AR4" s="12">
         <f t="shared" si="0"/>
         <v>39767105.700000003</v>
       </c>
-      <c r="AS4" s="11">
+      <c r="AS4" s="12">
         <f t="shared" si="0"/>
         <v>61819536.399999999</v>
       </c>
-      <c r="AT4" s="11">
+      <c r="AT4" s="12">
         <f t="shared" si="0"/>
         <v>13180857.199999999</v>
       </c>
-      <c r="AU4" s="11">
+      <c r="AU4" s="12">
         <f t="shared" si="0"/>
         <v>27908618.100000001</v>
       </c>
-      <c r="AV4" s="11">
+      <c r="AV4" s="12">
         <f t="shared" si="0"/>
         <v>44297912.100000001</v>
       </c>
-      <c r="AW4" s="11">
+      <c r="AW4" s="12">
         <f t="shared" si="0"/>
         <v>69532626.5</v>
       </c>
-      <c r="AX4" s="11">
+      <c r="AX4" s="12">
         <f t="shared" si="0"/>
         <v>15093342.4</v>
       </c>
-      <c r="AY4" s="11">
+      <c r="AY4" s="12">
         <f t="shared" si="0"/>
         <v>28399592.699999999</v>
       </c>
-      <c r="AZ4" s="11">
+      <c r="AZ4" s="12">
         <f t="shared" si="0"/>
         <v>45803255.200000003</v>
       </c>
-      <c r="BA4" s="11">
+      <c r="BA4" s="12">
         <f t="shared" si="0"/>
         <v>70649033.200000003</v>
       </c>
-      <c r="BB4" s="11">
+      <c r="BB4" s="12">
         <f t="shared" si="0"/>
         <v>15938671.5</v>
       </c>
-      <c r="BC4" s="11">
+      <c r="BC4" s="12">
         <f t="shared" si="0"/>
         <v>32265436.5</v>
       </c>
-      <c r="BD4" s="11">
+      <c r="BD4" s="12">
         <f t="shared" si="0"/>
         <v>53029365.700000003</v>
       </c>
-      <c r="BE4" s="11">
+      <c r="BE4" s="12">
         <f t="shared" si="0"/>
         <v>83951587.900000006</v>
       </c>
-      <c r="BF4" s="11">
+      <c r="BF4" s="12">
         <f t="shared" si="0"/>
         <v>19695592.800000001</v>
       </c>
-      <c r="BG4" s="11">
+      <c r="BG4" s="12">
         <f t="shared" si="0"/>
         <v>40034332.600000001</v>
       </c>
-      <c r="BH4" s="11">
+      <c r="BH4" s="12">
         <f t="shared" si="0"/>
         <v>65487797.899999999</v>
       </c>
-      <c r="BI4" s="11">
+      <c r="BI4" s="12">
         <f t="shared" si="0"/>
         <v>103765518.2</v>
       </c>
-      <c r="BJ4" s="11">
+      <c r="BJ4" s="12">
         <f t="shared" si="0"/>
         <v>23582637</v>
       </c>
-      <c r="BK4" s="11">
+      <c r="BK4" s="12">
         <f t="shared" si="0"/>
         <v>47244671.5</v>
       </c>
-      <c r="BL4" s="11">
+      <c r="BL4" s="12">
         <f t="shared" si="0"/>
         <v>75546820.299999997</v>
       </c>
-      <c r="BM4" s="11">
+      <c r="BM4" s="12">
+        <v>119442289.7</v>
+      </c>
+      <c r="BN4" s="12">
         <f t="shared" si="0"/>
-        <v>120561096.40000001</v>
-      </c>
-      <c r="BN4" s="15"/>
+        <v>26023903.800000001</v>
+      </c>
+      <c r="BO4" s="12">
+        <f t="shared" ref="BO4:BP4" si="1">SUM(BO5:BO25)</f>
+        <v>52342740.299999997</v>
+      </c>
+      <c r="BP4" s="12">
+        <f t="shared" si="1"/>
+        <v>84962626.099999994</v>
+      </c>
     </row>
-    <row r="5" spans="1:66" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="23" t="s">
-        <v>78</v>
+    <row r="5" spans="1:68" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="22" t="s">
+        <v>75</v>
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="12"/>
@@ -4674,12 +4757,20 @@
         <v>1931427.8</v>
       </c>
       <c r="BM5" s="12">
-        <v>3034101.7</v>
-      </c>
-      <c r="BN5" s="15"/>
+        <v>2626326.7000000002</v>
+      </c>
+      <c r="BN5" s="34">
+        <v>713428.8</v>
+      </c>
+      <c r="BO5" s="34">
+        <v>1299791.3999999999</v>
+      </c>
+      <c r="BP5" s="13">
+        <v>2228186.2999999998</v>
+      </c>
     </row>
-    <row r="6" spans="1:66" x14ac:dyDescent="0.2">
-      <c r="A6" s="23" t="s">
+    <row r="6" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="12">
@@ -4872,11 +4963,20 @@
         <v>2302576.7000000002</v>
       </c>
       <c r="BM6" s="12">
-        <v>3685297.6</v>
+        <v>3668371.9</v>
+      </c>
+      <c r="BN6" s="34">
+        <v>763320.1</v>
+      </c>
+      <c r="BO6" s="34">
+        <v>1604314.2</v>
+      </c>
+      <c r="BP6" s="13">
+        <v>2647057.6</v>
       </c>
     </row>
-    <row r="7" spans="1:66" x14ac:dyDescent="0.2">
-      <c r="A7" s="23" t="s">
+    <row r="7" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A7" s="22" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="12">
@@ -5069,11 +5169,20 @@
         <v>3157112.7</v>
       </c>
       <c r="BM7" s="12">
-        <v>4717853.0999999996</v>
+        <v>4187587.9</v>
+      </c>
+      <c r="BN7" s="34">
+        <v>1077687.8</v>
+      </c>
+      <c r="BO7" s="34">
+        <v>2291102.2000000002</v>
+      </c>
+      <c r="BP7" s="13">
+        <v>3599622.7</v>
       </c>
     </row>
-    <row r="8" spans="1:66" x14ac:dyDescent="0.2">
-      <c r="A8" s="23" t="s">
+    <row r="8" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A8" s="22" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="12">
@@ -5266,12 +5375,20 @@
         <v>3093209.7</v>
       </c>
       <c r="BM8" s="12">
-        <v>4974850.0999999996</v>
-      </c>
-      <c r="BN8" s="15"/>
+        <v>5322132</v>
+      </c>
+      <c r="BN8" s="34">
+        <v>1199159.3</v>
+      </c>
+      <c r="BO8" s="34">
+        <v>2406534.7999999998</v>
+      </c>
+      <c r="BP8" s="13">
+        <v>3778763.1</v>
+      </c>
     </row>
-    <row r="9" spans="1:66" x14ac:dyDescent="0.2">
-      <c r="A9" s="23" t="s">
+    <row r="9" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A9" s="22" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="12">
@@ -5464,11 +5581,20 @@
         <v>9682340.9000000004</v>
       </c>
       <c r="BM9" s="12">
-        <v>14950418.300000001</v>
+        <v>15237721.6</v>
+      </c>
+      <c r="BN9" s="34">
+        <v>3153451.1</v>
+      </c>
+      <c r="BO9" s="34">
+        <v>6661463.2999999998</v>
+      </c>
+      <c r="BP9" s="13">
+        <v>9864759.3000000007</v>
       </c>
     </row>
-    <row r="10" spans="1:66" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
+    <row r="10" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A10" s="22" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="12">
@@ -5661,11 +5787,20 @@
         <v>3026011.6</v>
       </c>
       <c r="BM10" s="12">
-        <v>4811055.5999999996</v>
+        <v>5014788.3</v>
+      </c>
+      <c r="BN10" s="34">
+        <v>1239384.1000000001</v>
+      </c>
+      <c r="BO10" s="34">
+        <v>2146896.1</v>
+      </c>
+      <c r="BP10" s="13">
+        <v>3351046.7</v>
       </c>
     </row>
-    <row r="11" spans="1:66" x14ac:dyDescent="0.2">
-      <c r="A11" s="23" t="s">
+    <row r="11" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A11" s="22" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="12">
@@ -5858,12 +5993,21 @@
         <v>1907237.1</v>
       </c>
       <c r="BM11" s="12">
-        <v>3108407.6</v>
+        <v>2926010.6</v>
+      </c>
+      <c r="BN11" s="34">
+        <v>638675.9</v>
+      </c>
+      <c r="BO11" s="34">
+        <v>1403328.4</v>
+      </c>
+      <c r="BP11" s="13">
+        <v>2226048.7000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:66" x14ac:dyDescent="0.2">
-      <c r="A12" s="23" t="s">
-        <v>74</v>
+    <row r="12" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A12" s="22" t="s">
+        <v>71</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
@@ -5943,11 +6087,20 @@
         <v>1207954.8</v>
       </c>
       <c r="BM12" s="12">
-        <v>1923707.9</v>
+        <v>1809417.6</v>
+      </c>
+      <c r="BN12" s="34">
+        <v>392798.7</v>
+      </c>
+      <c r="BO12" s="34">
+        <v>781003.4</v>
+      </c>
+      <c r="BP12" s="13">
+        <v>1402035.3</v>
       </c>
     </row>
-    <row r="13" spans="1:66" x14ac:dyDescent="0.2">
-      <c r="A13" s="23" t="s">
+    <row r="13" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A13" s="22" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="12">
@@ -6140,12 +6293,20 @@
         <v>5119584.3</v>
       </c>
       <c r="BM13" s="12">
-        <v>8449346.4000000004</v>
-      </c>
-      <c r="BN13" s="15"/>
+        <v>7711828.2000000002</v>
+      </c>
+      <c r="BN13" s="34">
+        <v>1690879.8</v>
+      </c>
+      <c r="BO13" s="34">
+        <v>3296690.9</v>
+      </c>
+      <c r="BP13" s="13">
+        <v>5805103</v>
+      </c>
     </row>
-    <row r="14" spans="1:66" x14ac:dyDescent="0.2">
-      <c r="A14" s="23" t="s">
+    <row r="14" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A14" s="22" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="12">
@@ -6338,11 +6499,20 @@
         <v>2711574.2</v>
       </c>
       <c r="BM14" s="12">
-        <v>4613160.5999999996</v>
+        <v>4436636.0999999996</v>
+      </c>
+      <c r="BN14" s="34">
+        <v>974585.8</v>
+      </c>
+      <c r="BO14" s="34">
+        <v>1771516.7</v>
+      </c>
+      <c r="BP14" s="13">
+        <v>3052487</v>
       </c>
     </row>
-    <row r="15" spans="1:66" x14ac:dyDescent="0.2">
-      <c r="A15" s="23" t="s">
+    <row r="15" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A15" s="22" t="s">
         <v>13</v>
       </c>
       <c r="B15" s="12">
@@ -6535,11 +6705,20 @@
         <v>1873331.5</v>
       </c>
       <c r="BM15" s="12">
-        <v>2860036.6</v>
+        <v>2573511.2999999998</v>
+      </c>
+      <c r="BN15" s="34">
+        <v>576162.5</v>
+      </c>
+      <c r="BO15" s="34">
+        <v>1300409.7</v>
+      </c>
+      <c r="BP15" s="13">
+        <v>2101681.5</v>
       </c>
     </row>
-    <row r="16" spans="1:66" x14ac:dyDescent="0.2">
-      <c r="A16" s="23" t="s">
+    <row r="16" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A16" s="22" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="12">
@@ -6732,11 +6911,20 @@
         <v>3523341.2</v>
       </c>
       <c r="BM16" s="12">
-        <v>4866995.3</v>
+        <v>4798701</v>
+      </c>
+      <c r="BN16" s="34">
+        <v>853411.5</v>
+      </c>
+      <c r="BO16" s="34">
+        <v>2217360.6</v>
+      </c>
+      <c r="BP16" s="13">
+        <v>3654775.7</v>
       </c>
     </row>
-    <row r="17" spans="1:65" x14ac:dyDescent="0.2">
-      <c r="A17" s="23" t="s">
+    <row r="17" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A17" s="22" t="s">
         <v>15</v>
       </c>
       <c r="B17" s="12">
@@ -6884,10 +7072,13 @@
       <c r="BJ17" s="13"/>
       <c r="BK17" s="13"/>
       <c r="BL17" s="13"/>
-      <c r="BM17" s="46"/>
+      <c r="BM17" s="42"/>
+      <c r="BN17" s="34"/>
+      <c r="BO17" s="34"/>
+      <c r="BP17" s="13"/>
     </row>
-    <row r="18" spans="1:65" x14ac:dyDescent="0.2">
-      <c r="A18" s="23" t="s">
+    <row r="18" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A18" s="22" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="12">
@@ -7080,11 +7271,20 @@
         <v>2547531.5</v>
       </c>
       <c r="BM18" s="12">
-        <v>4346514</v>
+        <v>4371041.7</v>
+      </c>
+      <c r="BN18" s="34">
+        <v>980252.5</v>
+      </c>
+      <c r="BO18" s="34">
+        <v>1815468</v>
+      </c>
+      <c r="BP18" s="13">
+        <v>3026319.9</v>
       </c>
     </row>
-    <row r="19" spans="1:65" x14ac:dyDescent="0.2">
-      <c r="A19" s="23" t="s">
+    <row r="19" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A19" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="12">
@@ -7277,12 +7477,21 @@
         <v>1536753.9</v>
       </c>
       <c r="BM19" s="12">
-        <v>2229282.2999999998</v>
+        <v>2227596.2999999998</v>
+      </c>
+      <c r="BN19" s="34">
+        <v>484557.1</v>
+      </c>
+      <c r="BO19" s="34">
+        <v>965108.2</v>
+      </c>
+      <c r="BP19" s="13">
+        <v>1809191.2</v>
       </c>
     </row>
-    <row r="20" spans="1:65" x14ac:dyDescent="0.2">
-      <c r="A20" s="23" t="s">
-        <v>75</v>
+    <row r="20" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A20" s="22" t="s">
+        <v>72</v>
       </c>
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
@@ -7406,12 +7615,21 @@
         <v>2699012</v>
       </c>
       <c r="BM20" s="12">
-        <v>4166425.1</v>
+        <v>3831527.6</v>
+      </c>
+      <c r="BN20" s="34">
+        <v>927563.6</v>
+      </c>
+      <c r="BO20" s="34">
+        <v>1757351.2</v>
+      </c>
+      <c r="BP20" s="13">
+        <v>3162813.7</v>
       </c>
     </row>
-    <row r="21" spans="1:65" x14ac:dyDescent="0.2">
-      <c r="A21" s="23" t="s">
-        <v>76</v>
+    <row r="21" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A21" s="22" t="s">
+        <v>73</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
@@ -7491,11 +7709,20 @@
         <v>1226557.7</v>
       </c>
       <c r="BM21" s="12">
-        <v>1949728.3</v>
+        <v>1969727.3</v>
+      </c>
+      <c r="BN21" s="34">
+        <v>430328.3</v>
+      </c>
+      <c r="BO21" s="34">
+        <v>798910.2</v>
+      </c>
+      <c r="BP21" s="13">
+        <v>1361367.8</v>
       </c>
     </row>
-    <row r="22" spans="1:65" x14ac:dyDescent="0.2">
-      <c r="A22" s="23" t="s">
+    <row r="22" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A22" s="22" t="s">
         <v>18</v>
       </c>
       <c r="B22" s="12">
@@ -7688,11 +7915,20 @@
         <v>3123022.1</v>
       </c>
       <c r="BM22" s="12">
-        <v>4470598.5</v>
+        <v>4459056.0999999996</v>
+      </c>
+      <c r="BN22" s="34">
+        <v>1086449.3</v>
+      </c>
+      <c r="BO22" s="34">
+        <v>1906711</v>
+      </c>
+      <c r="BP22" s="13">
+        <v>3336587.8</v>
       </c>
     </row>
-    <row r="23" spans="1:65" x14ac:dyDescent="0.2">
-      <c r="A23" s="23" t="s">
+    <row r="23" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A23" s="22" t="s">
         <v>19</v>
       </c>
       <c r="B23" s="12">
@@ -7885,11 +8121,20 @@
         <v>7840605.4000000004</v>
       </c>
       <c r="BM23" s="12">
-        <v>12874957.1</v>
+        <v>12960836</v>
+      </c>
+      <c r="BN23" s="34">
+        <v>2647542</v>
+      </c>
+      <c r="BO23" s="34">
+        <v>5454843.9000000004</v>
+      </c>
+      <c r="BP23" s="13">
+        <v>9201576.5</v>
       </c>
     </row>
-    <row r="24" spans="1:65" x14ac:dyDescent="0.2">
-      <c r="A24" s="23" t="s">
+    <row r="24" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A24" s="22" t="s">
         <v>20</v>
       </c>
       <c r="B24" s="12">
@@ -8082,12 +8327,21 @@
         <v>14591960.1</v>
       </c>
       <c r="BM24" s="12">
-        <v>24828705.800000001</v>
+        <v>25229706.800000001</v>
+      </c>
+      <c r="BN24" s="34">
+        <v>5321676</v>
+      </c>
+      <c r="BO24" s="34">
+        <v>10651833.5</v>
+      </c>
+      <c r="BP24" s="13">
+        <v>16429880.300000001</v>
       </c>
     </row>
-    <row r="25" spans="1:65" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="23" t="s">
-        <v>77</v>
+    <row r="25" spans="1:68" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="22" t="s">
+        <v>74</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="12"/>
@@ -8140,7 +8394,7 @@
       <c r="AL25" s="12"/>
       <c r="AM25" s="12"/>
       <c r="AN25" s="12"/>
-      <c r="AO25" s="38">
+      <c r="AO25" s="33">
         <v>1712054.1</v>
       </c>
       <c r="AP25" s="12"/>
@@ -8211,63 +8465,82 @@
         <v>2445675.1</v>
       </c>
       <c r="BM25" s="12">
-        <v>3699654.5</v>
+        <v>4079764.7</v>
+      </c>
+      <c r="BN25" s="34">
+        <v>872589.6</v>
+      </c>
+      <c r="BO25" s="34">
+        <v>1812102.6</v>
+      </c>
+      <c r="BP25" s="13">
+        <v>2923322</v>
       </c>
     </row>
-    <row r="26" spans="1:65" x14ac:dyDescent="0.2">
-      <c r="A26" s="16"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
-      <c r="K26" s="17"/>
-      <c r="L26" s="17"/>
-      <c r="M26" s="17"/>
-      <c r="N26" s="17"/>
-      <c r="O26" s="17"/>
-      <c r="P26" s="17"/>
-      <c r="Q26" s="17"/>
-      <c r="R26" s="17"/>
-      <c r="S26" s="17"/>
-      <c r="T26" s="17"/>
-      <c r="U26" s="17"/>
-      <c r="V26" s="17"/>
-      <c r="W26" s="17"/>
-      <c r="X26" s="17"/>
-      <c r="Y26" s="17"/>
-      <c r="Z26" s="17"/>
-      <c r="AA26" s="17"/>
-      <c r="AB26" s="17"/>
-      <c r="AC26" s="17"/>
-      <c r="AD26" s="17"/>
-      <c r="AE26" s="17"/>
-      <c r="AF26" s="17"/>
-      <c r="AG26" s="17"/>
-      <c r="AH26" s="17"/>
-      <c r="AI26" s="17"/>
-      <c r="AJ26" s="17"/>
-      <c r="AK26" s="17"/>
-      <c r="AL26" s="17"/>
-      <c r="AM26" s="17"/>
-      <c r="AN26" s="17"/>
-      <c r="AO26" s="17"/>
-      <c r="AP26" s="17"/>
-      <c r="AQ26" s="17"/>
+    <row r="26" spans="1:68" x14ac:dyDescent="0.2">
+      <c r="A26" s="15"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="16"/>
+      <c r="I26" s="16"/>
+      <c r="J26" s="16"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="16"/>
+      <c r="M26" s="16"/>
+      <c r="N26" s="16"/>
+      <c r="O26" s="16"/>
+      <c r="P26" s="16"/>
+      <c r="Q26" s="16"/>
+      <c r="R26" s="16"/>
+      <c r="S26" s="16"/>
+      <c r="T26" s="16"/>
+      <c r="U26" s="16"/>
+      <c r="V26" s="16"/>
+      <c r="W26" s="16"/>
+      <c r="X26" s="16"/>
+      <c r="Y26" s="16"/>
+      <c r="Z26" s="16"/>
+      <c r="AA26" s="16"/>
+      <c r="AB26" s="16"/>
+      <c r="AC26" s="16"/>
+      <c r="AD26" s="16"/>
+      <c r="AE26" s="16"/>
+      <c r="AF26" s="16"/>
+      <c r="AG26" s="16"/>
+      <c r="AH26" s="16"/>
+      <c r="AI26" s="16"/>
+      <c r="AJ26" s="16"/>
+      <c r="AK26" s="16"/>
+      <c r="AL26" s="16"/>
+      <c r="AM26" s="16"/>
+      <c r="AN26" s="16"/>
+      <c r="AO26" s="16"/>
+      <c r="AP26" s="16"/>
+      <c r="AQ26" s="16"/>
     </row>
-    <row r="27" spans="1:65" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="AO27" s="15"/>
+    <row r="27" spans="1:68" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="AO27" s="14"/>
     </row>
-    <row r="28" spans="1:65" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="14" t="s">
-        <v>73</v>
+    <row r="28" spans="1:68" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="35" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:68" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A29" s="35" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:68" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A30" s="35" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -8288,6 +8561,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Документ" ma:contentTypeID="0x010100370B4E274E87974096EDA171ECDE108C" ma:contentTypeVersion="0" ma:contentTypeDescription="Создание документа." ma:contentTypeScope="" ma:versionID="af0b12f176aaf80ed46566cf733fadb3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="53974d1da0c14f073d2cc649cae9f3e6">
     <xsd:element name="properties">
@@ -8336,12 +8615,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2582ECFD-169F-46C8-969A-B5703A703E29}">
   <ds:schemaRefs>
@@ -8351,6 +8624,20 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5181F81-2A3A-4D72-A9C0-5535159C2F7B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9ABBB370-5262-4C35-838B-BFB1C872F301}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8363,18 +8650,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5181F81-2A3A-4D72-A9C0-5535159C2F7B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>